<commit_message>
Fix Kalos Path Excel Sheet Challenges and Missing Pokemon constraints
Co-authored-by: lsampaio1337-beep <246645260+lsampaio1337-beep@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Kalos_Path.xlsx
+++ b/Kalos_Path.xlsx
@@ -4915,7 +4915,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C18"/>
+  <dimension ref="A1:C42"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -4933,10 +4933,10 @@
         <v>Challenge 1</v>
       </c>
       <c r="B2" t="str">
-        <v>Defeat Gym Leader Viola</v>
+        <v>Defeat Gym Leader in Route 2</v>
       </c>
       <c r="C2" t="str">
-        <v>Route 4</v>
+        <v>Santalune Forest</v>
       </c>
     </row>
     <row r="3">
@@ -4944,10 +4944,10 @@
         <v>Challenge 2</v>
       </c>
       <c r="B3" t="str">
-        <v>Reach Lumiose City and receive Kanto starter</v>
+        <v>Defeat 25 Pokemon in Santalune Forest</v>
       </c>
       <c r="C3" t="str">
-        <v>Route 5</v>
+        <v>Route 3</v>
       </c>
     </row>
     <row r="4">
@@ -4955,10 +4955,10 @@
         <v>Challenge 3</v>
       </c>
       <c r="B4" t="str">
-        <v>Reach Camphrier Town Daycare</v>
+        <v>Catch 5 different species in Route 3</v>
       </c>
       <c r="C4" t="str">
-        <v>Unlock Daycare</v>
+        <v>Route 22</v>
       </c>
     </row>
     <row r="5">
@@ -4966,10 +4966,10 @@
         <v>Challenge 4</v>
       </c>
       <c r="B5" t="str">
-        <v>Defeat Gym Leader Grant</v>
+        <v>Defeat Gym Leader in Route 22</v>
       </c>
       <c r="C5" t="str">
-        <v>Route 10</v>
+        <v>Route 4</v>
       </c>
     </row>
     <row r="6">
@@ -4977,10 +4977,10 @@
         <v>Challenge 5</v>
       </c>
       <c r="B6" t="str">
-        <v>Defeat Gym Leader Korrina</v>
+        <v>Catch 5 different species in Route 4</v>
       </c>
       <c r="C6" t="str">
-        <v>Route 12</v>
+        <v>Lumiose City</v>
       </c>
     </row>
     <row r="7">
@@ -4988,10 +4988,10 @@
         <v>Challenge 6</v>
       </c>
       <c r="B7" t="str">
-        <v>Defeat Gym Leader Ramos</v>
+        <v>Defeat 25 Pokemon in Lumiose City</v>
       </c>
       <c r="C7" t="str">
-        <v>Route 14</v>
+        <v>Route 5</v>
       </c>
     </row>
     <row r="8">
@@ -4999,10 +4999,10 @@
         <v>Challenge 7</v>
       </c>
       <c r="B8" t="str">
-        <v>Defeat Gym Leader Clemont</v>
+        <v>Defeat Gym Leader in Route 5</v>
       </c>
       <c r="C8" t="str">
-        <v>Route 15</v>
+        <v>Route 6</v>
       </c>
     </row>
     <row r="9">
@@ -5010,10 +5010,10 @@
         <v>Challenge 8</v>
       </c>
       <c r="B9" t="str">
-        <v>Defeat Gym Leader Valerie</v>
+        <v>Defeat 25 Pokemon in Route 6</v>
       </c>
       <c r="C9" t="str">
-        <v>Route 16</v>
+        <v>Route 7</v>
       </c>
     </row>
     <row r="10">
@@ -5021,10 +5021,10 @@
         <v>Challenge 9</v>
       </c>
       <c r="B10" t="str">
-        <v>Defeat Gym Leader Olympia</v>
+        <v>Catch 5 different species in Route 7</v>
       </c>
       <c r="C10" t="str">
-        <v>Team Flare HQ</v>
+        <v>Connecting Cave</v>
       </c>
     </row>
     <row r="11">
@@ -5032,10 +5032,10 @@
         <v>Challenge 10</v>
       </c>
       <c r="B11" t="str">
-        <v>Defeat Gym Leader Wulfric</v>
+        <v>Defeat Gym Leader in Connecting Cave</v>
       </c>
       <c r="C11" t="str">
-        <v>Route 21</v>
+        <v>Route 8</v>
       </c>
     </row>
     <row r="12">
@@ -5043,10 +5043,10 @@
         <v>Challenge 11</v>
       </c>
       <c r="B12" t="str">
-        <v>Defeat Elite Four Malva</v>
+        <v>Catch 5 different species in Route 8</v>
       </c>
       <c r="C12" t="str">
-        <v>Access Siebold</v>
+        <v>Route 9</v>
       </c>
     </row>
     <row r="13">
@@ -5054,10 +5054,10 @@
         <v>Challenge 12</v>
       </c>
       <c r="B13" t="str">
-        <v>Defeat Elite Four Siebold</v>
+        <v>Defeat 25 Pokemon in Route 9</v>
       </c>
       <c r="C13" t="str">
-        <v>Access Wikstrom</v>
+        <v>Glittering Cave</v>
       </c>
     </row>
     <row r="14">
@@ -5065,10 +5065,10 @@
         <v>Challenge 13</v>
       </c>
       <c r="B14" t="str">
-        <v>Defeat Elite Four Wikstrom</v>
+        <v>Defeat Gym Leader in Glittering Cave</v>
       </c>
       <c r="C14" t="str">
-        <v>Access Drasna</v>
+        <v>Cyllage City</v>
       </c>
     </row>
     <row r="15">
@@ -5076,10 +5076,10 @@
         <v>Challenge 14</v>
       </c>
       <c r="B15" t="str">
-        <v>Defeat Elite Four Drasna</v>
+        <v>Defeat 25 Pokemon in Cyllage City</v>
       </c>
       <c r="C15" t="str">
-        <v>Access Champion Diantha</v>
+        <v>Route 10</v>
       </c>
     </row>
     <row r="16">
@@ -5087,37 +5087,301 @@
         <v>Challenge 15</v>
       </c>
       <c r="B16" t="str">
-        <v>Defeat Champion Diantha</v>
+        <v>Catch 5 different species in Route 10</v>
       </c>
       <c r="C16" t="str">
-        <v>Unlock Post-Game Fishing Spots</v>
+        <v>Route 11</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Extra Challenge 1</v>
+        <v>Challenge 16</v>
       </c>
       <c r="B17" t="str">
-        <v>Catch Legendary Birds (Articuno/Zapdos/Moltres) at Sea Spirit's Den</v>
+        <v>Defeat Gym Leader in Route 11</v>
       </c>
       <c r="C17" t="str">
-        <v>Victory Road (Fishing)</v>
+        <v>Reflection Cave</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>Extra Challenge 2</v>
+        <v>Challenge 17</v>
       </c>
       <c r="B18" t="str">
-        <v>Reach Level 100 with 6 Kalos Pokemon</v>
+        <v>Catch 5 different species in Reflection Cave</v>
       </c>
       <c r="C18" t="str">
+        <v>Route 12</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>Challenge 18</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Defeat 25 Pokemon in Route 12</v>
+      </c>
+      <c r="C19" t="str">
+        <v>Route 13</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>Challenge 19</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Defeat Gym Leader in Route 13</v>
+      </c>
+      <c r="C20" t="str">
+        <v>Route 14</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>Challenge 20</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Defeat 25 Pokemon in Route 14</v>
+      </c>
+      <c r="C21" t="str">
+        <v>Route 15</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>Challenge 21</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Catch 5 different species in Route 15</v>
+      </c>
+      <c r="C22" t="str">
+        <v>Lost Hotel</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>Challenge 22</v>
+      </c>
+      <c r="B23" t="str">
+        <v>Defeat Gym Leader in Lost Hotel</v>
+      </c>
+      <c r="C23" t="str">
+        <v>Route 16</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>Challenge 23</v>
+      </c>
+      <c r="B24" t="str">
+        <v>Catch 5 different species in Route 16</v>
+      </c>
+      <c r="C24" t="str">
+        <v>Frost Cavern</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>Challenge 24</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Defeat 25 Pokemon in Frost Cavern</v>
+      </c>
+      <c r="C25" t="str">
+        <v>Route 17</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>Challenge 25</v>
+      </c>
+      <c r="B26" t="str">
+        <v>Defeat Gym Leader in Route 17</v>
+      </c>
+      <c r="C26" t="str">
+        <v>Team Flare HQ</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>Challenge 26</v>
+      </c>
+      <c r="B27" t="str">
+        <v>Defeat 25 Pokemon in Team Flare HQ</v>
+      </c>
+      <c r="C27" t="str">
+        <v>Route 18</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>Challenge 27</v>
+      </c>
+      <c r="B28" t="str">
+        <v>Catch 5 different species in Route 18</v>
+      </c>
+      <c r="C28" t="str">
+        <v>Route 19</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>Challenge 28</v>
+      </c>
+      <c r="B29" t="str">
+        <v>Defeat Gym Leader in Route 19</v>
+      </c>
+      <c r="C29" t="str">
+        <v>Route 20</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>Challenge 29</v>
+      </c>
+      <c r="B30" t="str">
+        <v>Catch 5 different species in Route 20</v>
+      </c>
+      <c r="C30" t="str">
+        <v>Pokémon Village</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>Challenge 30</v>
+      </c>
+      <c r="B31" t="str">
+        <v>Defeat 25 Pokemon in Pokémon Village</v>
+      </c>
+      <c r="C31" t="str">
+        <v>Route 21</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>Challenge 31</v>
+      </c>
+      <c r="B32" t="str">
+        <v>Defeat Gym Leader in Route 21</v>
+      </c>
+      <c r="C32" t="str">
+        <v>Victory Road</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>Challenge 32</v>
+      </c>
+      <c r="B33" t="str">
+        <v>Defeat 25 Pokemon in Victory Road</v>
+      </c>
+      <c r="C33" t="str">
+        <v>Parfum Palace (Fishing)</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>Extra Challenge 1 1</v>
+      </c>
+      <c r="B34" t="str">
+        <v>Catch 5 different species in Parfum Palace (Fishing)</v>
+      </c>
+      <c r="C34" t="str">
+        <v>Ambrette Town (Fishing)</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>Extra Challenge 1 2</v>
+      </c>
+      <c r="B35" t="str">
+        <v>Defeat Gym Leader in Ambrette Town (Fishing)</v>
+      </c>
+      <c r="C35" t="str">
+        <v>Cyllage City (Fishing)</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>Extra Challenge 1 3</v>
+      </c>
+      <c r="B36" t="str">
+        <v>Catch 5 different species in Cyllage City (Fishing)</v>
+      </c>
+      <c r="C36" t="str">
+        <v>Azure Bay (Fishing)</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>Extra Challenge 1 4</v>
+      </c>
+      <c r="B37" t="str">
+        <v>Defeat 25 Pokemon in Azure Bay (Fishing)</v>
+      </c>
+      <c r="C37" t="str">
+        <v>Coumarine City (Fishing)</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>Extra Challenge 1 5</v>
+      </c>
+      <c r="B38" t="str">
+        <v>Defeat Gym Leader in Coumarine City (Fishing)</v>
+      </c>
+      <c r="C38" t="str">
+        <v>Route 19 (Fishing)</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>Extra Challenge 1 6</v>
+      </c>
+      <c r="B39" t="str">
+        <v>Defeat 25 Pokemon in Route 19 (Fishing)</v>
+      </c>
+      <c r="C39" t="str">
+        <v>Pokémon Village (Fishing)</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>Extra Challenge 1 7</v>
+      </c>
+      <c r="B40" t="str">
+        <v>Catch 5 different species in Pokémon Village (Fishing)</v>
+      </c>
+      <c r="C40" t="str">
+        <v>Sea Spirit's Den</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>Challenge 33</v>
+      </c>
+      <c r="B41" t="str">
+        <v>Defeat Gym Leader in Sea Spirit's Den</v>
+      </c>
+      <c r="C41" t="str">
+        <v>Victory Road (Fishing)</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>Extra Challenge 1 8</v>
+      </c>
+      <c r="B42" t="str">
+        <v>Catch 5 different species in Victory Road (Fishing)</v>
+      </c>
+      <c r="C42" t="str">
         <v>Sea Spirit's Den (Fishing)</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C18"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C42"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -5151,7 +5415,7 @@
         <v>Route 5</v>
       </c>
       <c r="D2" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="3">
@@ -5165,7 +5429,7 @@
         <v>Route 5</v>
       </c>
       <c r="D3" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="4">
@@ -5179,7 +5443,7 @@
         <v>Route 5</v>
       </c>
       <c r="D4" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="5">
@@ -5193,7 +5457,7 @@
         <v>Route 5</v>
       </c>
       <c r="D5" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="6">
@@ -5207,7 +5471,7 @@
         <v>Route 5</v>
       </c>
       <c r="D6" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="7">
@@ -5221,7 +5485,7 @@
         <v>Route 5</v>
       </c>
       <c r="D7" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="8">
@@ -5235,7 +5499,7 @@
         <v>Route 5</v>
       </c>
       <c r="D8" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="9">
@@ -5249,7 +5513,7 @@
         <v>Route 5</v>
       </c>
       <c r="D9" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="10">
@@ -5263,7 +5527,7 @@
         <v>Route 5</v>
       </c>
       <c r="D10" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="11">
@@ -5291,7 +5555,7 @@
         <v>Route 5</v>
       </c>
       <c r="D12" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="13">
@@ -5361,7 +5625,7 @@
         <v>Route 5</v>
       </c>
       <c r="D17" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="18">
@@ -5375,7 +5639,7 @@
         <v>Route 5</v>
       </c>
       <c r="D18" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="19">
@@ -5417,7 +5681,7 @@
         <v>Route 5</v>
       </c>
       <c r="D21" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="22">
@@ -5431,7 +5695,7 @@
         <v>Route 5</v>
       </c>
       <c r="D22" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="23">
@@ -5445,7 +5709,7 @@
         <v>Route 5</v>
       </c>
       <c r="D23" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="24">
@@ -5459,7 +5723,7 @@
         <v>Route 5</v>
       </c>
       <c r="D24" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="25">
@@ -5501,7 +5765,7 @@
         <v>Route 5</v>
       </c>
       <c r="D27" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="28">
@@ -5515,7 +5779,7 @@
         <v>Route 5</v>
       </c>
       <c r="D28" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="29">
@@ -5529,7 +5793,7 @@
         <v>Route 5</v>
       </c>
       <c r="D29" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="30">
@@ -5627,7 +5891,7 @@
         <v>Route 5</v>
       </c>
       <c r="D36" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="37">
@@ -5641,7 +5905,7 @@
         <v>Route 5</v>
       </c>
       <c r="D37" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="38">
@@ -5851,7 +6115,7 @@
         <v>Route 5</v>
       </c>
       <c r="D52" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="53">
@@ -5865,7 +6129,7 @@
         <v>Route 10</v>
       </c>
       <c r="D53" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="54">
@@ -5907,7 +6171,7 @@
         <v>Route 10</v>
       </c>
       <c r="D56" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="57">
@@ -5921,7 +6185,7 @@
         <v>Route 10</v>
       </c>
       <c r="D57" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="58">
@@ -5935,7 +6199,7 @@
         <v>Route 10</v>
       </c>
       <c r="D58" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="59">
@@ -5949,7 +6213,7 @@
         <v>Route 10</v>
       </c>
       <c r="D59" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="60">
@@ -5963,7 +6227,7 @@
         <v>Route 10</v>
       </c>
       <c r="D60" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="61">
@@ -5977,7 +6241,7 @@
         <v>Route 10</v>
       </c>
       <c r="D61" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="62">
@@ -5991,7 +6255,7 @@
         <v>Route 10</v>
       </c>
       <c r="D62" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="63">
@@ -6005,7 +6269,7 @@
         <v>Route 10</v>
       </c>
       <c r="D63" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="64">
@@ -6019,7 +6283,7 @@
         <v>Route 10</v>
       </c>
       <c r="D64" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="65">
@@ -6033,7 +6297,7 @@
         <v>Route 10</v>
       </c>
       <c r="D65" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="66">
@@ -6047,7 +6311,7 @@
         <v>Route 10</v>
       </c>
       <c r="D66" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="67">
@@ -6061,7 +6325,7 @@
         <v>Route 10</v>
       </c>
       <c r="D67" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="68">
@@ -6075,7 +6339,7 @@
         <v>Route 10</v>
       </c>
       <c r="D68" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="69">
@@ -6089,7 +6353,7 @@
         <v>Route 10</v>
       </c>
       <c r="D69" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="70">
@@ -6103,7 +6367,7 @@
         <v>Route 10</v>
       </c>
       <c r="D70" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="71">
@@ -6201,7 +6465,7 @@
         <v>Route 10</v>
       </c>
       <c r="D77" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="78">
@@ -6215,7 +6479,7 @@
         <v>Route 10</v>
       </c>
       <c r="D78" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="79">
@@ -6229,7 +6493,7 @@
         <v>Route 10</v>
       </c>
       <c r="D79" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="80">
@@ -6243,7 +6507,7 @@
         <v>Route 10</v>
       </c>
       <c r="D80" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="81">
@@ -6355,7 +6619,7 @@
         <v>Route 10</v>
       </c>
       <c r="D88" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="89">
@@ -6369,7 +6633,7 @@
         <v>Route 10</v>
       </c>
       <c r="D89" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="90">
@@ -6383,7 +6647,7 @@
         <v>Route 10</v>
       </c>
       <c r="D90" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="91">
@@ -6453,7 +6717,7 @@
         <v>Route 10</v>
       </c>
       <c r="D95" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="96">
@@ -6467,7 +6731,7 @@
         <v>Route 10</v>
       </c>
       <c r="D96" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="97">
@@ -6509,7 +6773,7 @@
         <v>Route 10</v>
       </c>
       <c r="D99" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="100">
@@ -6523,7 +6787,7 @@
         <v>Route 10</v>
       </c>
       <c r="D100" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="101">
@@ -6537,7 +6801,7 @@
         <v>Route 10</v>
       </c>
       <c r="D101" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="102">
@@ -6551,7 +6815,7 @@
         <v>Route 10</v>
       </c>
       <c r="D102" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="103">
@@ -6593,7 +6857,7 @@
         <v>Route 15</v>
       </c>
       <c r="D105" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="106">
@@ -6607,7 +6871,7 @@
         <v>Route 15</v>
       </c>
       <c r="D106" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="107">
@@ -6621,7 +6885,7 @@
         <v>Route 15</v>
       </c>
       <c r="D107" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="108">
@@ -6691,7 +6955,7 @@
         <v>Route 15</v>
       </c>
       <c r="D112" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="113">
@@ -6705,7 +6969,7 @@
         <v>Route 15</v>
       </c>
       <c r="D113" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="114">
@@ -6719,7 +6983,7 @@
         <v>Route 15</v>
       </c>
       <c r="D114" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="115">
@@ -6747,7 +7011,7 @@
         <v>Route 15</v>
       </c>
       <c r="D116" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="117">
@@ -6761,7 +7025,7 @@
         <v>Route 15</v>
       </c>
       <c r="D117" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="118">
@@ -6775,7 +7039,7 @@
         <v>Route 15</v>
       </c>
       <c r="D118" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="119">
@@ -6789,7 +7053,7 @@
         <v>Route 15</v>
       </c>
       <c r="D119" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="120">
@@ -6803,7 +7067,7 @@
         <v>Route 15</v>
       </c>
       <c r="D120" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="121">
@@ -6817,7 +7081,7 @@
         <v>Route 15</v>
       </c>
       <c r="D121" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="122">
@@ -6831,7 +7095,7 @@
         <v>Route 15</v>
       </c>
       <c r="D122" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="123">
@@ -6845,7 +7109,7 @@
         <v>Route 15</v>
       </c>
       <c r="D123" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="124">
@@ -6859,7 +7123,7 @@
         <v>Route 15</v>
       </c>
       <c r="D124" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="125">
@@ -6873,7 +7137,7 @@
         <v>Route 15</v>
       </c>
       <c r="D125" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="126">
@@ -6887,7 +7151,7 @@
         <v>Route 15</v>
       </c>
       <c r="D126" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="127">
@@ -6901,7 +7165,7 @@
         <v>Route 15</v>
       </c>
       <c r="D127" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="128">
@@ -7083,7 +7347,7 @@
         <v>Route 15</v>
       </c>
       <c r="D140" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="141">
@@ -7097,7 +7361,7 @@
         <v>Route 15</v>
       </c>
       <c r="D141" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="142">
@@ -7125,7 +7389,7 @@
         <v>Route 15</v>
       </c>
       <c r="D143" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="144">
@@ -7139,7 +7403,7 @@
         <v>Route 15</v>
       </c>
       <c r="D144" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="145">
@@ -7153,7 +7417,7 @@
         <v>Route 15</v>
       </c>
       <c r="D145" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="146">
@@ -7167,7 +7431,7 @@
         <v>Route 15</v>
       </c>
       <c r="D146" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="147">
@@ -7181,7 +7445,7 @@
         <v>Route 15</v>
       </c>
       <c r="D147" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="148">
@@ -7195,7 +7459,7 @@
         <v>Route 15</v>
       </c>
       <c r="D148" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="149">
@@ -7209,7 +7473,7 @@
         <v>Route 15</v>
       </c>
       <c r="D149" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="150">
@@ -7223,7 +7487,7 @@
         <v>Route 15</v>
       </c>
       <c r="D150" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="151">
@@ -7237,7 +7501,7 @@
         <v>Route 15</v>
       </c>
       <c r="D151" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="152">
@@ -7251,7 +7515,7 @@
         <v>Route 15</v>
       </c>
       <c r="D152" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="153">
@@ -7265,7 +7529,7 @@
         <v>Route 20</v>
       </c>
       <c r="D153" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="154">
@@ -7279,7 +7543,7 @@
         <v>Route 20</v>
       </c>
       <c r="D154" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="155">
@@ -7293,7 +7557,7 @@
         <v>Route 20</v>
       </c>
       <c r="D155" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="156">
@@ -7307,7 +7571,7 @@
         <v>Route 20</v>
       </c>
       <c r="D156" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="157">
@@ -7321,7 +7585,7 @@
         <v>Route 20</v>
       </c>
       <c r="D157" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="158">
@@ -7335,7 +7599,7 @@
         <v>Route 20</v>
       </c>
       <c r="D158" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="159">
@@ -7349,7 +7613,7 @@
         <v>Route 20</v>
       </c>
       <c r="D159" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="160">
@@ -7363,7 +7627,7 @@
         <v>Route 20</v>
       </c>
       <c r="D160" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="161">
@@ -7377,7 +7641,7 @@
         <v>Route 20</v>
       </c>
       <c r="D161" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="162">
@@ -7391,7 +7655,7 @@
         <v>Route 20</v>
       </c>
       <c r="D162" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="163">
@@ -7405,7 +7669,7 @@
         <v>Route 20</v>
       </c>
       <c r="D163" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="164">
@@ -7419,7 +7683,7 @@
         <v>Route 20</v>
       </c>
       <c r="D164" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="165">
@@ -7433,7 +7697,7 @@
         <v>Route 20</v>
       </c>
       <c r="D165" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="166">
@@ -7447,7 +7711,7 @@
         <v>Route 20</v>
       </c>
       <c r="D166" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="167">
@@ -7461,7 +7725,7 @@
         <v>Route 20</v>
       </c>
       <c r="D167" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="168">
@@ -7475,7 +7739,7 @@
         <v>Route 20</v>
       </c>
       <c r="D168" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="169">
@@ -7489,7 +7753,7 @@
         <v>Route 20</v>
       </c>
       <c r="D169" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="170">
@@ -7503,7 +7767,7 @@
         <v>Route 20</v>
       </c>
       <c r="D170" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="171">
@@ -7517,7 +7781,7 @@
         <v>Route 20</v>
       </c>
       <c r="D171" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="172">
@@ -7531,7 +7795,7 @@
         <v>Route 20</v>
       </c>
       <c r="D172" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="173">
@@ -7545,7 +7809,7 @@
         <v>Route 20</v>
       </c>
       <c r="D173" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="174">
@@ -7559,7 +7823,7 @@
         <v>Route 20</v>
       </c>
       <c r="D174" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="175">
@@ -7573,7 +7837,7 @@
         <v>Route 20</v>
       </c>
       <c r="D175" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="176">
@@ -7587,7 +7851,7 @@
         <v>Route 20</v>
       </c>
       <c r="D176" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="177">
@@ -7601,7 +7865,7 @@
         <v>Route 20</v>
       </c>
       <c r="D177" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="178">
@@ -7615,7 +7879,7 @@
         <v>Route 20</v>
       </c>
       <c r="D178" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="179">
@@ -7629,7 +7893,7 @@
         <v>Route 20</v>
       </c>
       <c r="D179" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="180">
@@ -7643,7 +7907,7 @@
         <v>Route 20</v>
       </c>
       <c r="D180" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="181">
@@ -7657,7 +7921,7 @@
         <v>Route 20</v>
       </c>
       <c r="D181" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="182">
@@ -7671,7 +7935,7 @@
         <v>Route 20</v>
       </c>
       <c r="D182" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="183">
@@ -7685,7 +7949,7 @@
         <v>Route 20</v>
       </c>
       <c r="D183" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="184">
@@ -7699,7 +7963,7 @@
         <v>Route 20</v>
       </c>
       <c r="D184" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="185">
@@ -7713,7 +7977,7 @@
         <v>Route 20</v>
       </c>
       <c r="D185" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="186">
@@ -7727,7 +7991,7 @@
         <v>Route 20</v>
       </c>
       <c r="D186" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="187">
@@ -7741,7 +8005,7 @@
         <v>Route 20</v>
       </c>
       <c r="D187" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="188">
@@ -7755,7 +8019,7 @@
         <v>Route 20</v>
       </c>
       <c r="D188" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="189">
@@ -7769,7 +8033,7 @@
         <v>Route 20</v>
       </c>
       <c r="D189" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="190">
@@ -7783,7 +8047,7 @@
         <v>Route 20</v>
       </c>
       <c r="D190" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="191">
@@ -7797,7 +8061,7 @@
         <v>Route 20</v>
       </c>
       <c r="D191" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="192">
@@ -7811,7 +8075,7 @@
         <v>Route 20</v>
       </c>
       <c r="D192" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="193">
@@ -7825,7 +8089,7 @@
         <v>Route 20</v>
       </c>
       <c r="D193" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="194">
@@ -7839,7 +8103,7 @@
         <v>Route 20</v>
       </c>
       <c r="D194" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="195">
@@ -7853,7 +8117,7 @@
         <v>Route 20</v>
       </c>
       <c r="D195" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="196">
@@ -7867,7 +8131,7 @@
         <v>Route 20</v>
       </c>
       <c r="D196" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="197">
@@ -7881,7 +8145,7 @@
         <v>Route 20</v>
       </c>
       <c r="D197" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="198">
@@ -7895,7 +8159,7 @@
         <v>Route 20</v>
       </c>
       <c r="D198" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="199">
@@ -7909,7 +8173,7 @@
         <v>Route 20</v>
       </c>
       <c r="D199" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="200">
@@ -7923,7 +8187,7 @@
         <v>Route 20</v>
       </c>
       <c r="D200" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="201">
@@ -7937,7 +8201,7 @@
         <v>Route 20</v>
       </c>
       <c r="D201" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="202">
@@ -7951,7 +8215,7 @@
         <v>Route 20</v>
       </c>
       <c r="D202" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="203">
@@ -7965,7 +8229,7 @@
         <v>Route 20</v>
       </c>
       <c r="D203" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="204">
@@ -7979,7 +8243,7 @@
         <v>Route 20</v>
       </c>
       <c r="D204" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="205">
@@ -7993,7 +8257,7 @@
         <v>Route 20</v>
       </c>
       <c r="D205" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="206">
@@ -8007,7 +8271,7 @@
         <v>Route 20</v>
       </c>
       <c r="D206" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="207">
@@ -8021,7 +8285,7 @@
         <v>Route 20</v>
       </c>
       <c r="D207" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="208">
@@ -8035,7 +8299,7 @@
         <v>Route 20</v>
       </c>
       <c r="D208" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="209">
@@ -8049,7 +8313,7 @@
         <v>Route 20</v>
       </c>
       <c r="D209" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="210">
@@ -8063,7 +8327,7 @@
         <v>Route 20</v>
       </c>
       <c r="D210" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="211">
@@ -8077,7 +8341,7 @@
         <v>Route 20</v>
       </c>
       <c r="D211" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="212">
@@ -8091,7 +8355,7 @@
         <v>Route 20</v>
       </c>
       <c r="D212" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="213">
@@ -8105,7 +8369,7 @@
         <v>Route 20</v>
       </c>
       <c r="D213" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="214">
@@ -8119,7 +8383,7 @@
         <v>Route 20</v>
       </c>
       <c r="D214" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="215">
@@ -8133,7 +8397,7 @@
         <v>Route 20</v>
       </c>
       <c r="D215" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="216">
@@ -8147,7 +8411,7 @@
         <v>Route 20</v>
       </c>
       <c r="D216" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="217">
@@ -8161,7 +8425,7 @@
         <v>Route 20</v>
       </c>
       <c r="D217" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="218">
@@ -8175,7 +8439,7 @@
         <v>Route 20</v>
       </c>
       <c r="D218" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="219">
@@ -8189,7 +8453,7 @@
         <v>Route 20</v>
       </c>
       <c r="D219" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="220">
@@ -8203,7 +8467,7 @@
         <v>Route 20</v>
       </c>
       <c r="D220" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="221">
@@ -8217,7 +8481,7 @@
         <v>Route 20</v>
       </c>
       <c r="D221" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="222">
@@ -8231,7 +8495,7 @@
         <v>Route 20</v>
       </c>
       <c r="D222" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="223">
@@ -8245,7 +8509,7 @@
         <v>Route 20</v>
       </c>
       <c r="D223" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="224">
@@ -8259,7 +8523,7 @@
         <v>Route 20</v>
       </c>
       <c r="D224" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="225">
@@ -8273,7 +8537,7 @@
         <v>Route 20</v>
       </c>
       <c r="D225" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="226">
@@ -8287,7 +8551,7 @@
         <v>Route 20</v>
       </c>
       <c r="D226" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="227">
@@ -8301,7 +8565,7 @@
         <v>Route 20</v>
       </c>
       <c r="D227" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="228">
@@ -8315,7 +8579,7 @@
         <v>Route 20</v>
       </c>
       <c r="D228" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="229">
@@ -8329,7 +8593,7 @@
         <v>Route 20</v>
       </c>
       <c r="D229" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="230">
@@ -8343,7 +8607,7 @@
         <v>Route 20</v>
       </c>
       <c r="D230" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="231">
@@ -8357,7 +8621,7 @@
         <v>Route 20</v>
       </c>
       <c r="D231" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="232">
@@ -8371,7 +8635,7 @@
         <v>Route 20</v>
       </c>
       <c r="D232" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="233">
@@ -8385,7 +8649,7 @@
         <v>Route 20</v>
       </c>
       <c r="D233" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="234">
@@ -8399,7 +8663,7 @@
         <v>Route 20</v>
       </c>
       <c r="D234" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="235">
@@ -8413,7 +8677,7 @@
         <v>Route 20</v>
       </c>
       <c r="D235" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="236">
@@ -8427,7 +8691,7 @@
         <v>Route 20</v>
       </c>
       <c r="D236" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="237">
@@ -8441,7 +8705,7 @@
         <v>Route 20</v>
       </c>
       <c r="D237" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="238">
@@ -8455,7 +8719,7 @@
         <v>Route 20</v>
       </c>
       <c r="D238" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="239">
@@ -8469,7 +8733,7 @@
         <v>Route 20</v>
       </c>
       <c r="D239" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="240">
@@ -8483,7 +8747,7 @@
         <v>Route 20</v>
       </c>
       <c r="D240" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="241">
@@ -8497,7 +8761,7 @@
         <v>Route 20</v>
       </c>
       <c r="D241" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="242">
@@ -8511,7 +8775,7 @@
         <v>Route 20</v>
       </c>
       <c r="D242" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="243">
@@ -8525,7 +8789,7 @@
         <v>Route 20</v>
       </c>
       <c r="D243" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="244">
@@ -8539,7 +8803,7 @@
         <v>Route 20</v>
       </c>
       <c r="D244" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="245">
@@ -8553,7 +8817,7 @@
         <v>Route 20</v>
       </c>
       <c r="D245" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="246">
@@ -8567,7 +8831,7 @@
         <v>Route 20</v>
       </c>
       <c r="D246" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="247">

</xml_diff>

<commit_message>
Refine Kalos progression with exact Starter chains and Post-League Legendary Halls
Co-authored-by: lsampaio1337-beep <246645260+lsampaio1337-beep@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Kalos_Path.xlsx
+++ b/Kalos_Path.xlsx
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E428"/>
+  <dimension ref="A1:E460"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -6577,16 +6577,16 @@
         <v>67</v>
       </c>
       <c r="B364" t="str">
-        <v>Starter Depot Spot (Kalos)</v>
+        <v>Sea Spirit Den Entrance</v>
       </c>
       <c r="C364" t="str">
-        <v>Chespin</v>
+        <v>Qwilfish</v>
       </c>
       <c r="D364" t="str">
-        <v>88-93</v>
+        <v>70-75</v>
       </c>
       <c r="E364" t="str">
-        <v>25%</v>
+        <v>30%</v>
       </c>
     </row>
     <row r="365">
@@ -6594,16 +6594,16 @@
         <v>67</v>
       </c>
       <c r="B365" t="str">
-        <v>Starter Depot Spot (Kalos)</v>
+        <v>Sea Spirit Den Entrance</v>
       </c>
       <c r="C365" t="str">
-        <v>Fennekin</v>
+        <v>Reuniclus</v>
       </c>
       <c r="D365" t="str">
-        <v>88-93</v>
+        <v>70-75</v>
       </c>
       <c r="E365" t="str">
-        <v>20%</v>
+        <v>25%</v>
       </c>
     </row>
     <row r="366">
@@ -6611,13 +6611,13 @@
         <v>67</v>
       </c>
       <c r="B366" t="str">
-        <v>Starter Depot Spot (Kalos)</v>
+        <v>Sea Spirit Den Entrance</v>
       </c>
       <c r="C366" t="str">
-        <v>Froakie</v>
+        <v>Mothim</v>
       </c>
       <c r="D366" t="str">
-        <v>88-93</v>
+        <v>70-75</v>
       </c>
       <c r="E366" t="str">
         <v>20%</v>
@@ -6628,13 +6628,13 @@
         <v>67</v>
       </c>
       <c r="B367" t="str">
-        <v>Starter Depot Spot (Kalos)</v>
+        <v>Sea Spirit Den Entrance</v>
       </c>
       <c r="C367" t="str">
-        <v>Frogadier</v>
+        <v>Mawile</v>
       </c>
       <c r="D367" t="str">
-        <v>88-93</v>
+        <v>70-75</v>
       </c>
       <c r="E367" t="str">
         <v>15%</v>
@@ -6645,13 +6645,13 @@
         <v>67</v>
       </c>
       <c r="B368" t="str">
-        <v>Starter Depot Spot (Kalos)</v>
+        <v>Sea Spirit Den Entrance</v>
       </c>
       <c r="C368" t="str">
-        <v>Quilladin</v>
+        <v>Igglybuff</v>
       </c>
       <c r="D368" t="str">
-        <v>88-93</v>
+        <v>70-75</v>
       </c>
       <c r="E368" t="str">
         <v>10%</v>
@@ -6659,36 +6659,36 @@
     </row>
     <row r="369">
       <c r="A369">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B369" t="str">
-        <v>Starter Depot Spot (Kalos)</v>
+        <v>Sea Spirit Den Tunnels</v>
       </c>
       <c r="C369" t="str">
-        <v>Braixen</v>
+        <v>Gogoat</v>
       </c>
       <c r="D369" t="str">
-        <v>88-93</v>
+        <v>82-87</v>
       </c>
       <c r="E369" t="str">
-        <v>5%</v>
+        <v>30%</v>
       </c>
     </row>
     <row r="370">
       <c r="A370">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B370" t="str">
-        <v>Starter Depot Spot (Kalos)</v>
+        <v>Sea Spirit Den Tunnels</v>
       </c>
       <c r="C370" t="str">
-        <v>Pelipper</v>
+        <v>Slugma</v>
       </c>
       <c r="D370" t="str">
-        <v>88-93</v>
+        <v>82-87</v>
       </c>
       <c r="E370" t="str">
-        <v>5%</v>
+        <v>25%</v>
       </c>
     </row>
     <row r="371">
@@ -6696,16 +6696,16 @@
         <v>68</v>
       </c>
       <c r="B371" t="str">
-        <v>Starter Depot Spot (Kanto)</v>
+        <v>Sea Spirit Den Tunnels</v>
       </c>
       <c r="C371" t="str">
-        <v>Bulbasaur</v>
+        <v>Axew</v>
       </c>
       <c r="D371" t="str">
-        <v>98-100</v>
+        <v>82-87</v>
       </c>
       <c r="E371" t="str">
-        <v>25%</v>
+        <v>20%</v>
       </c>
     </row>
     <row r="372">
@@ -6713,16 +6713,16 @@
         <v>68</v>
       </c>
       <c r="B372" t="str">
-        <v>Starter Depot Spot (Kanto)</v>
+        <v>Sea Spirit Den Tunnels</v>
       </c>
       <c r="C372" t="str">
-        <v>Ivysaur</v>
+        <v>Illumise</v>
       </c>
       <c r="D372" t="str">
-        <v>98-100</v>
+        <v>82-87</v>
       </c>
       <c r="E372" t="str">
-        <v>20%</v>
+        <v>15%</v>
       </c>
     </row>
     <row r="373">
@@ -6730,84 +6730,84 @@
         <v>68</v>
       </c>
       <c r="B373" t="str">
-        <v>Starter Depot Spot (Kanto)</v>
+        <v>Sea Spirit Den Tunnels</v>
       </c>
       <c r="C373" t="str">
-        <v>Charmeleon</v>
+        <v>Shuppet</v>
       </c>
       <c r="D373" t="str">
-        <v>98-100</v>
+        <v>82-87</v>
       </c>
       <c r="E373" t="str">
-        <v>20%</v>
+        <v>10%</v>
       </c>
     </row>
     <row r="374">
       <c r="A374">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B374" t="str">
-        <v>Starter Depot Spot (Kanto)</v>
+        <v>Chambers of Emptiness</v>
       </c>
       <c r="C374" t="str">
-        <v>Charmander</v>
+        <v>Flygon</v>
       </c>
       <c r="D374" t="str">
-        <v>98-100</v>
+        <v>70-75</v>
       </c>
       <c r="E374" t="str">
-        <v>15%</v>
+        <v>30%</v>
       </c>
     </row>
     <row r="375">
       <c r="A375">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B375" t="str">
-        <v>Starter Depot Spot (Kanto)</v>
+        <v>Chambers of Emptiness</v>
       </c>
       <c r="C375" t="str">
-        <v>Squirtle</v>
+        <v>Absol</v>
       </c>
       <c r="D375" t="str">
-        <v>98-100</v>
+        <v>70-75</v>
       </c>
       <c r="E375" t="str">
-        <v>10%</v>
+        <v>25%</v>
       </c>
     </row>
     <row r="376">
       <c r="A376">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B376" t="str">
-        <v>Starter Depot Spot (Kanto)</v>
+        <v>Chambers of Emptiness</v>
       </c>
       <c r="C376" t="str">
-        <v>Wartortle</v>
+        <v>Carvanha</v>
       </c>
       <c r="D376" t="str">
-        <v>98-100</v>
+        <v>70-75</v>
       </c>
       <c r="E376" t="str">
-        <v>5%</v>
+        <v>20%</v>
       </c>
     </row>
     <row r="377">
       <c r="A377">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B377" t="str">
-        <v>Starter Depot Spot (Kanto)</v>
+        <v>Chambers of Emptiness</v>
       </c>
       <c r="C377" t="str">
-        <v>Hoopa</v>
+        <v>Wooper</v>
       </c>
       <c r="D377" t="str">
-        <v>98-100</v>
+        <v>70-75</v>
       </c>
       <c r="E377" t="str">
-        <v>5%</v>
+        <v>15%</v>
       </c>
     </row>
     <row r="378">
@@ -6815,84 +6815,84 @@
         <v>69</v>
       </c>
       <c r="B378" t="str">
-        <v>Sea Spirit Den Entrance</v>
+        <v>Chambers of Emptiness</v>
       </c>
       <c r="C378" t="str">
-        <v>Qwilfish</v>
+        <v>Diancie</v>
       </c>
       <c r="D378" t="str">
         <v>70-75</v>
       </c>
       <c r="E378" t="str">
-        <v>30%</v>
+        <v>10%</v>
       </c>
     </row>
     <row r="379">
       <c r="A379">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B379" t="str">
-        <v>Sea Spirit Den Entrance</v>
+        <v>Team Flare Secret HQ Entrance</v>
       </c>
       <c r="C379" t="str">
-        <v>Reuniclus</v>
+        <v>Geodude</v>
       </c>
       <c r="D379" t="str">
-        <v>70-75</v>
+        <v>82-87</v>
       </c>
       <c r="E379" t="str">
-        <v>25%</v>
+        <v>30%</v>
       </c>
     </row>
     <row r="380">
       <c r="A380">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B380" t="str">
-        <v>Sea Spirit Den Entrance</v>
+        <v>Team Flare Secret HQ Entrance</v>
       </c>
       <c r="C380" t="str">
-        <v>Mothim</v>
+        <v>Hoppip</v>
       </c>
       <c r="D380" t="str">
-        <v>70-75</v>
+        <v>82-87</v>
       </c>
       <c r="E380" t="str">
-        <v>20%</v>
+        <v>25%</v>
       </c>
     </row>
     <row r="381">
       <c r="A381">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B381" t="str">
-        <v>Sea Spirit Den Entrance</v>
+        <v>Team Flare Secret HQ Entrance</v>
       </c>
       <c r="C381" t="str">
-        <v>Mawile</v>
+        <v>Aegislash</v>
       </c>
       <c r="D381" t="str">
-        <v>70-75</v>
+        <v>82-87</v>
       </c>
       <c r="E381" t="str">
-        <v>15%</v>
+        <v>20%</v>
       </c>
     </row>
     <row r="382">
       <c r="A382">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B382" t="str">
-        <v>Sea Spirit Den Entrance</v>
+        <v>Team Flare Secret HQ Entrance</v>
       </c>
       <c r="C382" t="str">
-        <v>Igglybuff</v>
+        <v>Slowpoke</v>
       </c>
       <c r="D382" t="str">
-        <v>70-75</v>
+        <v>82-87</v>
       </c>
       <c r="E382" t="str">
-        <v>10%</v>
+        <v>15%</v>
       </c>
     </row>
     <row r="383">
@@ -6900,84 +6900,84 @@
         <v>70</v>
       </c>
       <c r="B383" t="str">
-        <v>Sea Spirit Den Tunnels</v>
+        <v>Team Flare Secret HQ Entrance</v>
       </c>
       <c r="C383" t="str">
-        <v>Gogoat</v>
+        <v>Bagon</v>
       </c>
       <c r="D383" t="str">
         <v>82-87</v>
       </c>
       <c r="E383" t="str">
-        <v>30%</v>
+        <v>10%</v>
       </c>
     </row>
     <row r="384">
       <c r="A384">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B384" t="str">
-        <v>Sea Spirit Den Tunnels</v>
+        <v>Mystic Tower Entrance</v>
       </c>
       <c r="C384" t="str">
-        <v>Slugma</v>
+        <v>Oddish</v>
       </c>
       <c r="D384" t="str">
-        <v>82-87</v>
+        <v>70-75</v>
       </c>
       <c r="E384" t="str">
-        <v>25%</v>
+        <v>30%</v>
       </c>
     </row>
     <row r="385">
       <c r="A385">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B385" t="str">
-        <v>Sea Spirit Den Tunnels</v>
+        <v>Mystic Tower Entrance</v>
       </c>
       <c r="C385" t="str">
-        <v>Axew</v>
+        <v>Simipour</v>
       </c>
       <c r="D385" t="str">
-        <v>82-87</v>
+        <v>70-75</v>
       </c>
       <c r="E385" t="str">
-        <v>20%</v>
+        <v>25%</v>
       </c>
     </row>
     <row r="386">
       <c r="A386">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B386" t="str">
-        <v>Sea Spirit Den Tunnels</v>
+        <v>Mystic Tower Entrance</v>
       </c>
       <c r="C386" t="str">
-        <v>Illumise</v>
+        <v>Swirlix</v>
       </c>
       <c r="D386" t="str">
-        <v>82-87</v>
+        <v>70-75</v>
       </c>
       <c r="E386" t="str">
-        <v>15%</v>
+        <v>20%</v>
       </c>
     </row>
     <row r="387">
       <c r="A387">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B387" t="str">
-        <v>Sea Spirit Den Tunnels</v>
+        <v>Mystic Tower Entrance</v>
       </c>
       <c r="C387" t="str">
-        <v>Shuppet</v>
+        <v>Salamence</v>
       </c>
       <c r="D387" t="str">
-        <v>82-87</v>
+        <v>70-75</v>
       </c>
       <c r="E387" t="str">
-        <v>10%</v>
+        <v>15%</v>
       </c>
     </row>
     <row r="388">
@@ -6985,84 +6985,84 @@
         <v>71</v>
       </c>
       <c r="B388" t="str">
-        <v>Sea Spirit Den Hall</v>
+        <v>Mystic Tower Entrance</v>
       </c>
       <c r="C388" t="str">
-        <v>Moltres</v>
+        <v>Zorua</v>
       </c>
       <c r="D388" t="str">
-        <v>98-100</v>
+        <v>70-75</v>
       </c>
       <c r="E388" t="str">
-        <v>30%</v>
+        <v>10%</v>
       </c>
     </row>
     <row r="389">
       <c r="A389">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B389" t="str">
-        <v>Sea Spirit Den Hall</v>
+        <v>Crystal Cave Tunnels</v>
       </c>
       <c r="C389" t="str">
-        <v>Zapdos</v>
+        <v>Gyarados</v>
       </c>
       <c r="D389" t="str">
-        <v>98-100</v>
+        <v>78-83</v>
       </c>
       <c r="E389" t="str">
-        <v>25%</v>
+        <v>30%</v>
       </c>
     </row>
     <row r="390">
       <c r="A390">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B390" t="str">
-        <v>Sea Spirit Den Hall</v>
+        <v>Crystal Cave Tunnels</v>
       </c>
       <c r="C390" t="str">
-        <v>Articuno</v>
+        <v>Scrafty</v>
       </c>
       <c r="D390" t="str">
-        <v>98-100</v>
+        <v>78-83</v>
       </c>
       <c r="E390" t="str">
-        <v>20%</v>
+        <v>25%</v>
       </c>
     </row>
     <row r="391">
       <c r="A391">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B391" t="str">
-        <v>Sea Spirit Den Hall</v>
+        <v>Crystal Cave Tunnels</v>
       </c>
       <c r="C391" t="str">
-        <v>Politoed</v>
+        <v>Panpour</v>
       </c>
       <c r="D391" t="str">
-        <v>98-100</v>
+        <v>78-83</v>
       </c>
       <c r="E391" t="str">
-        <v>15%</v>
+        <v>20%</v>
       </c>
     </row>
     <row r="392">
       <c r="A392">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B392" t="str">
-        <v>Sea Spirit Den Hall</v>
+        <v>Crystal Cave Tunnels</v>
       </c>
       <c r="C392" t="str">
-        <v>Shedinja</v>
+        <v>Karrablast</v>
       </c>
       <c r="D392" t="str">
-        <v>98-100</v>
+        <v>78-83</v>
       </c>
       <c r="E392" t="str">
-        <v>10%</v>
+        <v>15%</v>
       </c>
     </row>
     <row r="393">
@@ -7070,84 +7070,84 @@
         <v>72</v>
       </c>
       <c r="B393" t="str">
-        <v>Chambers of Emptiness</v>
+        <v>Crystal Cave Tunnels</v>
       </c>
       <c r="C393" t="str">
-        <v>Flygon</v>
+        <v>Spinarak</v>
       </c>
       <c r="D393" t="str">
-        <v>70-75</v>
+        <v>78-83</v>
       </c>
       <c r="E393" t="str">
-        <v>30%</v>
+        <v>10%</v>
       </c>
     </row>
     <row r="394">
       <c r="A394">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B394" t="str">
-        <v>Chambers of Emptiness</v>
+        <v>Secret Forest North</v>
       </c>
       <c r="C394" t="str">
-        <v>Absol</v>
+        <v>Roggenrola</v>
       </c>
       <c r="D394" t="str">
-        <v>70-75</v>
+        <v>86-91</v>
       </c>
       <c r="E394" t="str">
-        <v>25%</v>
+        <v>30%</v>
       </c>
     </row>
     <row r="395">
       <c r="A395">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B395" t="str">
-        <v>Chambers of Emptiness</v>
+        <v>Secret Forest North</v>
       </c>
       <c r="C395" t="str">
-        <v>Carvanha</v>
+        <v>Swanna</v>
       </c>
       <c r="D395" t="str">
-        <v>70-75</v>
+        <v>86-91</v>
       </c>
       <c r="E395" t="str">
-        <v>20%</v>
+        <v>25%</v>
       </c>
     </row>
     <row r="396">
       <c r="A396">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B396" t="str">
-        <v>Chambers of Emptiness</v>
+        <v>Secret Forest North</v>
       </c>
       <c r="C396" t="str">
-        <v>Wooper</v>
+        <v>Whismur</v>
       </c>
       <c r="D396" t="str">
-        <v>70-75</v>
+        <v>86-91</v>
       </c>
       <c r="E396" t="str">
-        <v>15%</v>
+        <v>20%</v>
       </c>
     </row>
     <row r="397">
       <c r="A397">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B397" t="str">
-        <v>Chambers of Emptiness</v>
+        <v>Secret Forest North</v>
       </c>
       <c r="C397" t="str">
-        <v>Diancie</v>
+        <v>Solrock</v>
       </c>
       <c r="D397" t="str">
-        <v>70-75</v>
+        <v>86-91</v>
       </c>
       <c r="E397" t="str">
-        <v>10%</v>
+        <v>15%</v>
       </c>
     </row>
     <row r="398">
@@ -7155,84 +7155,84 @@
         <v>73</v>
       </c>
       <c r="B398" t="str">
-        <v>Team Flare Secret HQ Entrance</v>
+        <v>Secret Forest North</v>
       </c>
       <c r="C398" t="str">
-        <v>Geodude</v>
+        <v>Malamar</v>
       </c>
       <c r="D398" t="str">
-        <v>82-87</v>
+        <v>86-91</v>
       </c>
       <c r="E398" t="str">
-        <v>30%</v>
+        <v>10%</v>
       </c>
     </row>
     <row r="399">
       <c r="A399">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B399" t="str">
-        <v>Team Flare Secret HQ Entrance</v>
+        <v>Path to Sea Spirit Den</v>
       </c>
       <c r="C399" t="str">
-        <v>Hoppip</v>
+        <v>Vanilluxe</v>
       </c>
       <c r="D399" t="str">
-        <v>82-87</v>
+        <v>75-95</v>
       </c>
       <c r="E399" t="str">
-        <v>25%</v>
+        <v>30%</v>
       </c>
     </row>
     <row r="400">
       <c r="A400">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B400" t="str">
-        <v>Team Flare Secret HQ Entrance</v>
+        <v>Path to Sea Spirit Den</v>
       </c>
       <c r="C400" t="str">
-        <v>Aegislash</v>
+        <v>Chandelure</v>
       </c>
       <c r="D400" t="str">
-        <v>82-87</v>
+        <v>75-95</v>
       </c>
       <c r="E400" t="str">
-        <v>20%</v>
+        <v>25%</v>
       </c>
     </row>
     <row r="401">
       <c r="A401">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B401" t="str">
-        <v>Team Flare Secret HQ Entrance</v>
+        <v>Path to Sea Spirit Den</v>
       </c>
       <c r="C401" t="str">
-        <v>Slowpoke</v>
+        <v>Cubone</v>
       </c>
       <c r="D401" t="str">
-        <v>82-87</v>
+        <v>75-95</v>
       </c>
       <c r="E401" t="str">
-        <v>15%</v>
+        <v>20%</v>
       </c>
     </row>
     <row r="402">
       <c r="A402">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B402" t="str">
-        <v>Team Flare Secret HQ Entrance</v>
+        <v>Path to Sea Spirit Den</v>
       </c>
       <c r="C402" t="str">
-        <v>Bagon</v>
+        <v>Pawniard</v>
       </c>
       <c r="D402" t="str">
-        <v>82-87</v>
+        <v>75-95</v>
       </c>
       <c r="E402" t="str">
-        <v>10%</v>
+        <v>15%</v>
       </c>
     </row>
     <row r="403">
@@ -7240,84 +7240,84 @@
         <v>74</v>
       </c>
       <c r="B403" t="str">
-        <v>Team Flare Secret HQ Hall</v>
+        <v>Path to Sea Spirit Den</v>
       </c>
       <c r="C403" t="str">
-        <v>Yveltal</v>
+        <v>Aerodactyl</v>
       </c>
       <c r="D403" t="str">
-        <v>98-100</v>
+        <v>75-95</v>
       </c>
       <c r="E403" t="str">
-        <v>30%</v>
+        <v>10%</v>
       </c>
     </row>
     <row r="404">
       <c r="A404">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B404" t="str">
-        <v>Team Flare Secret HQ Hall</v>
+        <v>2nd spot for Extra Challenge B</v>
       </c>
       <c r="C404" t="str">
-        <v>Zygarde</v>
+        <v>Glaceon</v>
       </c>
       <c r="D404" t="str">
-        <v>98-100</v>
+        <v>75-95</v>
       </c>
       <c r="E404" t="str">
-        <v>25%</v>
+        <v>30%</v>
       </c>
     </row>
     <row r="405">
       <c r="A405">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B405" t="str">
-        <v>Team Flare Secret HQ Hall</v>
+        <v>2nd spot for Extra Challenge B</v>
       </c>
       <c r="C405" t="str">
-        <v>Xerneas</v>
+        <v>Haxorus</v>
       </c>
       <c r="D405" t="str">
-        <v>98-100</v>
+        <v>75-95</v>
       </c>
       <c r="E405" t="str">
-        <v>20%</v>
+        <v>25%</v>
       </c>
     </row>
     <row r="406">
       <c r="A406">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B406" t="str">
-        <v>Team Flare Secret HQ Hall</v>
+        <v>2nd spot for Extra Challenge B</v>
       </c>
       <c r="C406" t="str">
-        <v>Alomomola</v>
+        <v>Huntail</v>
       </c>
       <c r="D406" t="str">
-        <v>98-100</v>
+        <v>75-95</v>
       </c>
       <c r="E406" t="str">
-        <v>15%</v>
+        <v>20%</v>
       </c>
     </row>
     <row r="407">
       <c r="A407">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B407" t="str">
-        <v>Team Flare Secret HQ Hall</v>
+        <v>2nd spot for Extra Challenge B</v>
       </c>
       <c r="C407" t="str">
-        <v>Golem</v>
+        <v>Blastoise</v>
       </c>
       <c r="D407" t="str">
-        <v>98-100</v>
+        <v>75-95</v>
       </c>
       <c r="E407" t="str">
-        <v>10%</v>
+        <v>15%</v>
       </c>
     </row>
     <row r="408">
@@ -7325,84 +7325,84 @@
         <v>75</v>
       </c>
       <c r="B408" t="str">
-        <v>Mystic Tower Entrance</v>
+        <v>2nd spot for Extra Challenge B</v>
       </c>
       <c r="C408" t="str">
-        <v>Oddish</v>
+        <v>Avalugg</v>
       </c>
       <c r="D408" t="str">
-        <v>70-75</v>
+        <v>75-95</v>
       </c>
       <c r="E408" t="str">
-        <v>30%</v>
+        <v>10%</v>
       </c>
     </row>
     <row r="409">
       <c r="A409">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B409" t="str">
-        <v>Mystic Tower Entrance</v>
+        <v>Path to Team Flare Secret HQ</v>
       </c>
       <c r="C409" t="str">
-        <v>Simipour</v>
+        <v>Bunnelby</v>
       </c>
       <c r="D409" t="str">
-        <v>70-75</v>
+        <v>75-95</v>
       </c>
       <c r="E409" t="str">
-        <v>25%</v>
+        <v>30%</v>
       </c>
     </row>
     <row r="410">
       <c r="A410">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B410" t="str">
-        <v>Mystic Tower Entrance</v>
+        <v>Path to Team Flare Secret HQ</v>
       </c>
       <c r="C410" t="str">
-        <v>Swirlix</v>
+        <v>Throh</v>
       </c>
       <c r="D410" t="str">
-        <v>70-75</v>
+        <v>75-95</v>
       </c>
       <c r="E410" t="str">
-        <v>20%</v>
+        <v>25%</v>
       </c>
     </row>
     <row r="411">
       <c r="A411">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B411" t="str">
-        <v>Mystic Tower Entrance</v>
+        <v>Path to Team Flare Secret HQ</v>
       </c>
       <c r="C411" t="str">
-        <v>Salamence</v>
+        <v>Duosion</v>
       </c>
       <c r="D411" t="str">
-        <v>70-75</v>
+        <v>75-95</v>
       </c>
       <c r="E411" t="str">
-        <v>15%</v>
+        <v>20%</v>
       </c>
     </row>
     <row r="412">
       <c r="A412">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B412" t="str">
-        <v>Mystic Tower Entrance</v>
+        <v>Path to Team Flare Secret HQ</v>
       </c>
       <c r="C412" t="str">
-        <v>Zorua</v>
+        <v>Raichu</v>
       </c>
       <c r="D412" t="str">
-        <v>70-75</v>
+        <v>75-95</v>
       </c>
       <c r="E412" t="str">
-        <v>10%</v>
+        <v>15%</v>
       </c>
     </row>
     <row r="413">
@@ -7410,84 +7410,84 @@
         <v>76</v>
       </c>
       <c r="B413" t="str">
-        <v>Crystal Cave Tunnels</v>
+        <v>Path to Team Flare Secret HQ</v>
       </c>
       <c r="C413" t="str">
-        <v>Gyarados</v>
+        <v>Furfrou</v>
       </c>
       <c r="D413" t="str">
-        <v>78-83</v>
+        <v>75-95</v>
       </c>
       <c r="E413" t="str">
-        <v>30%</v>
+        <v>10%</v>
       </c>
     </row>
     <row r="414">
       <c r="A414">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B414" t="str">
-        <v>Crystal Cave Tunnels</v>
+        <v>2nd spot for Extra Challenge C</v>
       </c>
       <c r="C414" t="str">
-        <v>Scrafty</v>
+        <v>Jynx</v>
       </c>
       <c r="D414" t="str">
-        <v>78-83</v>
+        <v>75-95</v>
       </c>
       <c r="E414" t="str">
-        <v>25%</v>
+        <v>30%</v>
       </c>
     </row>
     <row r="415">
       <c r="A415">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B415" t="str">
-        <v>Crystal Cave Tunnels</v>
+        <v>2nd spot for Extra Challenge C</v>
       </c>
       <c r="C415" t="str">
-        <v>Panpour</v>
+        <v>Yveltal</v>
       </c>
       <c r="D415" t="str">
-        <v>78-83</v>
+        <v>75-95</v>
       </c>
       <c r="E415" t="str">
-        <v>20%</v>
+        <v>25%</v>
       </c>
     </row>
     <row r="416">
       <c r="A416">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B416" t="str">
-        <v>Crystal Cave Tunnels</v>
+        <v>2nd spot for Extra Challenge C</v>
       </c>
       <c r="C416" t="str">
-        <v>Karrablast</v>
+        <v>Exeggcute</v>
       </c>
       <c r="D416" t="str">
-        <v>78-83</v>
+        <v>75-95</v>
       </c>
       <c r="E416" t="str">
-        <v>15%</v>
+        <v>20%</v>
       </c>
     </row>
     <row r="417">
       <c r="A417">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B417" t="str">
-        <v>Crystal Cave Tunnels</v>
+        <v>2nd spot for Extra Challenge C</v>
       </c>
       <c r="C417" t="str">
-        <v>Spinarak</v>
+        <v>Tentacruel</v>
       </c>
       <c r="D417" t="str">
-        <v>78-83</v>
+        <v>75-95</v>
       </c>
       <c r="E417" t="str">
-        <v>10%</v>
+        <v>15%</v>
       </c>
     </row>
     <row r="418">
@@ -7495,84 +7495,84 @@
         <v>77</v>
       </c>
       <c r="B418" t="str">
-        <v>Secret Forest North</v>
+        <v>2nd spot for Extra Challenge C</v>
       </c>
       <c r="C418" t="str">
-        <v>Roggenrola</v>
+        <v>Roserade</v>
       </c>
       <c r="D418" t="str">
-        <v>86-91</v>
+        <v>75-95</v>
       </c>
       <c r="E418" t="str">
-        <v>30%</v>
+        <v>10%</v>
       </c>
     </row>
     <row r="419">
       <c r="A419">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B419" t="str">
-        <v>Secret Forest North</v>
+        <v>Team Flare Secret HQ Gate</v>
       </c>
       <c r="C419" t="str">
-        <v>Swanna</v>
+        <v>Barboach</v>
       </c>
       <c r="D419" t="str">
-        <v>86-91</v>
+        <v>75-95</v>
       </c>
       <c r="E419" t="str">
-        <v>25%</v>
+        <v>30%</v>
       </c>
     </row>
     <row r="420">
       <c r="A420">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B420" t="str">
-        <v>Secret Forest North</v>
+        <v>Team Flare Secret HQ Gate</v>
       </c>
       <c r="C420" t="str">
-        <v>Whismur</v>
+        <v>Gulpin</v>
       </c>
       <c r="D420" t="str">
-        <v>86-91</v>
+        <v>75-95</v>
       </c>
       <c r="E420" t="str">
-        <v>20%</v>
+        <v>25%</v>
       </c>
     </row>
     <row r="421">
       <c r="A421">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B421" t="str">
-        <v>Secret Forest North</v>
+        <v>Team Flare Secret HQ Gate</v>
       </c>
       <c r="C421" t="str">
-        <v>Solrock</v>
+        <v>Pinsir</v>
       </c>
       <c r="D421" t="str">
-        <v>86-91</v>
+        <v>75-95</v>
       </c>
       <c r="E421" t="str">
-        <v>15%</v>
+        <v>20%</v>
       </c>
     </row>
     <row r="422">
       <c r="A422">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B422" t="str">
-        <v>Secret Forest North</v>
+        <v>Team Flare Secret HQ Gate</v>
       </c>
       <c r="C422" t="str">
-        <v>Malamar</v>
+        <v>Dragalge</v>
       </c>
       <c r="D422" t="str">
-        <v>86-91</v>
+        <v>75-95</v>
       </c>
       <c r="E422" t="str">
-        <v>10%</v>
+        <v>15%</v>
       </c>
     </row>
     <row r="423">
@@ -7580,113 +7580,657 @@
         <v>78</v>
       </c>
       <c r="B423" t="str">
-        <v>Ultimate Chamber</v>
+        <v>Team Flare Secret HQ Gate</v>
       </c>
       <c r="C423" t="str">
-        <v>Volcanion</v>
+        <v>Quagsire</v>
       </c>
       <c r="D423" t="str">
-        <v>98-100</v>
+        <v>75-95</v>
       </c>
       <c r="E423" t="str">
-        <v>30%</v>
+        <v>10%</v>
       </c>
     </row>
     <row r="424">
       <c r="A424">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B424" t="str">
-        <v>Ultimate Chamber</v>
+        <v>Path to Secret Ruins</v>
       </c>
       <c r="C424" t="str">
-        <v>Diancie</v>
+        <v>Hydreigon</v>
       </c>
       <c r="D424" t="str">
-        <v>98-100</v>
+        <v>75-95</v>
       </c>
       <c r="E424" t="str">
-        <v>25%</v>
+        <v>30%</v>
       </c>
     </row>
     <row r="425">
       <c r="A425">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B425" t="str">
-        <v>Ultimate Chamber</v>
+        <v>Path to Secret Ruins</v>
       </c>
       <c r="C425" t="str">
-        <v>Hoopa</v>
+        <v>Sandslash</v>
       </c>
       <c r="D425" t="str">
-        <v>98-100</v>
+        <v>75-95</v>
       </c>
       <c r="E425" t="str">
-        <v>15%</v>
+        <v>25%</v>
       </c>
     </row>
     <row r="426">
       <c r="A426">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B426" t="str">
-        <v>Ultimate Chamber</v>
+        <v>Path to Secret Ruins</v>
       </c>
       <c r="C426" t="str">
-        <v>Mewtwo</v>
+        <v>Cubchoo</v>
       </c>
       <c r="D426" t="str">
-        <v>98-100</v>
+        <v>75-95</v>
       </c>
       <c r="E426" t="str">
-        <v>15%</v>
+        <v>20%</v>
       </c>
     </row>
     <row r="427">
       <c r="A427">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B427" t="str">
-        <v>Ultimate Chamber</v>
+        <v>Path to Secret Ruins</v>
       </c>
       <c r="C427" t="str">
-        <v>Chatot</v>
+        <v>Zigzagoon</v>
       </c>
       <c r="D427" t="str">
-        <v>98-100</v>
+        <v>75-95</v>
       </c>
       <c r="E427" t="str">
-        <v>10%</v>
+        <v>15%</v>
       </c>
     </row>
     <row r="428">
       <c r="A428">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B428" t="str">
+        <v>Path to Secret Ruins</v>
+      </c>
+      <c r="C428" t="str">
+        <v>Bellossom</v>
+      </c>
+      <c r="D428" t="str">
+        <v>75-95</v>
+      </c>
+      <c r="E428" t="str">
+        <v>10%</v>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429">
+        <v>80</v>
+      </c>
+      <c r="B429" t="str">
+        <v>Underground Chambers (Crystal Cave Tunnels)</v>
+      </c>
+      <c r="C429" t="str">
+        <v>Bergmite</v>
+      </c>
+      <c r="D429" t="str">
+        <v>75-95</v>
+      </c>
+      <c r="E429" t="str">
+        <v>30%</v>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430">
+        <v>80</v>
+      </c>
+      <c r="B430" t="str">
+        <v>Underground Chambers (Crystal Cave Tunnels)</v>
+      </c>
+      <c r="C430" t="str">
+        <v>Carbink</v>
+      </c>
+      <c r="D430" t="str">
+        <v>75-95</v>
+      </c>
+      <c r="E430" t="str">
+        <v>25%</v>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431">
+        <v>80</v>
+      </c>
+      <c r="B431" t="str">
+        <v>Underground Chambers (Crystal Cave Tunnels)</v>
+      </c>
+      <c r="C431" t="str">
+        <v>Skitty</v>
+      </c>
+      <c r="D431" t="str">
+        <v>75-95</v>
+      </c>
+      <c r="E431" t="str">
+        <v>20%</v>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432">
+        <v>80</v>
+      </c>
+      <c r="B432" t="str">
+        <v>Underground Chambers (Crystal Cave Tunnels)</v>
+      </c>
+      <c r="C432" t="str">
+        <v>Golbat</v>
+      </c>
+      <c r="D432" t="str">
+        <v>75-95</v>
+      </c>
+      <c r="E432" t="str">
+        <v>15%</v>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433">
+        <v>80</v>
+      </c>
+      <c r="B433" t="str">
+        <v>Underground Chambers (Crystal Cave Tunnels)</v>
+      </c>
+      <c r="C433" t="str">
+        <v>Phantump</v>
+      </c>
+      <c r="D433" t="str">
+        <v>75-95</v>
+      </c>
+      <c r="E433" t="str">
+        <v>10%</v>
+      </c>
+    </row>
+    <row r="434">
+      <c r="A434">
+        <v>81</v>
+      </c>
+      <c r="B434" t="str">
+        <v>Garden Chambers (Secret Forest North)</v>
+      </c>
+      <c r="C434" t="str">
+        <v>Goomy</v>
+      </c>
+      <c r="D434" t="str">
+        <v>75-95</v>
+      </c>
+      <c r="E434" t="str">
+        <v>30%</v>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435">
+        <v>81</v>
+      </c>
+      <c r="B435" t="str">
+        <v>Garden Chambers (Secret Forest North)</v>
+      </c>
+      <c r="C435" t="str">
+        <v>Carnivine</v>
+      </c>
+      <c r="D435" t="str">
+        <v>75-95</v>
+      </c>
+      <c r="E435" t="str">
+        <v>25%</v>
+      </c>
+    </row>
+    <row r="436">
+      <c r="A436">
+        <v>81</v>
+      </c>
+      <c r="B436" t="str">
+        <v>Garden Chambers (Secret Forest North)</v>
+      </c>
+      <c r="C436" t="str">
+        <v>Swellow</v>
+      </c>
+      <c r="D436" t="str">
+        <v>75-95</v>
+      </c>
+      <c r="E436" t="str">
+        <v>20%</v>
+      </c>
+    </row>
+    <row r="437">
+      <c r="A437">
+        <v>81</v>
+      </c>
+      <c r="B437" t="str">
+        <v>Garden Chambers (Secret Forest North)</v>
+      </c>
+      <c r="C437" t="str">
+        <v>Magnemite</v>
+      </c>
+      <c r="D437" t="str">
+        <v>75-95</v>
+      </c>
+      <c r="E437" t="str">
+        <v>15%</v>
+      </c>
+    </row>
+    <row r="438">
+      <c r="A438">
+        <v>81</v>
+      </c>
+      <c r="B438" t="str">
+        <v>Garden Chambers (Secret Forest North)</v>
+      </c>
+      <c r="C438" t="str">
+        <v>Gastly</v>
+      </c>
+      <c r="D438" t="str">
+        <v>75-95</v>
+      </c>
+      <c r="E438" t="str">
+        <v>10%</v>
+      </c>
+    </row>
+    <row r="439">
+      <c r="A439">
+        <v>82</v>
+      </c>
+      <c r="B439" t="str">
+        <v>Starter Depot</v>
+      </c>
+      <c r="C439" t="str">
+        <v>Rowlet</v>
+      </c>
+      <c r="D439" t="str">
+        <v>40-45</v>
+      </c>
+      <c r="E439" t="str">
+        <v>16.66%</v>
+      </c>
+    </row>
+    <row r="440">
+      <c r="A440">
+        <v>82</v>
+      </c>
+      <c r="B440" t="str">
+        <v>Starter Depot</v>
+      </c>
+      <c r="C440" t="str">
+        <v>Litten</v>
+      </c>
+      <c r="D440" t="str">
+        <v>40-45</v>
+      </c>
+      <c r="E440" t="str">
+        <v>16.66%</v>
+      </c>
+    </row>
+    <row r="441">
+      <c r="A441">
+        <v>82</v>
+      </c>
+      <c r="B441" t="str">
+        <v>Starter Depot</v>
+      </c>
+      <c r="C441" t="str">
+        <v>Popplio</v>
+      </c>
+      <c r="D441" t="str">
+        <v>40-45</v>
+      </c>
+      <c r="E441" t="str">
+        <v>16.66%</v>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442">
+        <v>82</v>
+      </c>
+      <c r="B442" t="str">
+        <v>Starter Depot</v>
+      </c>
+      <c r="C442" t="str">
+        <v>Bulbasaur</v>
+      </c>
+      <c r="D442" t="str">
+        <v>40-45</v>
+      </c>
+      <c r="E442" t="str">
+        <v>16.66%</v>
+      </c>
+    </row>
+    <row r="443">
+      <c r="A443">
+        <v>82</v>
+      </c>
+      <c r="B443" t="str">
+        <v>Starter Depot</v>
+      </c>
+      <c r="C443" t="str">
+        <v>Charmander</v>
+      </c>
+      <c r="D443" t="str">
+        <v>40-45</v>
+      </c>
+      <c r="E443" t="str">
+        <v>16.66%</v>
+      </c>
+    </row>
+    <row r="444">
+      <c r="A444">
+        <v>82</v>
+      </c>
+      <c r="B444" t="str">
+        <v>Starter Depot</v>
+      </c>
+      <c r="C444" t="str">
+        <v>Squirtle</v>
+      </c>
+      <c r="D444" t="str">
+        <v>40-45</v>
+      </c>
+      <c r="E444" t="str">
+        <v>16.66%</v>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445">
+        <v>83</v>
+      </c>
+      <c r="B445" t="str">
+        <v>Starter Evolved Depot</v>
+      </c>
+      <c r="C445" t="str">
+        <v>Dartrix</v>
+      </c>
+      <c r="D445" t="str">
+        <v>45-50</v>
+      </c>
+      <c r="E445" t="str">
+        <v>16.66%</v>
+      </c>
+    </row>
+    <row r="446">
+      <c r="A446">
+        <v>83</v>
+      </c>
+      <c r="B446" t="str">
+        <v>Starter Evolved Depot</v>
+      </c>
+      <c r="C446" t="str">
+        <v>Torracat</v>
+      </c>
+      <c r="D446" t="str">
+        <v>45-50</v>
+      </c>
+      <c r="E446" t="str">
+        <v>16.66%</v>
+      </c>
+    </row>
+    <row r="447">
+      <c r="A447">
+        <v>83</v>
+      </c>
+      <c r="B447" t="str">
+        <v>Starter Evolved Depot</v>
+      </c>
+      <c r="C447" t="str">
+        <v>Brionne</v>
+      </c>
+      <c r="D447" t="str">
+        <v>45-50</v>
+      </c>
+      <c r="E447" t="str">
+        <v>16.66%</v>
+      </c>
+    </row>
+    <row r="448">
+      <c r="A448">
+        <v>83</v>
+      </c>
+      <c r="B448" t="str">
+        <v>Starter Evolved Depot</v>
+      </c>
+      <c r="C448" t="str">
+        <v>Ivysaur</v>
+      </c>
+      <c r="D448" t="str">
+        <v>45-50</v>
+      </c>
+      <c r="E448" t="str">
+        <v>16.66%</v>
+      </c>
+    </row>
+    <row r="449">
+      <c r="A449">
+        <v>83</v>
+      </c>
+      <c r="B449" t="str">
+        <v>Starter Evolved Depot</v>
+      </c>
+      <c r="C449" t="str">
+        <v>Charmeleon</v>
+      </c>
+      <c r="D449" t="str">
+        <v>45-50</v>
+      </c>
+      <c r="E449" t="str">
+        <v>16.66%</v>
+      </c>
+    </row>
+    <row r="450">
+      <c r="A450">
+        <v>83</v>
+      </c>
+      <c r="B450" t="str">
+        <v>Starter Evolved Depot</v>
+      </c>
+      <c r="C450" t="str">
+        <v>Blastoise</v>
+      </c>
+      <c r="D450" t="str">
+        <v>45-50</v>
+      </c>
+      <c r="E450" t="str">
+        <v>16.66%</v>
+      </c>
+    </row>
+    <row r="451">
+      <c r="A451">
+        <v>84</v>
+      </c>
+      <c r="B451" t="str">
         <v>Ultimate Chamber</v>
       </c>
-      <c r="C428" t="str">
-        <v>Slowking</v>
-      </c>
-      <c r="D428" t="str">
-        <v>98-100</v>
-      </c>
-      <c r="E428" t="str">
-        <v>5%</v>
+      <c r="C451" t="str">
+        <v>Volcanion</v>
+      </c>
+      <c r="D451" t="str">
+        <v>100-110</v>
+      </c>
+      <c r="E451" t="str">
+        <v>25%</v>
+      </c>
+    </row>
+    <row r="452">
+      <c r="A452">
+        <v>84</v>
+      </c>
+      <c r="B452" t="str">
+        <v>Ultimate Chamber</v>
+      </c>
+      <c r="C452" t="str">
+        <v>Diancie</v>
+      </c>
+      <c r="D452" t="str">
+        <v>100-110</v>
+      </c>
+      <c r="E452" t="str">
+        <v>25%</v>
+      </c>
+    </row>
+    <row r="453">
+      <c r="A453">
+        <v>84</v>
+      </c>
+      <c r="B453" t="str">
+        <v>Ultimate Chamber</v>
+      </c>
+      <c r="C453" t="str">
+        <v>Hoopa</v>
+      </c>
+      <c r="D453" t="str">
+        <v>100-110</v>
+      </c>
+      <c r="E453" t="str">
+        <v>25%</v>
+      </c>
+    </row>
+    <row r="454">
+      <c r="A454">
+        <v>84</v>
+      </c>
+      <c r="B454" t="str">
+        <v>Ultimate Chamber</v>
+      </c>
+      <c r="C454" t="str">
+        <v>Mewtwo</v>
+      </c>
+      <c r="D454" t="str">
+        <v>100-110</v>
+      </c>
+      <c r="E454" t="str">
+        <v>25%</v>
+      </c>
+    </row>
+    <row r="455">
+      <c r="A455">
+        <v>85</v>
+      </c>
+      <c r="B455" t="str">
+        <v>Team Flare Secret HQ Hall</v>
+      </c>
+      <c r="C455" t="str">
+        <v>Yveltal</v>
+      </c>
+      <c r="D455" t="str">
+        <v>110-120</v>
+      </c>
+      <c r="E455" t="str">
+        <v>33%</v>
+      </c>
+    </row>
+    <row r="456">
+      <c r="A456">
+        <v>85</v>
+      </c>
+      <c r="B456" t="str">
+        <v>Team Flare Secret HQ Hall</v>
+      </c>
+      <c r="C456" t="str">
+        <v>Zygarde</v>
+      </c>
+      <c r="D456" t="str">
+        <v>110-120</v>
+      </c>
+      <c r="E456" t="str">
+        <v>33%</v>
+      </c>
+    </row>
+    <row r="457">
+      <c r="A457">
+        <v>85</v>
+      </c>
+      <c r="B457" t="str">
+        <v>Team Flare Secret HQ Hall</v>
+      </c>
+      <c r="C457" t="str">
+        <v>Xerneas</v>
+      </c>
+      <c r="D457" t="str">
+        <v>110-120</v>
+      </c>
+      <c r="E457" t="str">
+        <v>33%</v>
+      </c>
+    </row>
+    <row r="458">
+      <c r="A458">
+        <v>86</v>
+      </c>
+      <c r="B458" t="str">
+        <v>Sea Spirit Den Hall</v>
+      </c>
+      <c r="C458" t="str">
+        <v>Articuno</v>
+      </c>
+      <c r="D458" t="str">
+        <v>100</v>
+      </c>
+      <c r="E458" t="str">
+        <v>33%</v>
+      </c>
+    </row>
+    <row r="459">
+      <c r="A459">
+        <v>86</v>
+      </c>
+      <c r="B459" t="str">
+        <v>Sea Spirit Den Hall</v>
+      </c>
+      <c r="C459" t="str">
+        <v>Zapdos</v>
+      </c>
+      <c r="D459" t="str">
+        <v>100</v>
+      </c>
+      <c r="E459" t="str">
+        <v>33%</v>
+      </c>
+    </row>
+    <row r="460">
+      <c r="A460">
+        <v>86</v>
+      </c>
+      <c r="B460" t="str">
+        <v>Sea Spirit Den Hall</v>
+      </c>
+      <c r="C460" t="str">
+        <v>Moltres</v>
+      </c>
+      <c r="D460" t="str">
+        <v>100</v>
+      </c>
+      <c r="E460" t="str">
+        <v>33%</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E428"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E460"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C75"/>
+  <dimension ref="A1:C84"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -8081,7 +8625,7 @@
         <v>Defeat the Gym Leader at Coumarine City Gym</v>
       </c>
       <c r="C36" t="str">
-        <v>Unlock Coumarine City (Fishing) AND Unlock Kiloude City</v>
+        <v>Unlock Coumarine City (Fishing) AND Unlock Starter Depot</v>
       </c>
     </row>
     <row r="37">
@@ -8383,139 +8927,238 @@
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>Final Challenge</v>
+        <v>Extra Challenge A 1</v>
       </c>
       <c r="B64" t="str">
-        <v>Defeat the Kalos Champion at Kalos Pokemon League</v>
+        <v>Capture 1 Rowlet and 1 Litten and 1 Popplio</v>
       </c>
       <c r="C64" t="str">
-        <v>Unlock Sea Spirit Den Entrance, Chambers of Emptiness, Mystic Tower Entrance</v>
+        <v>Unlock Starter Evolved Depot</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>Extra Challenge Starter 1</v>
+        <v>Extra Challenge A 2</v>
       </c>
       <c r="B65" t="str">
-        <v>Complete objectives in Kiloude City</v>
+        <v>Capture 1 Dartrix and 1 Torracat and 1 Brionne</v>
       </c>
       <c r="C65" t="str">
-        <v>Unlock Friend Safari</v>
+        <v>Unlock Kiloude City</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>Extra Challenge Starter 2</v>
+        <v>Extra Challenge A 3</v>
       </c>
       <c r="B66" t="str">
-        <v>Complete objectives in Friend Safari</v>
+        <v>Complete objectives in Kiloude City</v>
       </c>
       <c r="C66" t="str">
-        <v>Unlock Battle Maison</v>
+        <v>Unlock Friend Safari</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>Extra Challenge Starter 3</v>
+        <v>Extra Challenge A 4</v>
       </c>
       <c r="B67" t="str">
-        <v>Complete objectives in Battle Maison</v>
+        <v>Complete objectives in Friend Safari</v>
       </c>
       <c r="C67" t="str">
-        <v>Unlock Starter Depot Spot (Kalos)</v>
+        <v>Unlock Battle Maison</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>Extra Challenge Starter 4</v>
+        <v>Extra Challenge A 5</v>
       </c>
       <c r="B68" t="str">
-        <v>Defeat all Ultra Rares to access the Legendary Hall in Starter Depot Spot (Kalos)</v>
+        <v>Complete objectives in Battle Maison</v>
       </c>
       <c r="C68" t="str">
-        <v>Unlock Starter Depot Spot (Kanto)</v>
+        <v>Earn 1 Masterball</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>Extra Challenge B 1</v>
+        <v>Final Challenge</v>
       </c>
       <c r="B69" t="str">
-        <v>Complete objectives in Sea Spirit Den Entrance</v>
+        <v>Defeat the Kalos Champion at Kalos Pokemon League</v>
       </c>
       <c r="C69" t="str">
-        <v>Unlock Sea Spirit Den Tunnels</v>
+        <v>Unlock Path to Sea Spirit Den (first spot for Extra Challenge B), Path to Team Flare Secret HQ (first spot for Extra Challenge C), Path to Secret Ruins (first spot for Extra Challenge D)</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>Extra Challenge B 2</v>
+        <v>Extra Challenge B 1</v>
       </c>
       <c r="B70" t="str">
-        <v>Defeat all Ultra Rares to access the Legendary Hall in Sea Spirit Den Tunnels</v>
+        <v>Complete objectives on Path to Sea Spirit Den</v>
       </c>
       <c r="C70" t="str">
-        <v>Unlock Sea Spirit Den Hall</v>
+        <v>Unlock 2nd spot for Extra Challenge B</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>Extra Challenge C 1</v>
+        <v>Extra Challenge B 2</v>
       </c>
       <c r="B71" t="str">
-        <v>Complete objectives in Chambers of Emptiness</v>
+        <v>Complete objectives on 2nd spot for Extra Challenge B</v>
       </c>
       <c r="C71" t="str">
-        <v>Unlock Team Flare Secret HQ Entrance</v>
+        <v>Unlock Sea Spirit Den Entrance</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>Extra Challenge C 2</v>
+        <v>Extra Challenge B 3</v>
       </c>
       <c r="B72" t="str">
-        <v>Defeat all Ultra Rares to access the Legendary Hall in Team Flare Secret HQ Entrance</v>
+        <v>Complete objectives in Sea Spirit Den Entrance</v>
       </c>
       <c r="C72" t="str">
-        <v>Unlock Team Flare Secret HQ Hall</v>
+        <v>Unlock Sea Spirit Den Tunnels</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>Extra Challenge D 1</v>
+        <v>Extra Challenge B 4</v>
       </c>
       <c r="B73" t="str">
-        <v>Complete objectives in Mystic Tower Entrance</v>
+        <v>Complete objectives in Sea Spirit Den Tunnels</v>
       </c>
       <c r="C73" t="str">
-        <v>Unlock Crystal Cave Tunnels</v>
+        <v>Unlock Sea Spirit Den Hall</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>Extra Challenge D 2</v>
+        <v>Extra Challenge B 5</v>
       </c>
       <c r="B74" t="str">
-        <v>Complete objectives in Crystal Cave Tunnels</v>
+        <v>Capture 1 Articuno 1 Zapdos 1 Moltres</v>
       </c>
       <c r="C74" t="str">
-        <v>Unlock Secret Forest North</v>
+        <v>Earn 2 Masterball</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="str">
+        <v>Extra Challenge C 1</v>
+      </c>
+      <c r="B75" t="str">
+        <v>Complete objectives on Path to Team Flare Secret HQ</v>
+      </c>
+      <c r="C75" t="str">
+        <v>Unlock 2nd spot for Extra Challenge C</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="str">
+        <v>Extra Challenge C 2</v>
+      </c>
+      <c r="B76" t="str">
+        <v>Complete objectives on 2nd spot for Extra Challenge C</v>
+      </c>
+      <c r="C76" t="str">
+        <v>Unlock Team Flare Secret HQ Gate</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="str">
+        <v>Extra Challenge C 3</v>
+      </c>
+      <c r="B77" t="str">
+        <v>Complete objectives in Team Flare Secret HQ Gate</v>
+      </c>
+      <c r="C77" t="str">
+        <v>Unlock Team Flare Secret HQ Entrance</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="str">
+        <v>Extra Challenge C 4</v>
+      </c>
+      <c r="B78" t="str">
+        <v>Complete objectives in Team Flare Secret HQ Entrance</v>
+      </c>
+      <c r="C78" t="str">
+        <v>Unlock Team Flare Secret HQ Hall</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="str">
+        <v>Extra Challenge C 5</v>
+      </c>
+      <c r="B79" t="str">
+        <v>Capture 1 Ybeltal 1 Zygarde 1 Xerneas</v>
+      </c>
+      <c r="C79" t="str">
+        <v>Earn 2 Masterball</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="str">
+        <v>Extra Challenge D 1</v>
+      </c>
+      <c r="B80" t="str">
+        <v>Complete objectives on Path to Secret Ruins</v>
+      </c>
+      <c r="C80" t="str">
+        <v>Unlock Underground Chambers (Crystal Cave Tunnels)</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="str">
+        <v>Extra Challenge D 2</v>
+      </c>
+      <c r="B81" t="str">
+        <v>Complete objectives in Underground Chambers</v>
+      </c>
+      <c r="C81" t="str">
+        <v>Unlock Garden Chambers (Secret Forest North)</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="str">
         <v>Extra Challenge D 3</v>
       </c>
-      <c r="B75" t="str">
-        <v>Defeat all Ultra Rares to access the Legendary Hall in Secret Forest North</v>
-      </c>
-      <c r="C75" t="str">
+      <c r="B82" t="str">
+        <v>Complete objectives in Garden Chambers</v>
+      </c>
+      <c r="C82" t="str">
+        <v>Unlock Chambers of Emptiness</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="str">
+        <v>Extra Challenge D 4</v>
+      </c>
+      <c r="B83" t="str">
+        <v>Complete objectives in Chambers of Emptiness</v>
+      </c>
+      <c r="C83" t="str">
         <v>Unlock Ultimate Chamber</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="str">
+        <v>Extra Challenge D 5</v>
+      </c>
+      <c r="B84" t="str">
+        <v>Capture 1 Volcanion 1 Diance 1 Hoopa 1 Mewtwo</v>
+      </c>
+      <c r="C84" t="str">
+        <v>Earn 2 Masterball</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C75"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C84"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Finalize Kalos paths with precise Challenge renames and scaled level tiers
Co-authored-by: lsampaio1337-beep <246645260+lsampaio1337-beep@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Kalos_Path.xlsx
+++ b/Kalos_Path.xlsx
@@ -2061,7 +2061,7 @@
         <v>Grumpig</v>
       </c>
       <c r="D98" t="str">
-        <v>16-18</v>
+        <v>17-19</v>
       </c>
       <c r="E98" t="str">
         <v>30%</v>
@@ -2078,7 +2078,7 @@
         <v>Swalot</v>
       </c>
       <c r="D99" t="str">
-        <v>16-18</v>
+        <v>17-19</v>
       </c>
       <c r="E99" t="str">
         <v>25%</v>
@@ -2095,7 +2095,7 @@
         <v>Sandslash</v>
       </c>
       <c r="D100" t="str">
-        <v>16-18</v>
+        <v>17-19</v>
       </c>
       <c r="E100" t="str">
         <v>15%</v>
@@ -2112,7 +2112,7 @@
         <v>Litleo</v>
       </c>
       <c r="D101" t="str">
-        <v>16-18</v>
+        <v>17-19</v>
       </c>
       <c r="E101" t="str">
         <v>15%</v>
@@ -2129,7 +2129,7 @@
         <v>Shelmet</v>
       </c>
       <c r="D102" t="str">
-        <v>16-18</v>
+        <v>17-19</v>
       </c>
       <c r="E102" t="str">
         <v>10%</v>
@@ -2146,7 +2146,7 @@
         <v>Bisharp</v>
       </c>
       <c r="D103" t="str">
-        <v>16-18</v>
+        <v>17-19</v>
       </c>
       <c r="E103" t="str">
         <v>5%</v>
@@ -2163,7 +2163,7 @@
         <v>Nidoran-f</v>
       </c>
       <c r="D104" t="str">
-        <v>17-19</v>
+        <v>18-20</v>
       </c>
       <c r="E104" t="str">
         <v>30%</v>
@@ -2180,7 +2180,7 @@
         <v>Seadra</v>
       </c>
       <c r="D105" t="str">
-        <v>17-19</v>
+        <v>18-20</v>
       </c>
       <c r="E105" t="str">
         <v>25%</v>
@@ -2197,7 +2197,7 @@
         <v>Ferroseed</v>
       </c>
       <c r="D106" t="str">
-        <v>17-19</v>
+        <v>18-20</v>
       </c>
       <c r="E106" t="str">
         <v>15%</v>
@@ -2214,7 +2214,7 @@
         <v>Honedge</v>
       </c>
       <c r="D107" t="str">
-        <v>17-19</v>
+        <v>18-20</v>
       </c>
       <c r="E107" t="str">
         <v>15%</v>
@@ -2231,7 +2231,7 @@
         <v>Larvitar</v>
       </c>
       <c r="D108" t="str">
-        <v>17-19</v>
+        <v>18-20</v>
       </c>
       <c r="E108" t="str">
         <v>10%</v>
@@ -2248,7 +2248,7 @@
         <v>Spritzee</v>
       </c>
       <c r="D109" t="str">
-        <v>17-19</v>
+        <v>18-20</v>
       </c>
       <c r="E109" t="str">
         <v>5%</v>
@@ -2265,7 +2265,7 @@
         <v>Whirlipede</v>
       </c>
       <c r="D110" t="str">
-        <v>18-20</v>
+        <v>19-21</v>
       </c>
       <c r="E110" t="str">
         <v>30%</v>
@@ -2282,7 +2282,7 @@
         <v>Hariyama</v>
       </c>
       <c r="D111" t="str">
-        <v>18-20</v>
+        <v>19-21</v>
       </c>
       <c r="E111" t="str">
         <v>25%</v>
@@ -2299,7 +2299,7 @@
         <v>Lucario</v>
       </c>
       <c r="D112" t="str">
-        <v>18-20</v>
+        <v>19-21</v>
       </c>
       <c r="E112" t="str">
         <v>15%</v>
@@ -2316,7 +2316,7 @@
         <v>Volbeat</v>
       </c>
       <c r="D113" t="str">
-        <v>18-20</v>
+        <v>19-21</v>
       </c>
       <c r="E113" t="str">
         <v>15%</v>
@@ -2333,7 +2333,7 @@
         <v>Voltorb</v>
       </c>
       <c r="D114" t="str">
-        <v>18-20</v>
+        <v>19-21</v>
       </c>
       <c r="E114" t="str">
         <v>10%</v>
@@ -2350,7 +2350,7 @@
         <v>Flareon</v>
       </c>
       <c r="D115" t="str">
-        <v>18-20</v>
+        <v>19-21</v>
       </c>
       <c r="E115" t="str">
         <v>5%</v>
@@ -2367,7 +2367,7 @@
         <v>Krookodile</v>
       </c>
       <c r="D116" t="str">
-        <v>19-21</v>
+        <v>20-22</v>
       </c>
       <c r="E116" t="str">
         <v>30%</v>
@@ -2384,7 +2384,7 @@
         <v>Rotom</v>
       </c>
       <c r="D117" t="str">
-        <v>19-21</v>
+        <v>20-22</v>
       </c>
       <c r="E117" t="str">
         <v>25%</v>
@@ -2401,7 +2401,7 @@
         <v>Dunsparce</v>
       </c>
       <c r="D118" t="str">
-        <v>19-21</v>
+        <v>20-22</v>
       </c>
       <c r="E118" t="str">
         <v>15%</v>
@@ -2418,7 +2418,7 @@
         <v>Lunatone</v>
       </c>
       <c r="D119" t="str">
-        <v>19-21</v>
+        <v>20-22</v>
       </c>
       <c r="E119" t="str">
         <v>15%</v>
@@ -2435,7 +2435,7 @@
         <v>Machamp</v>
       </c>
       <c r="D120" t="str">
-        <v>19-21</v>
+        <v>20-22</v>
       </c>
       <c r="E120" t="str">
         <v>10%</v>
@@ -2452,7 +2452,7 @@
         <v>Alakazam</v>
       </c>
       <c r="D121" t="str">
-        <v>19-21</v>
+        <v>20-22</v>
       </c>
       <c r="E121" t="str">
         <v>5%</v>
@@ -2469,7 +2469,7 @@
         <v>Doduo</v>
       </c>
       <c r="D122" t="str">
-        <v>20-22</v>
+        <v>21-23</v>
       </c>
       <c r="E122" t="str">
         <v>30%</v>
@@ -2486,7 +2486,7 @@
         <v>Gourgeist</v>
       </c>
       <c r="D123" t="str">
-        <v>20-22</v>
+        <v>21-23</v>
       </c>
       <c r="E123" t="str">
         <v>25%</v>
@@ -2503,7 +2503,7 @@
         <v>Mienfoo</v>
       </c>
       <c r="D124" t="str">
-        <v>20-22</v>
+        <v>21-23</v>
       </c>
       <c r="E124" t="str">
         <v>15%</v>
@@ -2520,7 +2520,7 @@
         <v>Honchkrow</v>
       </c>
       <c r="D125" t="str">
-        <v>20-22</v>
+        <v>21-23</v>
       </c>
       <c r="E125" t="str">
         <v>15%</v>
@@ -2537,7 +2537,7 @@
         <v>Kadabra</v>
       </c>
       <c r="D126" t="str">
-        <v>20-22</v>
+        <v>21-23</v>
       </c>
       <c r="E126" t="str">
         <v>10%</v>
@@ -2554,7 +2554,7 @@
         <v>Drifblim</v>
       </c>
       <c r="D127" t="str">
-        <v>20-22</v>
+        <v>21-23</v>
       </c>
       <c r="E127" t="str">
         <v>5%</v>
@@ -2673,7 +2673,7 @@
         <v>Throh</v>
       </c>
       <c r="D134" t="str">
-        <v>23-25</v>
+        <v>25-30</v>
       </c>
       <c r="E134" t="str">
         <v>30%</v>
@@ -2690,7 +2690,7 @@
         <v>Skorupi</v>
       </c>
       <c r="D135" t="str">
-        <v>23-25</v>
+        <v>25-30</v>
       </c>
       <c r="E135" t="str">
         <v>25%</v>
@@ -2707,7 +2707,7 @@
         <v>Scraggy</v>
       </c>
       <c r="D136" t="str">
-        <v>23-25</v>
+        <v>25-30</v>
       </c>
       <c r="E136" t="str">
         <v>15%</v>
@@ -2724,7 +2724,7 @@
         <v>Hippowdon</v>
       </c>
       <c r="D137" t="str">
-        <v>23-25</v>
+        <v>25-30</v>
       </c>
       <c r="E137" t="str">
         <v>15%</v>
@@ -2741,7 +2741,7 @@
         <v>Spoink</v>
       </c>
       <c r="D138" t="str">
-        <v>23-25</v>
+        <v>25-30</v>
       </c>
       <c r="E138" t="str">
         <v>10%</v>
@@ -2758,7 +2758,7 @@
         <v>Tentacruel</v>
       </c>
       <c r="D139" t="str">
-        <v>23-25</v>
+        <v>25-30</v>
       </c>
       <c r="E139" t="str">
         <v>5%</v>
@@ -2775,7 +2775,7 @@
         <v>Poochyena</v>
       </c>
       <c r="D140" t="str">
-        <v>24-26</v>
+        <v>23-25</v>
       </c>
       <c r="E140" t="str">
         <v>30%</v>
@@ -2792,7 +2792,7 @@
         <v>Volcanion</v>
       </c>
       <c r="D141" t="str">
-        <v>24-26</v>
+        <v>23-25</v>
       </c>
       <c r="E141" t="str">
         <v>25%</v>
@@ -2809,7 +2809,7 @@
         <v>Huntail</v>
       </c>
       <c r="D142" t="str">
-        <v>24-26</v>
+        <v>23-25</v>
       </c>
       <c r="E142" t="str">
         <v>15%</v>
@@ -2826,7 +2826,7 @@
         <v>Rhyperior</v>
       </c>
       <c r="D143" t="str">
-        <v>24-26</v>
+        <v>23-25</v>
       </c>
       <c r="E143" t="str">
         <v>15%</v>
@@ -2843,7 +2843,7 @@
         <v>Delibird</v>
       </c>
       <c r="D144" t="str">
-        <v>24-26</v>
+        <v>23-25</v>
       </c>
       <c r="E144" t="str">
         <v>10%</v>
@@ -2860,7 +2860,7 @@
         <v>Gloom</v>
       </c>
       <c r="D145" t="str">
-        <v>24-26</v>
+        <v>23-25</v>
       </c>
       <c r="E145" t="str">
         <v>5%</v>
@@ -2877,7 +2877,7 @@
         <v>Zubat</v>
       </c>
       <c r="D146" t="str">
-        <v>25-27</v>
+        <v>24-26</v>
       </c>
       <c r="E146" t="str">
         <v>30%</v>
@@ -2894,7 +2894,7 @@
         <v>Lapras</v>
       </c>
       <c r="D147" t="str">
-        <v>25-27</v>
+        <v>24-26</v>
       </c>
       <c r="E147" t="str">
         <v>25%</v>
@@ -2911,7 +2911,7 @@
         <v>Pawniard</v>
       </c>
       <c r="D148" t="str">
-        <v>25-27</v>
+        <v>24-26</v>
       </c>
       <c r="E148" t="str">
         <v>15%</v>
@@ -2928,7 +2928,7 @@
         <v>Vanillite</v>
       </c>
       <c r="D149" t="str">
-        <v>25-27</v>
+        <v>24-26</v>
       </c>
       <c r="E149" t="str">
         <v>15%</v>
@@ -2945,7 +2945,7 @@
         <v>Yanmega</v>
       </c>
       <c r="D150" t="str">
-        <v>25-27</v>
+        <v>24-26</v>
       </c>
       <c r="E150" t="str">
         <v>10%</v>
@@ -2962,7 +2962,7 @@
         <v>Zoroark</v>
       </c>
       <c r="D151" t="str">
-        <v>25-27</v>
+        <v>24-26</v>
       </c>
       <c r="E151" t="str">
         <v>5%</v>
@@ -2979,7 +2979,7 @@
         <v>Magcargo</v>
       </c>
       <c r="D152" t="str">
-        <v>26-28</v>
+        <v>25-27</v>
       </c>
       <c r="E152" t="str">
         <v>30%</v>
@@ -2996,7 +2996,7 @@
         <v>Corsola</v>
       </c>
       <c r="D153" t="str">
-        <v>26-28</v>
+        <v>25-27</v>
       </c>
       <c r="E153" t="str">
         <v>25%</v>
@@ -3013,7 +3013,7 @@
         <v>Barboach</v>
       </c>
       <c r="D154" t="str">
-        <v>26-28</v>
+        <v>25-27</v>
       </c>
       <c r="E154" t="str">
         <v>15%</v>
@@ -3030,7 +3030,7 @@
         <v>Minun</v>
       </c>
       <c r="D155" t="str">
-        <v>26-28</v>
+        <v>25-27</v>
       </c>
       <c r="E155" t="str">
         <v>15%</v>
@@ -3047,7 +3047,7 @@
         <v>Mantine</v>
       </c>
       <c r="D156" t="str">
-        <v>26-28</v>
+        <v>25-27</v>
       </c>
       <c r="E156" t="str">
         <v>10%</v>
@@ -3064,7 +3064,7 @@
         <v>Poliwag</v>
       </c>
       <c r="D157" t="str">
-        <v>26-28</v>
+        <v>25-27</v>
       </c>
       <c r="E157" t="str">
         <v>5%</v>
@@ -3081,7 +3081,7 @@
         <v>Wailord</v>
       </c>
       <c r="D158" t="str">
-        <v>27-29</v>
+        <v>30-35</v>
       </c>
       <c r="E158" t="str">
         <v>30%</v>
@@ -3098,7 +3098,7 @@
         <v>Pyroar</v>
       </c>
       <c r="D159" t="str">
-        <v>27-29</v>
+        <v>30-35</v>
       </c>
       <c r="E159" t="str">
         <v>25%</v>
@@ -3115,7 +3115,7 @@
         <v>Escavalier</v>
       </c>
       <c r="D160" t="str">
-        <v>27-29</v>
+        <v>30-35</v>
       </c>
       <c r="E160" t="str">
         <v>15%</v>
@@ -3132,7 +3132,7 @@
         <v>Avalugg</v>
       </c>
       <c r="D161" t="str">
-        <v>27-29</v>
+        <v>30-35</v>
       </c>
       <c r="E161" t="str">
         <v>15%</v>
@@ -3149,7 +3149,7 @@
         <v>Aerodactyl</v>
       </c>
       <c r="D162" t="str">
-        <v>27-29</v>
+        <v>30-35</v>
       </c>
       <c r="E162" t="str">
         <v>10%</v>
@@ -3166,7 +3166,7 @@
         <v>Chimecho</v>
       </c>
       <c r="D163" t="str">
-        <v>27-29</v>
+        <v>30-35</v>
       </c>
       <c r="E163" t="str">
         <v>5%</v>
@@ -3183,7 +3183,7 @@
         <v>Lanturn</v>
       </c>
       <c r="D164" t="str">
-        <v>28-30</v>
+        <v>26-28</v>
       </c>
       <c r="E164" t="str">
         <v>30%</v>
@@ -3200,7 +3200,7 @@
         <v>Onix</v>
       </c>
       <c r="D165" t="str">
-        <v>28-30</v>
+        <v>26-28</v>
       </c>
       <c r="E165" t="str">
         <v>25%</v>
@@ -3217,7 +3217,7 @@
         <v>Nidoking</v>
       </c>
       <c r="D166" t="str">
-        <v>28-30</v>
+        <v>26-28</v>
       </c>
       <c r="E166" t="str">
         <v>15%</v>
@@ -3234,7 +3234,7 @@
         <v>Shuckle</v>
       </c>
       <c r="D167" t="str">
-        <v>28-30</v>
+        <v>26-28</v>
       </c>
       <c r="E167" t="str">
         <v>15%</v>
@@ -3251,7 +3251,7 @@
         <v>Yanma</v>
       </c>
       <c r="D168" t="str">
-        <v>28-30</v>
+        <v>26-28</v>
       </c>
       <c r="E168" t="str">
         <v>10%</v>
@@ -3268,7 +3268,7 @@
         <v>Meditite</v>
       </c>
       <c r="D169" t="str">
-        <v>28-30</v>
+        <v>26-28</v>
       </c>
       <c r="E169" t="str">
         <v>5%</v>
@@ -3285,7 +3285,7 @@
         <v>Glaceon</v>
       </c>
       <c r="D170" t="str">
-        <v>29-31</v>
+        <v>27-29</v>
       </c>
       <c r="E170" t="str">
         <v>30%</v>
@@ -3302,7 +3302,7 @@
         <v>Wailmer</v>
       </c>
       <c r="D171" t="str">
-        <v>29-31</v>
+        <v>27-29</v>
       </c>
       <c r="E171" t="str">
         <v>25%</v>
@@ -3319,7 +3319,7 @@
         <v>Sneasel</v>
       </c>
       <c r="D172" t="str">
-        <v>29-31</v>
+        <v>27-29</v>
       </c>
       <c r="E172" t="str">
         <v>15%</v>
@@ -3336,7 +3336,7 @@
         <v>Stunky</v>
       </c>
       <c r="D173" t="str">
-        <v>29-31</v>
+        <v>27-29</v>
       </c>
       <c r="E173" t="str">
         <v>15%</v>
@@ -3353,7 +3353,7 @@
         <v>Timburr</v>
       </c>
       <c r="D174" t="str">
-        <v>29-31</v>
+        <v>27-29</v>
       </c>
       <c r="E174" t="str">
         <v>10%</v>
@@ -3370,7 +3370,7 @@
         <v>Articuno</v>
       </c>
       <c r="D175" t="str">
-        <v>29-31</v>
+        <v>27-29</v>
       </c>
       <c r="E175" t="str">
         <v>5%</v>
@@ -3387,7 +3387,7 @@
         <v>Kangaskhan</v>
       </c>
       <c r="D176" t="str">
-        <v>30-32</v>
+        <v>35-40</v>
       </c>
       <c r="E176" t="str">
         <v>30%</v>
@@ -3404,7 +3404,7 @@
         <v>Haxorus</v>
       </c>
       <c r="D177" t="str">
-        <v>30-32</v>
+        <v>35-40</v>
       </c>
       <c r="E177" t="str">
         <v>25%</v>
@@ -3421,7 +3421,7 @@
         <v>Jumpluff</v>
       </c>
       <c r="D178" t="str">
-        <v>30-32</v>
+        <v>35-40</v>
       </c>
       <c r="E178" t="str">
         <v>15%</v>
@@ -3438,7 +3438,7 @@
         <v>Spewpa</v>
       </c>
       <c r="D179" t="str">
-        <v>30-32</v>
+        <v>35-40</v>
       </c>
       <c r="E179" t="str">
         <v>15%</v>
@@ -3455,7 +3455,7 @@
         <v>Doublade</v>
       </c>
       <c r="D180" t="str">
-        <v>30-32</v>
+        <v>35-40</v>
       </c>
       <c r="E180" t="str">
         <v>10%</v>
@@ -3472,7 +3472,7 @@
         <v>Raichu</v>
       </c>
       <c r="D181" t="str">
-        <v>30-32</v>
+        <v>35-40</v>
       </c>
       <c r="E181" t="str">
         <v>5%</v>
@@ -3489,7 +3489,7 @@
         <v>Pumpkaboo</v>
       </c>
       <c r="D182" t="str">
-        <v>31-33</v>
+        <v>28-30</v>
       </c>
       <c r="E182" t="str">
         <v>30%</v>
@@ -3506,7 +3506,7 @@
         <v>Butterfree</v>
       </c>
       <c r="D183" t="str">
-        <v>31-33</v>
+        <v>28-30</v>
       </c>
       <c r="E183" t="str">
         <v>25%</v>
@@ -3523,7 +3523,7 @@
         <v>Magneton</v>
       </c>
       <c r="D184" t="str">
-        <v>31-33</v>
+        <v>28-30</v>
       </c>
       <c r="E184" t="str">
         <v>15%</v>
@@ -3540,7 +3540,7 @@
         <v>Vanillish</v>
       </c>
       <c r="D185" t="str">
-        <v>31-33</v>
+        <v>28-30</v>
       </c>
       <c r="E185" t="str">
         <v>15%</v>
@@ -3557,7 +3557,7 @@
         <v>Sliggoo</v>
       </c>
       <c r="D186" t="str">
-        <v>31-33</v>
+        <v>28-30</v>
       </c>
       <c r="E186" t="str">
         <v>10%</v>
@@ -3574,7 +3574,7 @@
         <v>Bergmite</v>
       </c>
       <c r="D187" t="str">
-        <v>31-33</v>
+        <v>28-30</v>
       </c>
       <c r="E187" t="str">
         <v>5%</v>
@@ -3591,7 +3591,7 @@
         <v>Furfrou</v>
       </c>
       <c r="D188" t="str">
-        <v>32-35</v>
+        <v>29-32</v>
       </c>
       <c r="E188" t="str">
         <v>30%</v>
@@ -3608,7 +3608,7 @@
         <v>Nidoran-m</v>
       </c>
       <c r="D189" t="str">
-        <v>32-35</v>
+        <v>29-32</v>
       </c>
       <c r="E189" t="str">
         <v>25%</v>
@@ -3625,7 +3625,7 @@
         <v>Murkrow</v>
       </c>
       <c r="D190" t="str">
-        <v>32-35</v>
+        <v>29-32</v>
       </c>
       <c r="E190" t="str">
         <v>15%</v>
@@ -3642,7 +3642,7 @@
         <v>Electrode</v>
       </c>
       <c r="D191" t="str">
-        <v>32-35</v>
+        <v>29-32</v>
       </c>
       <c r="E191" t="str">
         <v>15%</v>
@@ -3659,7 +3659,7 @@
         <v>Farfetchd</v>
       </c>
       <c r="D192" t="str">
-        <v>32-35</v>
+        <v>29-32</v>
       </c>
       <c r="E192" t="str">
         <v>10%</v>
@@ -3676,7 +3676,7 @@
         <v>Taillow</v>
       </c>
       <c r="D193" t="str">
-        <v>32-35</v>
+        <v>29-32</v>
       </c>
       <c r="E193" t="str">
         <v>5%</v>
@@ -3693,7 +3693,7 @@
         <v>Ducklett</v>
       </c>
       <c r="D194" t="str">
-        <v>33-36</v>
+        <v>30-33</v>
       </c>
       <c r="E194" t="str">
         <v>30%</v>
@@ -3710,7 +3710,7 @@
         <v>Tyranitar</v>
       </c>
       <c r="D195" t="str">
-        <v>33-36</v>
+        <v>30-33</v>
       </c>
       <c r="E195" t="str">
         <v>25%</v>
@@ -3727,7 +3727,7 @@
         <v>Gulpin</v>
       </c>
       <c r="D196" t="str">
-        <v>33-36</v>
+        <v>30-33</v>
       </c>
       <c r="E196" t="str">
         <v>20%</v>
@@ -3744,7 +3744,7 @@
         <v>Swellow</v>
       </c>
       <c r="D197" t="str">
-        <v>33-36</v>
+        <v>30-33</v>
       </c>
       <c r="E197" t="str">
         <v>15%</v>
@@ -3761,7 +3761,7 @@
         <v>Skarmory</v>
       </c>
       <c r="D198" t="str">
-        <v>33-36</v>
+        <v>30-33</v>
       </c>
       <c r="E198" t="str">
         <v>10%</v>
@@ -3778,7 +3778,7 @@
         <v>Wormadam</v>
       </c>
       <c r="D199" t="str">
-        <v>34-37</v>
+        <v>40-45</v>
       </c>
       <c r="E199" t="str">
         <v>30%</v>
@@ -3795,7 +3795,7 @@
         <v>Quagsire</v>
       </c>
       <c r="D200" t="str">
-        <v>34-37</v>
+        <v>40-45</v>
       </c>
       <c r="E200" t="str">
         <v>25%</v>
@@ -3812,7 +3812,7 @@
         <v>Crustle</v>
       </c>
       <c r="D201" t="str">
-        <v>34-37</v>
+        <v>40-45</v>
       </c>
       <c r="E201" t="str">
         <v>20%</v>
@@ -3829,7 +3829,7 @@
         <v>Graveler</v>
       </c>
       <c r="D202" t="str">
-        <v>34-37</v>
+        <v>40-45</v>
       </c>
       <c r="E202" t="str">
         <v>15%</v>
@@ -3846,7 +3846,7 @@
         <v>Venusaur</v>
       </c>
       <c r="D203" t="str">
-        <v>34-37</v>
+        <v>40-45</v>
       </c>
       <c r="E203" t="str">
         <v>10%</v>
@@ -3863,7 +3863,7 @@
         <v>Machop</v>
       </c>
       <c r="D204" t="str">
-        <v>35-38</v>
+        <v>31-34</v>
       </c>
       <c r="E204" t="str">
         <v>30%</v>
@@ -3880,7 +3880,7 @@
         <v>Sudowoodo</v>
       </c>
       <c r="D205" t="str">
-        <v>35-38</v>
+        <v>31-34</v>
       </c>
       <c r="E205" t="str">
         <v>25%</v>
@@ -3897,7 +3897,7 @@
         <v>Budew</v>
       </c>
       <c r="D206" t="str">
-        <v>35-38</v>
+        <v>31-34</v>
       </c>
       <c r="E206" t="str">
         <v>20%</v>
@@ -3914,7 +3914,7 @@
         <v>Granbull</v>
       </c>
       <c r="D207" t="str">
-        <v>35-38</v>
+        <v>31-34</v>
       </c>
       <c r="E207" t="str">
         <v>15%</v>
@@ -3931,7 +3931,7 @@
         <v>Noibat</v>
       </c>
       <c r="D208" t="str">
-        <v>35-38</v>
+        <v>31-34</v>
       </c>
       <c r="E208" t="str">
         <v>10%</v>
@@ -3948,7 +3948,7 @@
         <v>Ekans</v>
       </c>
       <c r="D209" t="str">
-        <v>36-39</v>
+        <v>33-35</v>
       </c>
       <c r="E209" t="str">
         <v>30%</v>
@@ -3965,7 +3965,7 @@
         <v>Gardevoir</v>
       </c>
       <c r="D210" t="str">
-        <v>36-39</v>
+        <v>33-35</v>
       </c>
       <c r="E210" t="str">
         <v>25%</v>
@@ -3982,7 +3982,7 @@
         <v>Gothorita</v>
       </c>
       <c r="D211" t="str">
-        <v>36-39</v>
+        <v>33-35</v>
       </c>
       <c r="E211" t="str">
         <v>20%</v>
@@ -3999,7 +3999,7 @@
         <v>Sigilyph</v>
       </c>
       <c r="D212" t="str">
-        <v>36-39</v>
+        <v>33-35</v>
       </c>
       <c r="E212" t="str">
         <v>15%</v>
@@ -4016,7 +4016,7 @@
         <v>Foongus</v>
       </c>
       <c r="D213" t="str">
-        <v>36-39</v>
+        <v>33-35</v>
       </c>
       <c r="E213" t="str">
         <v>10%</v>
@@ -4033,7 +4033,7 @@
         <v>Medicham</v>
       </c>
       <c r="D214" t="str">
-        <v>37-40</v>
+        <v>34-36</v>
       </c>
       <c r="E214" t="str">
         <v>30%</v>
@@ -4050,7 +4050,7 @@
         <v>Piloswine</v>
       </c>
       <c r="D215" t="str">
-        <v>37-40</v>
+        <v>34-36</v>
       </c>
       <c r="E215" t="str">
         <v>25%</v>
@@ -4067,7 +4067,7 @@
         <v>Roserade</v>
       </c>
       <c r="D216" t="str">
-        <v>37-40</v>
+        <v>34-36</v>
       </c>
       <c r="E216" t="str">
         <v>20%</v>
@@ -4084,7 +4084,7 @@
         <v>Teddiursa</v>
       </c>
       <c r="D217" t="str">
-        <v>37-40</v>
+        <v>34-36</v>
       </c>
       <c r="E217" t="str">
         <v>15%</v>
@@ -4101,7 +4101,7 @@
         <v>Garbodor</v>
       </c>
       <c r="D218" t="str">
-        <v>37-40</v>
+        <v>34-36</v>
       </c>
       <c r="E218" t="str">
         <v>10%</v>
@@ -4118,7 +4118,7 @@
         <v>Bellsprout</v>
       </c>
       <c r="D219" t="str">
-        <v>38-41</v>
+        <v>35-37</v>
       </c>
       <c r="E219" t="str">
         <v>30%</v>
@@ -4135,7 +4135,7 @@
         <v>Hydreigon</v>
       </c>
       <c r="D220" t="str">
-        <v>38-41</v>
+        <v>35-37</v>
       </c>
       <c r="E220" t="str">
         <v>25%</v>
@@ -4152,7 +4152,7 @@
         <v>Exeggcute</v>
       </c>
       <c r="D221" t="str">
-        <v>38-41</v>
+        <v>35-37</v>
       </c>
       <c r="E221" t="str">
         <v>20%</v>
@@ -4169,7 +4169,7 @@
         <v>Skitty</v>
       </c>
       <c r="D222" t="str">
-        <v>38-41</v>
+        <v>35-37</v>
       </c>
       <c r="E222" t="str">
         <v>15%</v>
@@ -4186,7 +4186,7 @@
         <v>Sawk</v>
       </c>
       <c r="D223" t="str">
-        <v>38-41</v>
+        <v>35-37</v>
       </c>
       <c r="E223" t="str">
         <v>10%</v>
@@ -4203,7 +4203,7 @@
         <v>Chingling</v>
       </c>
       <c r="D224" t="str">
-        <v>39-42</v>
+        <v>36-39</v>
       </c>
       <c r="E224" t="str">
         <v>30%</v>
@@ -4220,7 +4220,7 @@
         <v>Exploud</v>
       </c>
       <c r="D225" t="str">
-        <v>39-42</v>
+        <v>36-39</v>
       </c>
       <c r="E225" t="str">
         <v>25%</v>
@@ -4237,7 +4237,7 @@
         <v>Inkay</v>
       </c>
       <c r="D226" t="str">
-        <v>39-42</v>
+        <v>36-39</v>
       </c>
       <c r="E226" t="str">
         <v>20%</v>
@@ -4254,7 +4254,7 @@
         <v>Skiddo</v>
       </c>
       <c r="D227" t="str">
-        <v>39-42</v>
+        <v>36-39</v>
       </c>
       <c r="E227" t="str">
         <v>15%</v>
@@ -4271,7 +4271,7 @@
         <v>Gastly</v>
       </c>
       <c r="D228" t="str">
-        <v>39-42</v>
+        <v>36-39</v>
       </c>
       <c r="E228" t="str">
         <v>10%</v>
@@ -4288,7 +4288,7 @@
         <v>Umbreon</v>
       </c>
       <c r="D229" t="str">
-        <v>40-44</v>
+        <v>37-40</v>
       </c>
       <c r="E229" t="str">
         <v>30%</v>
@@ -4305,7 +4305,7 @@
         <v>Trapinch</v>
       </c>
       <c r="D230" t="str">
-        <v>40-44</v>
+        <v>37-40</v>
       </c>
       <c r="E230" t="str">
         <v>25%</v>
@@ -4322,7 +4322,7 @@
         <v>Gorebyss</v>
       </c>
       <c r="D231" t="str">
-        <v>40-44</v>
+        <v>37-40</v>
       </c>
       <c r="E231" t="str">
         <v>20%</v>
@@ -4339,7 +4339,7 @@
         <v>Tauros</v>
       </c>
       <c r="D232" t="str">
-        <v>40-44</v>
+        <v>37-40</v>
       </c>
       <c r="E232" t="str">
         <v>15%</v>
@@ -4356,7 +4356,7 @@
         <v>Flabebe</v>
       </c>
       <c r="D233" t="str">
-        <v>40-44</v>
+        <v>37-40</v>
       </c>
       <c r="E233" t="str">
         <v>10%</v>
@@ -4373,7 +4373,7 @@
         <v>Shelgon</v>
       </c>
       <c r="D234" t="str">
-        <v>41-45</v>
+        <v>38-41</v>
       </c>
       <c r="E234" t="str">
         <v>30%</v>
@@ -4390,7 +4390,7 @@
         <v>Wobbuffet</v>
       </c>
       <c r="D235" t="str">
-        <v>41-45</v>
+        <v>38-41</v>
       </c>
       <c r="E235" t="str">
         <v>25%</v>
@@ -4407,7 +4407,7 @@
         <v>Loudred</v>
       </c>
       <c r="D236" t="str">
-        <v>41-45</v>
+        <v>38-41</v>
       </c>
       <c r="E236" t="str">
         <v>20%</v>
@@ -4424,7 +4424,7 @@
         <v>Bonsly</v>
       </c>
       <c r="D237" t="str">
-        <v>41-45</v>
+        <v>38-41</v>
       </c>
       <c r="E237" t="str">
         <v>15%</v>
@@ -4441,7 +4441,7 @@
         <v>Nosepass</v>
       </c>
       <c r="D238" t="str">
-        <v>41-45</v>
+        <v>38-41</v>
       </c>
       <c r="E238" t="str">
         <v>10%</v>
@@ -4458,7 +4458,7 @@
         <v>Rhydon</v>
       </c>
       <c r="D239" t="str">
-        <v>42-46</v>
+        <v>39-42</v>
       </c>
       <c r="E239" t="str">
         <v>30%</v>
@@ -4475,7 +4475,7 @@
         <v>Staraptor</v>
       </c>
       <c r="D240" t="str">
-        <v>42-46</v>
+        <v>39-42</v>
       </c>
       <c r="E240" t="str">
         <v>25%</v>
@@ -4492,7 +4492,7 @@
         <v>Goomy</v>
       </c>
       <c r="D241" t="str">
-        <v>42-46</v>
+        <v>39-42</v>
       </c>
       <c r="E241" t="str">
         <v>20%</v>
@@ -4509,7 +4509,7 @@
         <v>Torkoal</v>
       </c>
       <c r="D242" t="str">
-        <v>42-46</v>
+        <v>39-42</v>
       </c>
       <c r="E242" t="str">
         <v>15%</v>
@@ -4526,7 +4526,7 @@
         <v>Florges</v>
       </c>
       <c r="D243" t="str">
-        <v>42-46</v>
+        <v>39-42</v>
       </c>
       <c r="E243" t="str">
         <v>10%</v>
@@ -4543,7 +4543,7 @@
         <v>Golbat</v>
       </c>
       <c r="D244" t="str">
-        <v>44-47</v>
+        <v>40-43</v>
       </c>
       <c r="E244" t="str">
         <v>30%</v>
@@ -4560,7 +4560,7 @@
         <v>Drifloon</v>
       </c>
       <c r="D245" t="str">
-        <v>44-47</v>
+        <v>40-43</v>
       </c>
       <c r="E245" t="str">
         <v>25%</v>
@@ -4577,7 +4577,7 @@
         <v>Dwebble</v>
       </c>
       <c r="D246" t="str">
-        <v>44-47</v>
+        <v>40-43</v>
       </c>
       <c r="E246" t="str">
         <v>20%</v>
@@ -4594,7 +4594,7 @@
         <v>Zapdos</v>
       </c>
       <c r="D247" t="str">
-        <v>44-47</v>
+        <v>40-43</v>
       </c>
       <c r="E247" t="str">
         <v>15%</v>
@@ -4611,7 +4611,7 @@
         <v>Conkeldurr</v>
       </c>
       <c r="D248" t="str">
-        <v>44-47</v>
+        <v>40-43</v>
       </c>
       <c r="E248" t="str">
         <v>10%</v>
@@ -4628,7 +4628,7 @@
         <v>Dragonair</v>
       </c>
       <c r="D249" t="str">
-        <v>45-48</v>
+        <v>41-44</v>
       </c>
       <c r="E249" t="str">
         <v>30%</v>
@@ -4645,7 +4645,7 @@
         <v>Noctowl</v>
       </c>
       <c r="D250" t="str">
-        <v>45-48</v>
+        <v>41-44</v>
       </c>
       <c r="E250" t="str">
         <v>25%</v>
@@ -4662,7 +4662,7 @@
         <v>Gligar</v>
       </c>
       <c r="D251" t="str">
-        <v>45-48</v>
+        <v>41-44</v>
       </c>
       <c r="E251" t="str">
         <v>20%</v>
@@ -4679,7 +4679,7 @@
         <v>Lampent</v>
       </c>
       <c r="D252" t="str">
-        <v>45-48</v>
+        <v>41-44</v>
       </c>
       <c r="E252" t="str">
         <v>15%</v>
@@ -4696,7 +4696,7 @@
         <v>Ditto</v>
       </c>
       <c r="D253" t="str">
-        <v>45-48</v>
+        <v>41-44</v>
       </c>
       <c r="E253" t="str">
         <v>10%</v>
@@ -4713,7 +4713,7 @@
         <v>Relicanth</v>
       </c>
       <c r="D254" t="str">
-        <v>46-49</v>
+        <v>42-45</v>
       </c>
       <c r="E254" t="str">
         <v>30%</v>
@@ -4730,7 +4730,7 @@
         <v>Gothita</v>
       </c>
       <c r="D255" t="str">
-        <v>46-49</v>
+        <v>42-45</v>
       </c>
       <c r="E255" t="str">
         <v>25%</v>
@@ -4747,7 +4747,7 @@
         <v>Munchlax</v>
       </c>
       <c r="D256" t="str">
-        <v>46-49</v>
+        <v>42-45</v>
       </c>
       <c r="E256" t="str">
         <v>20%</v>
@@ -4764,7 +4764,7 @@
         <v>Gliscor</v>
       </c>
       <c r="D257" t="str">
-        <v>46-49</v>
+        <v>42-45</v>
       </c>
       <c r="E257" t="str">
         <v>15%</v>
@@ -4781,7 +4781,7 @@
         <v>Kakuna</v>
       </c>
       <c r="D258" t="str">
-        <v>46-49</v>
+        <v>42-45</v>
       </c>
       <c r="E258" t="str">
         <v>10%</v>
@@ -4798,7 +4798,7 @@
         <v>Patrat</v>
       </c>
       <c r="D259" t="str">
-        <v>47-50</v>
+        <v>43-47</v>
       </c>
       <c r="E259" t="str">
         <v>30%</v>
@@ -4815,7 +4815,7 @@
         <v>Dugtrio</v>
       </c>
       <c r="D260" t="str">
-        <v>47-50</v>
+        <v>43-47</v>
       </c>
       <c r="E260" t="str">
         <v>25%</v>
@@ -4832,7 +4832,7 @@
         <v>Hippopotas</v>
       </c>
       <c r="D261" t="str">
-        <v>47-50</v>
+        <v>43-47</v>
       </c>
       <c r="E261" t="str">
         <v>20%</v>
@@ -4849,7 +4849,7 @@
         <v>Ursaring</v>
       </c>
       <c r="D262" t="str">
-        <v>47-50</v>
+        <v>43-47</v>
       </c>
       <c r="E262" t="str">
         <v>15%</v>
@@ -4866,7 +4866,7 @@
         <v>Spinda</v>
       </c>
       <c r="D263" t="str">
-        <v>47-50</v>
+        <v>43-47</v>
       </c>
       <c r="E263" t="str">
         <v>10%</v>
@@ -4883,7 +4883,7 @@
         <v>Floatzel</v>
       </c>
       <c r="D264" t="str">
-        <v>48-51</v>
+        <v>44-48</v>
       </c>
       <c r="E264" t="str">
         <v>30%</v>
@@ -4900,7 +4900,7 @@
         <v>Marowak</v>
       </c>
       <c r="D265" t="str">
-        <v>48-51</v>
+        <v>44-48</v>
       </c>
       <c r="E265" t="str">
         <v>25%</v>
@@ -4917,7 +4917,7 @@
         <v>Mareep</v>
       </c>
       <c r="D266" t="str">
-        <v>48-51</v>
+        <v>44-48</v>
       </c>
       <c r="E266" t="str">
         <v>20%</v>
@@ -4934,7 +4934,7 @@
         <v>Spearow</v>
       </c>
       <c r="D267" t="str">
-        <v>48-51</v>
+        <v>44-48</v>
       </c>
       <c r="E267" t="str">
         <v>15%</v>
@@ -4951,7 +4951,7 @@
         <v>Weavile</v>
       </c>
       <c r="D268" t="str">
-        <v>48-51</v>
+        <v>44-48</v>
       </c>
       <c r="E268" t="str">
         <v>10%</v>
@@ -4968,7 +4968,7 @@
         <v>Swablu</v>
       </c>
       <c r="D269" t="str">
-        <v>49-53</v>
+        <v>45-49</v>
       </c>
       <c r="E269" t="str">
         <v>30%</v>
@@ -4985,7 +4985,7 @@
         <v>Clauncher</v>
       </c>
       <c r="D270" t="str">
-        <v>49-53</v>
+        <v>45-49</v>
       </c>
       <c r="E270" t="str">
         <v>25%</v>
@@ -5002,7 +5002,7 @@
         <v>Crawdaunt</v>
       </c>
       <c r="D271" t="str">
-        <v>49-53</v>
+        <v>45-49</v>
       </c>
       <c r="E271" t="str">
         <v>20%</v>
@@ -5019,7 +5019,7 @@
         <v>Skiploom</v>
       </c>
       <c r="D272" t="str">
-        <v>49-53</v>
+        <v>45-49</v>
       </c>
       <c r="E272" t="str">
         <v>15%</v>
@@ -5036,7 +5036,7 @@
         <v>Greninja</v>
       </c>
       <c r="D273" t="str">
-        <v>49-53</v>
+        <v>45-49</v>
       </c>
       <c r="E273" t="str">
         <v>10%</v>
@@ -5053,7 +5053,7 @@
         <v>Moltres</v>
       </c>
       <c r="D274" t="str">
-        <v>50-54</v>
+        <v>46-50</v>
       </c>
       <c r="E274" t="str">
         <v>30%</v>
@@ -5070,7 +5070,7 @@
         <v>Pansear</v>
       </c>
       <c r="D275" t="str">
-        <v>50-54</v>
+        <v>46-50</v>
       </c>
       <c r="E275" t="str">
         <v>25%</v>
@@ -5087,7 +5087,7 @@
         <v>Audino</v>
       </c>
       <c r="D276" t="str">
-        <v>50-54</v>
+        <v>46-50</v>
       </c>
       <c r="E276" t="str">
         <v>20%</v>
@@ -5104,7 +5104,7 @@
         <v>Flaaffy</v>
       </c>
       <c r="D277" t="str">
-        <v>50-54</v>
+        <v>46-50</v>
       </c>
       <c r="E277" t="str">
         <v>15%</v>
@@ -5121,7 +5121,7 @@
         <v>Durant</v>
       </c>
       <c r="D278" t="str">
-        <v>50-54</v>
+        <v>46-50</v>
       </c>
       <c r="E278" t="str">
         <v>10%</v>
@@ -5138,7 +5138,7 @@
         <v>Metapod</v>
       </c>
       <c r="D279" t="str">
-        <v>51-55</v>
+        <v>47-51</v>
       </c>
       <c r="E279" t="str">
         <v>30%</v>
@@ -5155,7 +5155,7 @@
         <v>Whiscash</v>
       </c>
       <c r="D280" t="str">
-        <v>51-55</v>
+        <v>47-51</v>
       </c>
       <c r="E280" t="str">
         <v>25%</v>
@@ -5172,7 +5172,7 @@
         <v>Lotad</v>
       </c>
       <c r="D281" t="str">
-        <v>51-55</v>
+        <v>47-51</v>
       </c>
       <c r="E281" t="str">
         <v>20%</v>
@@ -5189,7 +5189,7 @@
         <v>Caterpie</v>
       </c>
       <c r="D282" t="str">
-        <v>51-55</v>
+        <v>47-51</v>
       </c>
       <c r="E282" t="str">
         <v>15%</v>
@@ -5206,7 +5206,7 @@
         <v>Gigalith</v>
       </c>
       <c r="D283" t="str">
-        <v>51-55</v>
+        <v>47-51</v>
       </c>
       <c r="E283" t="str">
         <v>10%</v>
@@ -5223,7 +5223,7 @@
         <v>Pidgeot</v>
       </c>
       <c r="D284" t="str">
-        <v>52-56</v>
+        <v>49-52</v>
       </c>
       <c r="E284" t="str">
         <v>30%</v>
@@ -5240,7 +5240,7 @@
         <v>Golett</v>
       </c>
       <c r="D285" t="str">
-        <v>52-56</v>
+        <v>49-52</v>
       </c>
       <c r="E285" t="str">
         <v>25%</v>
@@ -5257,7 +5257,7 @@
         <v>Vespiquen</v>
       </c>
       <c r="D286" t="str">
-        <v>52-56</v>
+        <v>49-52</v>
       </c>
       <c r="E286" t="str">
         <v>20%</v>
@@ -5274,7 +5274,7 @@
         <v>Pidgey</v>
       </c>
       <c r="D287" t="str">
-        <v>52-56</v>
+        <v>49-52</v>
       </c>
       <c r="E287" t="str">
         <v>15%</v>
@@ -5291,7 +5291,7 @@
         <v>Liepard</v>
       </c>
       <c r="D288" t="str">
-        <v>52-56</v>
+        <v>49-52</v>
       </c>
       <c r="E288" t="str">
         <v>10%</v>
@@ -5308,7 +5308,7 @@
         <v>Bibarel</v>
       </c>
       <c r="D289" t="str">
-        <v>53-57</v>
+        <v>50-53</v>
       </c>
       <c r="E289" t="str">
         <v>30%</v>
@@ -5325,7 +5325,7 @@
         <v>Banette</v>
       </c>
       <c r="D290" t="str">
-        <v>53-57</v>
+        <v>50-53</v>
       </c>
       <c r="E290" t="str">
         <v>25%</v>
@@ -5342,7 +5342,7 @@
         <v>Dratini</v>
       </c>
       <c r="D291" t="str">
-        <v>53-57</v>
+        <v>50-53</v>
       </c>
       <c r="E291" t="str">
         <v>20%</v>
@@ -5359,7 +5359,7 @@
         <v>Haunter</v>
       </c>
       <c r="D292" t="str">
-        <v>53-57</v>
+        <v>50-53</v>
       </c>
       <c r="E292" t="str">
         <v>15%</v>
@@ -5376,7 +5376,7 @@
         <v>Ledian</v>
       </c>
       <c r="D293" t="str">
-        <v>53-57</v>
+        <v>50-53</v>
       </c>
       <c r="E293" t="str">
         <v>10%</v>
@@ -5393,7 +5393,7 @@
         <v>Azumarill</v>
       </c>
       <c r="D294" t="str">
-        <v>54-58</v>
+        <v>51-55</v>
       </c>
       <c r="E294" t="str">
         <v>30%</v>
@@ -5410,7 +5410,7 @@
         <v>Seaking</v>
       </c>
       <c r="D295" t="str">
-        <v>54-58</v>
+        <v>51-55</v>
       </c>
       <c r="E295" t="str">
         <v>25%</v>
@@ -5427,7 +5427,7 @@
         <v>Scatterbug</v>
       </c>
       <c r="D296" t="str">
-        <v>54-58</v>
+        <v>51-55</v>
       </c>
       <c r="E296" t="str">
         <v>20%</v>
@@ -5444,7 +5444,7 @@
         <v>Fletchling</v>
       </c>
       <c r="D297" t="str">
-        <v>54-58</v>
+        <v>51-55</v>
       </c>
       <c r="E297" t="str">
         <v>15%</v>
@@ -5461,7 +5461,7 @@
         <v>Remoraid</v>
       </c>
       <c r="D298" t="str">
-        <v>54-58</v>
+        <v>51-55</v>
       </c>
       <c r="E298" t="str">
         <v>10%</v>
@@ -5478,7 +5478,7 @@
         <v>Seviper</v>
       </c>
       <c r="D299" t="str">
-        <v>55-59</v>
+        <v>52-56</v>
       </c>
       <c r="E299" t="str">
         <v>30%</v>
@@ -5495,7 +5495,7 @@
         <v>Buizel</v>
       </c>
       <c r="D300" t="str">
-        <v>55-59</v>
+        <v>52-56</v>
       </c>
       <c r="E300" t="str">
         <v>25%</v>
@@ -5512,7 +5512,7 @@
         <v>Snover</v>
       </c>
       <c r="D301" t="str">
-        <v>55-59</v>
+        <v>52-56</v>
       </c>
       <c r="E301" t="str">
         <v>20%</v>
@@ -5529,7 +5529,7 @@
         <v>Aron</v>
       </c>
       <c r="D302" t="str">
-        <v>55-59</v>
+        <v>52-56</v>
       </c>
       <c r="E302" t="str">
         <v>15%</v>
@@ -5546,7 +5546,7 @@
         <v>Pichu</v>
       </c>
       <c r="D303" t="str">
-        <v>55-59</v>
+        <v>52-56</v>
       </c>
       <c r="E303" t="str">
         <v>10%</v>
@@ -5563,7 +5563,7 @@
         <v>Ralts</v>
       </c>
       <c r="D304" t="str">
-        <v>56-60</v>
+        <v>53-57</v>
       </c>
       <c r="E304" t="str">
         <v>30%</v>
@@ -5580,7 +5580,7 @@
         <v>Heatmor</v>
       </c>
       <c r="D305" t="str">
-        <v>56-60</v>
+        <v>53-57</v>
       </c>
       <c r="E305" t="str">
         <v>25%</v>
@@ -5597,7 +5597,7 @@
         <v>Shellder</v>
       </c>
       <c r="D306" t="str">
-        <v>56-60</v>
+        <v>53-57</v>
       </c>
       <c r="E306" t="str">
         <v>20%</v>
@@ -5614,7 +5614,7 @@
         <v>Gabite</v>
       </c>
       <c r="D307" t="str">
-        <v>56-60</v>
+        <v>53-57</v>
       </c>
       <c r="E307" t="str">
         <v>15%</v>
@@ -5631,7 +5631,7 @@
         <v>Aurorus</v>
       </c>
       <c r="D308" t="str">
-        <v>56-60</v>
+        <v>53-57</v>
       </c>
       <c r="E308" t="str">
         <v>10%</v>
@@ -5648,7 +5648,7 @@
         <v>Emolga</v>
       </c>
       <c r="D309" t="str">
-        <v>57-62</v>
+        <v>54-58</v>
       </c>
       <c r="E309" t="str">
         <v>30%</v>
@@ -5665,7 +5665,7 @@
         <v>Masquerain</v>
       </c>
       <c r="D310" t="str">
-        <v>57-62</v>
+        <v>54-58</v>
       </c>
       <c r="E310" t="str">
         <v>25%</v>
@@ -5682,7 +5682,7 @@
         <v>Noivern</v>
       </c>
       <c r="D311" t="str">
-        <v>57-62</v>
+        <v>54-58</v>
       </c>
       <c r="E311" t="str">
         <v>20%</v>
@@ -5699,7 +5699,7 @@
         <v>Binacle</v>
       </c>
       <c r="D312" t="str">
-        <v>57-62</v>
+        <v>54-58</v>
       </c>
       <c r="E312" t="str">
         <v>15%</v>
@@ -5716,7 +5716,7 @@
         <v>Swoobat</v>
       </c>
       <c r="D313" t="str">
-        <v>57-62</v>
+        <v>54-58</v>
       </c>
       <c r="E313" t="str">
         <v>10%</v>
@@ -5733,7 +5733,7 @@
         <v>Luvdisc</v>
       </c>
       <c r="D314" t="str">
-        <v>58-63</v>
+        <v>55-59</v>
       </c>
       <c r="E314" t="str">
         <v>30%</v>
@@ -5750,7 +5750,7 @@
         <v>Ariados</v>
       </c>
       <c r="D315" t="str">
-        <v>58-63</v>
+        <v>55-59</v>
       </c>
       <c r="E315" t="str">
         <v>25%</v>
@@ -5767,7 +5767,7 @@
         <v>Venipede</v>
       </c>
       <c r="D316" t="str">
-        <v>58-63</v>
+        <v>55-59</v>
       </c>
       <c r="E316" t="str">
         <v>20%</v>
@@ -5784,7 +5784,7 @@
         <v>Clamperl</v>
       </c>
       <c r="D317" t="str">
-        <v>58-63</v>
+        <v>55-59</v>
       </c>
       <c r="E317" t="str">
         <v>15%</v>
@@ -5801,7 +5801,7 @@
         <v>Mime-jr</v>
       </c>
       <c r="D318" t="str">
-        <v>58-63</v>
+        <v>55-59</v>
       </c>
       <c r="E318" t="str">
         <v>10%</v>
@@ -5818,7 +5818,7 @@
         <v>Toxicroak</v>
       </c>
       <c r="D319" t="str">
-        <v>59-64</v>
+        <v>56-60</v>
       </c>
       <c r="E319" t="str">
         <v>30%</v>
@@ -5835,7 +5835,7 @@
         <v>Surskit</v>
       </c>
       <c r="D320" t="str">
-        <v>59-64</v>
+        <v>56-60</v>
       </c>
       <c r="E320" t="str">
         <v>25%</v>
@@ -5852,7 +5852,7 @@
         <v>Zigzagoon</v>
       </c>
       <c r="D321" t="str">
-        <v>59-64</v>
+        <v>56-60</v>
       </c>
       <c r="E321" t="str">
         <v>20%</v>
@@ -5869,7 +5869,7 @@
         <v>Staryu</v>
       </c>
       <c r="D322" t="str">
-        <v>59-64</v>
+        <v>56-60</v>
       </c>
       <c r="E322" t="str">
         <v>15%</v>
@@ -5886,7 +5886,7 @@
         <v>Manectric</v>
       </c>
       <c r="D323" t="str">
-        <v>59-64</v>
+        <v>56-60</v>
       </c>
       <c r="E323" t="str">
         <v>10%</v>
@@ -5903,7 +5903,7 @@
         <v>Azurill</v>
       </c>
       <c r="D324" t="str">
-        <v>60-65</v>
+        <v>57-61</v>
       </c>
       <c r="E324" t="str">
         <v>30%</v>
@@ -5920,7 +5920,7 @@
         <v>Xerneas</v>
       </c>
       <c r="D325" t="str">
-        <v>60-65</v>
+        <v>57-61</v>
       </c>
       <c r="E325" t="str">
         <v>25%</v>
@@ -5937,7 +5937,7 @@
         <v>Ferrothorn</v>
       </c>
       <c r="D326" t="str">
-        <v>60-65</v>
+        <v>57-61</v>
       </c>
       <c r="E326" t="str">
         <v>20%</v>
@@ -5954,7 +5954,7 @@
         <v>Kecleon</v>
       </c>
       <c r="D327" t="str">
-        <v>60-65</v>
+        <v>57-61</v>
       </c>
       <c r="E327" t="str">
         <v>15%</v>
@@ -5971,7 +5971,7 @@
         <v>Jolteon</v>
       </c>
       <c r="D328" t="str">
-        <v>60-65</v>
+        <v>57-61</v>
       </c>
       <c r="E328" t="str">
         <v>10%</v>
@@ -5988,7 +5988,7 @@
         <v>Leafeon</v>
       </c>
       <c r="D329" t="str">
-        <v>61-66</v>
+        <v>58-63</v>
       </c>
       <c r="E329" t="str">
         <v>30%</v>
@@ -6005,7 +6005,7 @@
         <v>Weedle</v>
       </c>
       <c r="D330" t="str">
-        <v>61-66</v>
+        <v>58-63</v>
       </c>
       <c r="E330" t="str">
         <v>25%</v>
@@ -6022,7 +6022,7 @@
         <v>Croagunk</v>
       </c>
       <c r="D331" t="str">
-        <v>61-66</v>
+        <v>58-63</v>
       </c>
       <c r="E331" t="str">
         <v>20%</v>
@@ -6039,7 +6039,7 @@
         <v>Lickitung</v>
       </c>
       <c r="D332" t="str">
-        <v>61-66</v>
+        <v>58-63</v>
       </c>
       <c r="E332" t="str">
         <v>15%</v>
@@ -6056,7 +6056,7 @@
         <v>Aggron</v>
       </c>
       <c r="D333" t="str">
-        <v>61-66</v>
+        <v>58-63</v>
       </c>
       <c r="E333" t="str">
         <v>10%</v>
@@ -6073,7 +6073,7 @@
         <v>Octillery</v>
       </c>
       <c r="D334" t="str">
-        <v>62-67</v>
+        <v>59-64</v>
       </c>
       <c r="E334" t="str">
         <v>30%</v>
@@ -6090,7 +6090,7 @@
         <v>Pansage</v>
       </c>
       <c r="D335" t="str">
-        <v>62-67</v>
+        <v>59-64</v>
       </c>
       <c r="E335" t="str">
         <v>25%</v>
@@ -6107,7 +6107,7 @@
         <v>Corphish</v>
       </c>
       <c r="D336" t="str">
-        <v>62-67</v>
+        <v>59-64</v>
       </c>
       <c r="E336" t="str">
         <v>20%</v>
@@ -6124,7 +6124,7 @@
         <v>Garchomp</v>
       </c>
       <c r="D337" t="str">
-        <v>62-67</v>
+        <v>59-64</v>
       </c>
       <c r="E337" t="str">
         <v>15%</v>
@@ -6141,7 +6141,7 @@
         <v>Sentret</v>
       </c>
       <c r="D338" t="str">
-        <v>62-67</v>
+        <v>59-64</v>
       </c>
       <c r="E338" t="str">
         <v>10%</v>
@@ -6158,7 +6158,7 @@
         <v>Deino</v>
       </c>
       <c r="D339" t="str">
-        <v>63-68</v>
+        <v>60-65</v>
       </c>
       <c r="E339" t="str">
         <v>30%</v>
@@ -6175,7 +6175,7 @@
         <v>Magikarp</v>
       </c>
       <c r="D340" t="str">
-        <v>63-68</v>
+        <v>60-65</v>
       </c>
       <c r="E340" t="str">
         <v>25%</v>
@@ -6192,7 +6192,7 @@
         <v>Tyrunt</v>
       </c>
       <c r="D341" t="str">
-        <v>63-68</v>
+        <v>60-65</v>
       </c>
       <c r="E341" t="str">
         <v>20%</v>
@@ -6209,7 +6209,7 @@
         <v>Wingull</v>
       </c>
       <c r="D342" t="str">
-        <v>63-68</v>
+        <v>60-65</v>
       </c>
       <c r="E342" t="str">
         <v>15%</v>
@@ -6226,7 +6226,7 @@
         <v>Pancham</v>
       </c>
       <c r="D343" t="str">
-        <v>63-68</v>
+        <v>60-65</v>
       </c>
       <c r="E343" t="str">
         <v>10%</v>
@@ -6243,7 +6243,7 @@
         <v>Cloyster</v>
       </c>
       <c r="D344" t="str">
-        <v>65-70</v>
+        <v>61-66</v>
       </c>
       <c r="E344" t="str">
         <v>30%</v>
@@ -6260,7 +6260,7 @@
         <v>Lickilicky</v>
       </c>
       <c r="D345" t="str">
-        <v>65-70</v>
+        <v>61-66</v>
       </c>
       <c r="E345" t="str">
         <v>25%</v>
@@ -6277,7 +6277,7 @@
         <v>Floette</v>
       </c>
       <c r="D346" t="str">
-        <v>65-70</v>
+        <v>61-66</v>
       </c>
       <c r="E346" t="str">
         <v>20%</v>
@@ -6294,7 +6294,7 @@
         <v>Wynaut</v>
       </c>
       <c r="D347" t="str">
-        <v>65-70</v>
+        <v>61-66</v>
       </c>
       <c r="E347" t="str">
         <v>15%</v>
@@ -6311,7 +6311,7 @@
         <v>Amaura</v>
       </c>
       <c r="D348" t="str">
-        <v>65-70</v>
+        <v>61-66</v>
       </c>
       <c r="E348" t="str">
         <v>10%</v>
@@ -6328,7 +6328,7 @@
         <v>Tentacool</v>
       </c>
       <c r="D349" t="str">
-        <v>70-75</v>
+        <v>50-57</v>
       </c>
       <c r="E349" t="str">
         <v>30%</v>
@@ -6345,7 +6345,7 @@
         <v>Zygarde</v>
       </c>
       <c r="D350" t="str">
-        <v>70-75</v>
+        <v>50-57</v>
       </c>
       <c r="E350" t="str">
         <v>25%</v>
@@ -6362,7 +6362,7 @@
         <v>Cryogonal</v>
       </c>
       <c r="D351" t="str">
-        <v>70-75</v>
+        <v>50-57</v>
       </c>
       <c r="E351" t="str">
         <v>20%</v>
@@ -6379,7 +6379,7 @@
         <v>Espurr</v>
       </c>
       <c r="D352" t="str">
-        <v>70-75</v>
+        <v>50-57</v>
       </c>
       <c r="E352" t="str">
         <v>15%</v>
@@ -6396,7 +6396,7 @@
         <v>Ledyba</v>
       </c>
       <c r="D353" t="str">
-        <v>70-75</v>
+        <v>50-57</v>
       </c>
       <c r="E353" t="str">
         <v>10%</v>
@@ -6413,7 +6413,7 @@
         <v>Riolu</v>
       </c>
       <c r="D354" t="str">
-        <v>76-81</v>
+        <v>55-62</v>
       </c>
       <c r="E354" t="str">
         <v>30%</v>
@@ -6430,7 +6430,7 @@
         <v>Scyther</v>
       </c>
       <c r="D355" t="str">
-        <v>76-81</v>
+        <v>55-62</v>
       </c>
       <c r="E355" t="str">
         <v>25%</v>
@@ -6447,7 +6447,7 @@
         <v>Altaria</v>
       </c>
       <c r="D356" t="str">
-        <v>76-81</v>
+        <v>55-62</v>
       </c>
       <c r="E356" t="str">
         <v>20%</v>
@@ -6464,7 +6464,7 @@
         <v>Gothitelle</v>
       </c>
       <c r="D357" t="str">
-        <v>76-81</v>
+        <v>55-62</v>
       </c>
       <c r="E357" t="str">
         <v>15%</v>
@@ -6481,7 +6481,7 @@
         <v>Psyduck</v>
       </c>
       <c r="D358" t="str">
-        <v>76-81</v>
+        <v>55-62</v>
       </c>
       <c r="E358" t="str">
         <v>10%</v>
@@ -6498,7 +6498,7 @@
         <v>Druddigon</v>
       </c>
       <c r="D359" t="str">
-        <v>82-87</v>
+        <v>63-70</v>
       </c>
       <c r="E359" t="str">
         <v>30%</v>
@@ -6515,7 +6515,7 @@
         <v>Mienshao</v>
       </c>
       <c r="D360" t="str">
-        <v>82-87</v>
+        <v>63-70</v>
       </c>
       <c r="E360" t="str">
         <v>25%</v>
@@ -6532,7 +6532,7 @@
         <v>Heracross</v>
       </c>
       <c r="D361" t="str">
-        <v>82-87</v>
+        <v>63-70</v>
       </c>
       <c r="E361" t="str">
         <v>20%</v>
@@ -6549,7 +6549,7 @@
         <v>Talonflame</v>
       </c>
       <c r="D362" t="str">
-        <v>82-87</v>
+        <v>63-70</v>
       </c>
       <c r="E362" t="str">
         <v>15%</v>
@@ -6566,7 +6566,7 @@
         <v>Skrelp</v>
       </c>
       <c r="D363" t="str">
-        <v>82-87</v>
+        <v>63-70</v>
       </c>
       <c r="E363" t="str">
         <v>10%</v>
@@ -6583,7 +6583,7 @@
         <v>Qwilfish</v>
       </c>
       <c r="D364" t="str">
-        <v>70-75</v>
+        <v>84-91</v>
       </c>
       <c r="E364" t="str">
         <v>30%</v>
@@ -6600,7 +6600,7 @@
         <v>Reuniclus</v>
       </c>
       <c r="D365" t="str">
-        <v>70-75</v>
+        <v>84-91</v>
       </c>
       <c r="E365" t="str">
         <v>25%</v>
@@ -6617,7 +6617,7 @@
         <v>Mothim</v>
       </c>
       <c r="D366" t="str">
-        <v>70-75</v>
+        <v>84-91</v>
       </c>
       <c r="E366" t="str">
         <v>20%</v>
@@ -6634,7 +6634,7 @@
         <v>Mawile</v>
       </c>
       <c r="D367" t="str">
-        <v>70-75</v>
+        <v>84-91</v>
       </c>
       <c r="E367" t="str">
         <v>15%</v>
@@ -6651,7 +6651,7 @@
         <v>Igglybuff</v>
       </c>
       <c r="D368" t="str">
-        <v>70-75</v>
+        <v>84-91</v>
       </c>
       <c r="E368" t="str">
         <v>10%</v>
@@ -6668,7 +6668,7 @@
         <v>Gogoat</v>
       </c>
       <c r="D369" t="str">
-        <v>82-87</v>
+        <v>91-98</v>
       </c>
       <c r="E369" t="str">
         <v>30%</v>
@@ -6685,7 +6685,7 @@
         <v>Slugma</v>
       </c>
       <c r="D370" t="str">
-        <v>82-87</v>
+        <v>91-98</v>
       </c>
       <c r="E370" t="str">
         <v>25%</v>
@@ -6702,7 +6702,7 @@
         <v>Axew</v>
       </c>
       <c r="D371" t="str">
-        <v>82-87</v>
+        <v>91-98</v>
       </c>
       <c r="E371" t="str">
         <v>20%</v>
@@ -6719,7 +6719,7 @@
         <v>Illumise</v>
       </c>
       <c r="D372" t="str">
-        <v>82-87</v>
+        <v>91-98</v>
       </c>
       <c r="E372" t="str">
         <v>15%</v>
@@ -6736,7 +6736,7 @@
         <v>Shuppet</v>
       </c>
       <c r="D373" t="str">
-        <v>82-87</v>
+        <v>91-98</v>
       </c>
       <c r="E373" t="str">
         <v>10%</v>
@@ -6753,7 +6753,7 @@
         <v>Flygon</v>
       </c>
       <c r="D374" t="str">
-        <v>70-75</v>
+        <v>91-98</v>
       </c>
       <c r="E374" t="str">
         <v>30%</v>
@@ -6770,7 +6770,7 @@
         <v>Absol</v>
       </c>
       <c r="D375" t="str">
-        <v>70-75</v>
+        <v>91-98</v>
       </c>
       <c r="E375" t="str">
         <v>25%</v>
@@ -6787,7 +6787,7 @@
         <v>Carvanha</v>
       </c>
       <c r="D376" t="str">
-        <v>70-75</v>
+        <v>91-98</v>
       </c>
       <c r="E376" t="str">
         <v>20%</v>
@@ -6804,7 +6804,7 @@
         <v>Wooper</v>
       </c>
       <c r="D377" t="str">
-        <v>70-75</v>
+        <v>91-98</v>
       </c>
       <c r="E377" t="str">
         <v>15%</v>
@@ -6821,7 +6821,7 @@
         <v>Diancie</v>
       </c>
       <c r="D378" t="str">
-        <v>70-75</v>
+        <v>91-98</v>
       </c>
       <c r="E378" t="str">
         <v>10%</v>
@@ -6838,7 +6838,7 @@
         <v>Geodude</v>
       </c>
       <c r="D379" t="str">
-        <v>82-87</v>
+        <v>91-98</v>
       </c>
       <c r="E379" t="str">
         <v>30%</v>
@@ -6855,7 +6855,7 @@
         <v>Hoppip</v>
       </c>
       <c r="D380" t="str">
-        <v>82-87</v>
+        <v>91-98</v>
       </c>
       <c r="E380" t="str">
         <v>25%</v>
@@ -6872,7 +6872,7 @@
         <v>Aegislash</v>
       </c>
       <c r="D381" t="str">
-        <v>82-87</v>
+        <v>91-98</v>
       </c>
       <c r="E381" t="str">
         <v>20%</v>
@@ -6889,7 +6889,7 @@
         <v>Slowpoke</v>
       </c>
       <c r="D382" t="str">
-        <v>82-87</v>
+        <v>91-98</v>
       </c>
       <c r="E382" t="str">
         <v>15%</v>
@@ -6906,7 +6906,7 @@
         <v>Bagon</v>
       </c>
       <c r="D383" t="str">
-        <v>82-87</v>
+        <v>91-98</v>
       </c>
       <c r="E383" t="str">
         <v>10%</v>
@@ -6923,7 +6923,7 @@
         <v>Oddish</v>
       </c>
       <c r="D384" t="str">
-        <v>70-75</v>
+        <v>62-67</v>
       </c>
       <c r="E384" t="str">
         <v>30%</v>
@@ -6940,7 +6940,7 @@
         <v>Simipour</v>
       </c>
       <c r="D385" t="str">
-        <v>70-75</v>
+        <v>62-67</v>
       </c>
       <c r="E385" t="str">
         <v>25%</v>
@@ -6957,7 +6957,7 @@
         <v>Swirlix</v>
       </c>
       <c r="D386" t="str">
-        <v>70-75</v>
+        <v>62-67</v>
       </c>
       <c r="E386" t="str">
         <v>20%</v>
@@ -6974,7 +6974,7 @@
         <v>Salamence</v>
       </c>
       <c r="D387" t="str">
-        <v>70-75</v>
+        <v>62-67</v>
       </c>
       <c r="E387" t="str">
         <v>15%</v>
@@ -6991,7 +6991,7 @@
         <v>Zorua</v>
       </c>
       <c r="D388" t="str">
-        <v>70-75</v>
+        <v>62-67</v>
       </c>
       <c r="E388" t="str">
         <v>10%</v>
@@ -7008,7 +7008,7 @@
         <v>Gyarados</v>
       </c>
       <c r="D389" t="str">
-        <v>78-83</v>
+        <v>63-68</v>
       </c>
       <c r="E389" t="str">
         <v>30%</v>
@@ -7025,7 +7025,7 @@
         <v>Scrafty</v>
       </c>
       <c r="D390" t="str">
-        <v>78-83</v>
+        <v>63-68</v>
       </c>
       <c r="E390" t="str">
         <v>25%</v>
@@ -7042,7 +7042,7 @@
         <v>Panpour</v>
       </c>
       <c r="D391" t="str">
-        <v>78-83</v>
+        <v>63-68</v>
       </c>
       <c r="E391" t="str">
         <v>20%</v>
@@ -7059,7 +7059,7 @@
         <v>Karrablast</v>
       </c>
       <c r="D392" t="str">
-        <v>78-83</v>
+        <v>63-68</v>
       </c>
       <c r="E392" t="str">
         <v>15%</v>
@@ -7076,7 +7076,7 @@
         <v>Spinarak</v>
       </c>
       <c r="D393" t="str">
-        <v>78-83</v>
+        <v>63-68</v>
       </c>
       <c r="E393" t="str">
         <v>10%</v>
@@ -7093,7 +7093,7 @@
         <v>Roggenrola</v>
       </c>
       <c r="D394" t="str">
-        <v>86-91</v>
+        <v>65-70</v>
       </c>
       <c r="E394" t="str">
         <v>30%</v>
@@ -7110,7 +7110,7 @@
         <v>Swanna</v>
       </c>
       <c r="D395" t="str">
-        <v>86-91</v>
+        <v>65-70</v>
       </c>
       <c r="E395" t="str">
         <v>25%</v>
@@ -7127,7 +7127,7 @@
         <v>Whismur</v>
       </c>
       <c r="D396" t="str">
-        <v>86-91</v>
+        <v>65-70</v>
       </c>
       <c r="E396" t="str">
         <v>20%</v>
@@ -7144,7 +7144,7 @@
         <v>Solrock</v>
       </c>
       <c r="D397" t="str">
-        <v>86-91</v>
+        <v>65-70</v>
       </c>
       <c r="E397" t="str">
         <v>15%</v>
@@ -7161,7 +7161,7 @@
         <v>Malamar</v>
       </c>
       <c r="D398" t="str">
-        <v>86-91</v>
+        <v>65-70</v>
       </c>
       <c r="E398" t="str">
         <v>10%</v>
@@ -7178,7 +7178,7 @@
         <v>Vanilluxe</v>
       </c>
       <c r="D399" t="str">
-        <v>75-95</v>
+        <v>70-77</v>
       </c>
       <c r="E399" t="str">
         <v>30%</v>
@@ -7195,7 +7195,7 @@
         <v>Chandelure</v>
       </c>
       <c r="D400" t="str">
-        <v>75-95</v>
+        <v>70-77</v>
       </c>
       <c r="E400" t="str">
         <v>25%</v>
@@ -7212,7 +7212,7 @@
         <v>Cubone</v>
       </c>
       <c r="D401" t="str">
-        <v>75-95</v>
+        <v>70-77</v>
       </c>
       <c r="E401" t="str">
         <v>20%</v>
@@ -7229,7 +7229,7 @@
         <v>Pawniard</v>
       </c>
       <c r="D402" t="str">
-        <v>75-95</v>
+        <v>70-77</v>
       </c>
       <c r="E402" t="str">
         <v>15%</v>
@@ -7246,7 +7246,7 @@
         <v>Aerodactyl</v>
       </c>
       <c r="D403" t="str">
-        <v>75-95</v>
+        <v>70-77</v>
       </c>
       <c r="E403" t="str">
         <v>10%</v>
@@ -7257,13 +7257,13 @@
         <v>75</v>
       </c>
       <c r="B404" t="str">
-        <v>2nd spot for Extra Challenge B</v>
+        <v>Sea Spirit Den Outer Depths</v>
       </c>
       <c r="C404" t="str">
         <v>Glaceon</v>
       </c>
       <c r="D404" t="str">
-        <v>75-95</v>
+        <v>77-84</v>
       </c>
       <c r="E404" t="str">
         <v>30%</v>
@@ -7274,13 +7274,13 @@
         <v>75</v>
       </c>
       <c r="B405" t="str">
-        <v>2nd spot for Extra Challenge B</v>
+        <v>Sea Spirit Den Outer Depths</v>
       </c>
       <c r="C405" t="str">
         <v>Haxorus</v>
       </c>
       <c r="D405" t="str">
-        <v>75-95</v>
+        <v>77-84</v>
       </c>
       <c r="E405" t="str">
         <v>25%</v>
@@ -7291,13 +7291,13 @@
         <v>75</v>
       </c>
       <c r="B406" t="str">
-        <v>2nd spot for Extra Challenge B</v>
+        <v>Sea Spirit Den Outer Depths</v>
       </c>
       <c r="C406" t="str">
         <v>Huntail</v>
       </c>
       <c r="D406" t="str">
-        <v>75-95</v>
+        <v>77-84</v>
       </c>
       <c r="E406" t="str">
         <v>20%</v>
@@ -7308,13 +7308,13 @@
         <v>75</v>
       </c>
       <c r="B407" t="str">
-        <v>2nd spot for Extra Challenge B</v>
+        <v>Sea Spirit Den Outer Depths</v>
       </c>
       <c r="C407" t="str">
         <v>Blastoise</v>
       </c>
       <c r="D407" t="str">
-        <v>75-95</v>
+        <v>77-84</v>
       </c>
       <c r="E407" t="str">
         <v>15%</v>
@@ -7325,13 +7325,13 @@
         <v>75</v>
       </c>
       <c r="B408" t="str">
-        <v>2nd spot for Extra Challenge B</v>
+        <v>Sea Spirit Den Outer Depths</v>
       </c>
       <c r="C408" t="str">
         <v>Avalugg</v>
       </c>
       <c r="D408" t="str">
-        <v>75-95</v>
+        <v>77-84</v>
       </c>
       <c r="E408" t="str">
         <v>10%</v>
@@ -7348,7 +7348,7 @@
         <v>Bunnelby</v>
       </c>
       <c r="D409" t="str">
-        <v>75-95</v>
+        <v>70-77</v>
       </c>
       <c r="E409" t="str">
         <v>30%</v>
@@ -7365,7 +7365,7 @@
         <v>Throh</v>
       </c>
       <c r="D410" t="str">
-        <v>75-95</v>
+        <v>70-77</v>
       </c>
       <c r="E410" t="str">
         <v>25%</v>
@@ -7382,7 +7382,7 @@
         <v>Duosion</v>
       </c>
       <c r="D411" t="str">
-        <v>75-95</v>
+        <v>70-77</v>
       </c>
       <c r="E411" t="str">
         <v>20%</v>
@@ -7399,7 +7399,7 @@
         <v>Raichu</v>
       </c>
       <c r="D412" t="str">
-        <v>75-95</v>
+        <v>70-77</v>
       </c>
       <c r="E412" t="str">
         <v>15%</v>
@@ -7416,7 +7416,7 @@
         <v>Furfrou</v>
       </c>
       <c r="D413" t="str">
-        <v>75-95</v>
+        <v>70-77</v>
       </c>
       <c r="E413" t="str">
         <v>10%</v>
@@ -7427,13 +7427,13 @@
         <v>77</v>
       </c>
       <c r="B414" t="str">
-        <v>2nd spot for Extra Challenge C</v>
+        <v>2nd spot for Extra Challenge E</v>
       </c>
       <c r="C414" t="str">
         <v>Jynx</v>
       </c>
       <c r="D414" t="str">
-        <v>75-95</v>
+        <v>77-84</v>
       </c>
       <c r="E414" t="str">
         <v>30%</v>
@@ -7444,13 +7444,13 @@
         <v>77</v>
       </c>
       <c r="B415" t="str">
-        <v>2nd spot for Extra Challenge C</v>
+        <v>2nd spot for Extra Challenge E</v>
       </c>
       <c r="C415" t="str">
         <v>Yveltal</v>
       </c>
       <c r="D415" t="str">
-        <v>75-95</v>
+        <v>77-84</v>
       </c>
       <c r="E415" t="str">
         <v>25%</v>
@@ -7461,13 +7461,13 @@
         <v>77</v>
       </c>
       <c r="B416" t="str">
-        <v>2nd spot for Extra Challenge C</v>
+        <v>2nd spot for Extra Challenge E</v>
       </c>
       <c r="C416" t="str">
         <v>Exeggcute</v>
       </c>
       <c r="D416" t="str">
-        <v>75-95</v>
+        <v>77-84</v>
       </c>
       <c r="E416" t="str">
         <v>20%</v>
@@ -7478,13 +7478,13 @@
         <v>77</v>
       </c>
       <c r="B417" t="str">
-        <v>2nd spot for Extra Challenge C</v>
+        <v>2nd spot for Extra Challenge E</v>
       </c>
       <c r="C417" t="str">
         <v>Tentacruel</v>
       </c>
       <c r="D417" t="str">
-        <v>75-95</v>
+        <v>77-84</v>
       </c>
       <c r="E417" t="str">
         <v>15%</v>
@@ -7495,13 +7495,13 @@
         <v>77</v>
       </c>
       <c r="B418" t="str">
-        <v>2nd spot for Extra Challenge C</v>
+        <v>2nd spot for Extra Challenge E</v>
       </c>
       <c r="C418" t="str">
         <v>Roserade</v>
       </c>
       <c r="D418" t="str">
-        <v>75-95</v>
+        <v>77-84</v>
       </c>
       <c r="E418" t="str">
         <v>10%</v>
@@ -7518,7 +7518,7 @@
         <v>Barboach</v>
       </c>
       <c r="D419" t="str">
-        <v>75-95</v>
+        <v>84-91</v>
       </c>
       <c r="E419" t="str">
         <v>30%</v>
@@ -7535,7 +7535,7 @@
         <v>Gulpin</v>
       </c>
       <c r="D420" t="str">
-        <v>75-95</v>
+        <v>84-91</v>
       </c>
       <c r="E420" t="str">
         <v>25%</v>
@@ -7552,7 +7552,7 @@
         <v>Pinsir</v>
       </c>
       <c r="D421" t="str">
-        <v>75-95</v>
+        <v>84-91</v>
       </c>
       <c r="E421" t="str">
         <v>20%</v>
@@ -7569,7 +7569,7 @@
         <v>Dragalge</v>
       </c>
       <c r="D422" t="str">
-        <v>75-95</v>
+        <v>84-91</v>
       </c>
       <c r="E422" t="str">
         <v>15%</v>
@@ -7586,7 +7586,7 @@
         <v>Quagsire</v>
       </c>
       <c r="D423" t="str">
-        <v>75-95</v>
+        <v>84-91</v>
       </c>
       <c r="E423" t="str">
         <v>10%</v>
@@ -7603,7 +7603,7 @@
         <v>Hydreigon</v>
       </c>
       <c r="D424" t="str">
-        <v>75-95</v>
+        <v>70-77</v>
       </c>
       <c r="E424" t="str">
         <v>30%</v>
@@ -7620,7 +7620,7 @@
         <v>Sandslash</v>
       </c>
       <c r="D425" t="str">
-        <v>75-95</v>
+        <v>70-77</v>
       </c>
       <c r="E425" t="str">
         <v>25%</v>
@@ -7637,7 +7637,7 @@
         <v>Cubchoo</v>
       </c>
       <c r="D426" t="str">
-        <v>75-95</v>
+        <v>70-77</v>
       </c>
       <c r="E426" t="str">
         <v>20%</v>
@@ -7654,7 +7654,7 @@
         <v>Zigzagoon</v>
       </c>
       <c r="D427" t="str">
-        <v>75-95</v>
+        <v>70-77</v>
       </c>
       <c r="E427" t="str">
         <v>15%</v>
@@ -7671,7 +7671,7 @@
         <v>Bellossom</v>
       </c>
       <c r="D428" t="str">
-        <v>75-95</v>
+        <v>70-77</v>
       </c>
       <c r="E428" t="str">
         <v>10%</v>
@@ -7688,7 +7688,7 @@
         <v>Bergmite</v>
       </c>
       <c r="D429" t="str">
-        <v>75-95</v>
+        <v>77-84</v>
       </c>
       <c r="E429" t="str">
         <v>30%</v>
@@ -7705,7 +7705,7 @@
         <v>Carbink</v>
       </c>
       <c r="D430" t="str">
-        <v>75-95</v>
+        <v>77-84</v>
       </c>
       <c r="E430" t="str">
         <v>25%</v>
@@ -7722,7 +7722,7 @@
         <v>Skitty</v>
       </c>
       <c r="D431" t="str">
-        <v>75-95</v>
+        <v>77-84</v>
       </c>
       <c r="E431" t="str">
         <v>20%</v>
@@ -7739,7 +7739,7 @@
         <v>Golbat</v>
       </c>
       <c r="D432" t="str">
-        <v>75-95</v>
+        <v>77-84</v>
       </c>
       <c r="E432" t="str">
         <v>15%</v>
@@ -7756,7 +7756,7 @@
         <v>Phantump</v>
       </c>
       <c r="D433" t="str">
-        <v>75-95</v>
+        <v>77-84</v>
       </c>
       <c r="E433" t="str">
         <v>10%</v>
@@ -7773,7 +7773,7 @@
         <v>Goomy</v>
       </c>
       <c r="D434" t="str">
-        <v>75-95</v>
+        <v>84-91</v>
       </c>
       <c r="E434" t="str">
         <v>30%</v>
@@ -7790,7 +7790,7 @@
         <v>Carnivine</v>
       </c>
       <c r="D435" t="str">
-        <v>75-95</v>
+        <v>84-91</v>
       </c>
       <c r="E435" t="str">
         <v>25%</v>
@@ -7807,7 +7807,7 @@
         <v>Swellow</v>
       </c>
       <c r="D436" t="str">
-        <v>75-95</v>
+        <v>84-91</v>
       </c>
       <c r="E436" t="str">
         <v>20%</v>
@@ -7824,7 +7824,7 @@
         <v>Magnemite</v>
       </c>
       <c r="D437" t="str">
-        <v>75-95</v>
+        <v>84-91</v>
       </c>
       <c r="E437" t="str">
         <v>15%</v>
@@ -7841,7 +7841,7 @@
         <v>Gastly</v>
       </c>
       <c r="D438" t="str">
-        <v>75-95</v>
+        <v>84-91</v>
       </c>
       <c r="E438" t="str">
         <v>10%</v>
@@ -7960,7 +7960,7 @@
         <v>Dartrix</v>
       </c>
       <c r="D445" t="str">
-        <v>45-50</v>
+        <v>45-51</v>
       </c>
       <c r="E445" t="str">
         <v>16.66%</v>
@@ -7977,7 +7977,7 @@
         <v>Torracat</v>
       </c>
       <c r="D446" t="str">
-        <v>45-50</v>
+        <v>45-51</v>
       </c>
       <c r="E446" t="str">
         <v>16.66%</v>
@@ -7994,7 +7994,7 @@
         <v>Brionne</v>
       </c>
       <c r="D447" t="str">
-        <v>45-50</v>
+        <v>45-51</v>
       </c>
       <c r="E447" t="str">
         <v>16.66%</v>
@@ -8011,7 +8011,7 @@
         <v>Ivysaur</v>
       </c>
       <c r="D448" t="str">
-        <v>45-50</v>
+        <v>45-51</v>
       </c>
       <c r="E448" t="str">
         <v>16.66%</v>
@@ -8028,7 +8028,7 @@
         <v>Charmeleon</v>
       </c>
       <c r="D449" t="str">
-        <v>45-50</v>
+        <v>45-51</v>
       </c>
       <c r="E449" t="str">
         <v>16.66%</v>
@@ -8045,7 +8045,7 @@
         <v>Blastoise</v>
       </c>
       <c r="D450" t="str">
-        <v>45-50</v>
+        <v>45-51</v>
       </c>
       <c r="E450" t="str">
         <v>16.66%</v>
@@ -8230,7 +8230,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C84"/>
+  <dimension ref="A1:C87"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -8482,7 +8482,7 @@
         <v>Defeat the Gym Leader at Cyllage City Gym</v>
       </c>
       <c r="C23" t="str">
-        <v>Unlock Cyllage City (Fishing)</v>
+        <v>Unlock Route 10 AND Unlock Cyllage City (Fishing) (first spot for Extra Challenge A)</v>
       </c>
     </row>
     <row r="24">
@@ -8490,10 +8490,10 @@
         <v>Challenge 23</v>
       </c>
       <c r="B24" t="str">
-        <v>Catch 5 different species in Cyllage City (Fishing)</v>
+        <v>Catch 5 different species in Route 10</v>
       </c>
       <c r="C24" t="str">
-        <v>Unlock Route 10</v>
+        <v>Unlock Geosenge Town</v>
       </c>
     </row>
     <row r="25">
@@ -8501,10 +8501,10 @@
         <v>Challenge 24</v>
       </c>
       <c r="B25" t="str">
-        <v>Defeat 25 Pokemon in Route 10</v>
+        <v>Defeat 25 Pokemon in Geosenge Town</v>
       </c>
       <c r="C25" t="str">
-        <v>Unlock Geosenge Town</v>
+        <v>Unlock Route 11</v>
       </c>
     </row>
     <row r="26">
@@ -8512,10 +8512,10 @@
         <v>Challenge 25</v>
       </c>
       <c r="B26" t="str">
-        <v>Catch 5 different species in Geosenge Town</v>
+        <v>Catch 5 different species in Route 11</v>
       </c>
       <c r="C26" t="str">
-        <v>Unlock Route 11</v>
+        <v>Unlock Shalour City</v>
       </c>
     </row>
     <row r="27">
@@ -8523,10 +8523,10 @@
         <v>Challenge 26</v>
       </c>
       <c r="B27" t="str">
-        <v>Defeat 25 Pokemon in Route 11</v>
+        <v>Defeat 25 Pokemon in Shalour City</v>
       </c>
       <c r="C27" t="str">
-        <v>Unlock Reflection Cave</v>
+        <v>Unlock Shalour City Gym</v>
       </c>
     </row>
     <row r="28">
@@ -8534,10 +8534,10 @@
         <v>Challenge 27</v>
       </c>
       <c r="B28" t="str">
-        <v>Catch 5 different species in Reflection Cave</v>
+        <v>Defeat the Gym Leader at Shalour City Gym</v>
       </c>
       <c r="C28" t="str">
-        <v>Unlock Shalour City</v>
+        <v>Unlock Route 12</v>
       </c>
     </row>
     <row r="29">
@@ -8545,10 +8545,10 @@
         <v>Challenge 28</v>
       </c>
       <c r="B29" t="str">
-        <v>Defeat 25 Pokemon in Shalour City</v>
+        <v>Defeat 25 Pokemon in Route 12</v>
       </c>
       <c r="C29" t="str">
-        <v>Unlock Shalour City Gym</v>
+        <v>Unlock Azure Bay</v>
       </c>
     </row>
     <row r="30">
@@ -8556,10 +8556,10 @@
         <v>Challenge 29</v>
       </c>
       <c r="B30" t="str">
-        <v>Defeat the Gym Leader at Shalour City Gym</v>
+        <v>Catch 5 different species in Azure Bay</v>
       </c>
       <c r="C30" t="str">
-        <v>Unlock Tower of Mastery</v>
+        <v>Unlock Azure Bay (Fishing)</v>
       </c>
     </row>
     <row r="31">
@@ -8567,10 +8567,10 @@
         <v>Challenge 30</v>
       </c>
       <c r="B31" t="str">
-        <v>Defeat 25 Pokemon in Tower of Mastery</v>
+        <v>Defeat 25 Pokemon in Azure Bay (Fishing)</v>
       </c>
       <c r="C31" t="str">
-        <v>Unlock Route 12</v>
+        <v>Unlock Coumarine City Gym</v>
       </c>
     </row>
     <row r="32">
@@ -8578,10 +8578,10 @@
         <v>Challenge 31</v>
       </c>
       <c r="B32" t="str">
-        <v>Catch 5 different species in Route 12</v>
+        <v>Defeat the Gym Leader at Coumarine City Gym</v>
       </c>
       <c r="C32" t="str">
-        <v>Unlock Azure Bay</v>
+        <v>Unlock Coumarine City (Fishing) AND Unlock Starter Depot (first spot for Extra Challenge B)</v>
       </c>
     </row>
     <row r="33">
@@ -8589,10 +8589,10 @@
         <v>Challenge 32</v>
       </c>
       <c r="B33" t="str">
-        <v>Defeat 25 Pokemon in Azure Bay</v>
+        <v>Defeat 25 Pokemon in Coumarine City (Fishing)</v>
       </c>
       <c r="C33" t="str">
-        <v>Unlock Azure Bay (Fishing)</v>
+        <v>Unlock Route 13</v>
       </c>
     </row>
     <row r="34">
@@ -8600,10 +8600,10 @@
         <v>Challenge 33</v>
       </c>
       <c r="B34" t="str">
-        <v>Catch 5 different species in Azure Bay (Fishing)</v>
+        <v>Catch 5 different species in Route 13</v>
       </c>
       <c r="C34" t="str">
-        <v>Unlock Coumarine City</v>
+        <v>Unlock Lumiose City (North)</v>
       </c>
     </row>
     <row r="35">
@@ -8611,10 +8611,10 @@
         <v>Challenge 34</v>
       </c>
       <c r="B35" t="str">
-        <v>Defeat 25 Pokemon in Coumarine City</v>
+        <v>Defeat 25 Pokemon in Lumiose City (North)</v>
       </c>
       <c r="C35" t="str">
-        <v>Unlock Coumarine City Gym</v>
+        <v>Unlock Lumiose City Gym</v>
       </c>
     </row>
     <row r="36">
@@ -8622,10 +8622,10 @@
         <v>Challenge 35</v>
       </c>
       <c r="B36" t="str">
-        <v>Defeat the Gym Leader at Coumarine City Gym</v>
+        <v>Defeat the Gym Leader at Lumiose City Gym</v>
       </c>
       <c r="C36" t="str">
-        <v>Unlock Coumarine City (Fishing) AND Unlock Starter Depot</v>
+        <v>Unlock Route 14</v>
       </c>
     </row>
     <row r="37">
@@ -8633,10 +8633,10 @@
         <v>Challenge 36</v>
       </c>
       <c r="B37" t="str">
-        <v>Defeat 25 Pokemon in Coumarine City (Fishing)</v>
+        <v>Defeat 25 Pokemon in Route 14</v>
       </c>
       <c r="C37" t="str">
-        <v>Unlock Route 13</v>
+        <v>Unlock Laverre City</v>
       </c>
     </row>
     <row r="38">
@@ -8644,10 +8644,10 @@
         <v>Challenge 37</v>
       </c>
       <c r="B38" t="str">
-        <v>Catch 5 different species in Route 13</v>
+        <v>Catch 5 different species in Laverre City</v>
       </c>
       <c r="C38" t="str">
-        <v>Unlock Lumiose City (North)</v>
+        <v>Unlock Laverre City Gym</v>
       </c>
     </row>
     <row r="39">
@@ -8655,10 +8655,10 @@
         <v>Challenge 38</v>
       </c>
       <c r="B39" t="str">
-        <v>Defeat 25 Pokemon in Lumiose City (North)</v>
+        <v>Defeat the Gym Leader at Laverre City Gym</v>
       </c>
       <c r="C39" t="str">
-        <v>Unlock Lumiose City Gym</v>
+        <v>Unlock Route 15</v>
       </c>
     </row>
     <row r="40">
@@ -8666,10 +8666,10 @@
         <v>Challenge 39</v>
       </c>
       <c r="B40" t="str">
-        <v>Defeat the Gym Leader at Lumiose City Gym</v>
+        <v>Catch 5 different species in Route 15</v>
       </c>
       <c r="C40" t="str">
-        <v>Unlock Route 14</v>
+        <v>Unlock Lost Hotel</v>
       </c>
     </row>
     <row r="41">
@@ -8677,10 +8677,10 @@
         <v>Challenge 40</v>
       </c>
       <c r="B41" t="str">
-        <v>Defeat 25 Pokemon in Route 14</v>
+        <v>Defeat 25 Pokemon in Lost Hotel</v>
       </c>
       <c r="C41" t="str">
-        <v>Unlock Laverre City</v>
+        <v>Unlock Dendemille Town</v>
       </c>
     </row>
     <row r="42">
@@ -8688,10 +8688,10 @@
         <v>Challenge 41</v>
       </c>
       <c r="B42" t="str">
-        <v>Catch 5 different species in Laverre City</v>
+        <v>Catch 5 different species in Dendemille Town</v>
       </c>
       <c r="C42" t="str">
-        <v>Unlock Laverre City Gym</v>
+        <v>Unlock Route 16</v>
       </c>
     </row>
     <row r="43">
@@ -8699,10 +8699,10 @@
         <v>Challenge 42</v>
       </c>
       <c r="B43" t="str">
-        <v>Defeat the Gym Leader at Laverre City Gym</v>
+        <v>Defeat 25 Pokemon in Route 16</v>
       </c>
       <c r="C43" t="str">
-        <v>Unlock Route 15</v>
+        <v>Unlock Frost Cavern</v>
       </c>
     </row>
     <row r="44">
@@ -8710,10 +8710,10 @@
         <v>Challenge 43</v>
       </c>
       <c r="B44" t="str">
-        <v>Catch 5 different species in Route 15</v>
+        <v>Catch 5 different species in Frost Cavern</v>
       </c>
       <c r="C44" t="str">
-        <v>Unlock Lost Hotel</v>
+        <v>Unlock Anistar City</v>
       </c>
     </row>
     <row r="45">
@@ -8721,10 +8721,10 @@
         <v>Challenge 44</v>
       </c>
       <c r="B45" t="str">
-        <v>Defeat 25 Pokemon in Lost Hotel</v>
+        <v>Defeat 25 Pokemon in Anistar City</v>
       </c>
       <c r="C45" t="str">
-        <v>Unlock Dendemille Town</v>
+        <v>Unlock Anistar City Gym</v>
       </c>
     </row>
     <row r="46">
@@ -8732,10 +8732,10 @@
         <v>Challenge 45</v>
       </c>
       <c r="B46" t="str">
-        <v>Catch 5 different species in Dendemille Town</v>
+        <v>Defeat the Gym Leader at Anistar City Gym</v>
       </c>
       <c r="C46" t="str">
-        <v>Unlock Route 16</v>
+        <v>Unlock Route 17</v>
       </c>
     </row>
     <row r="47">
@@ -8743,10 +8743,10 @@
         <v>Challenge 46</v>
       </c>
       <c r="B47" t="str">
-        <v>Defeat 25 Pokemon in Route 16</v>
+        <v>Defeat 25 Pokemon in Route 17</v>
       </c>
       <c r="C47" t="str">
-        <v>Unlock Frost Cavern</v>
+        <v>Unlock Couriway Town</v>
       </c>
     </row>
     <row r="48">
@@ -8754,10 +8754,10 @@
         <v>Challenge 47</v>
       </c>
       <c r="B48" t="str">
-        <v>Catch 5 different species in Frost Cavern</v>
+        <v>Catch 5 different species in Couriway Town</v>
       </c>
       <c r="C48" t="str">
-        <v>Unlock Anistar City</v>
+        <v>Unlock Route 18</v>
       </c>
     </row>
     <row r="49">
@@ -8765,10 +8765,10 @@
         <v>Challenge 48</v>
       </c>
       <c r="B49" t="str">
-        <v>Defeat 25 Pokemon in Anistar City</v>
+        <v>Defeat 25 Pokemon in Route 18</v>
       </c>
       <c r="C49" t="str">
-        <v>Unlock Anistar City Gym</v>
+        <v>Unlock Terminus Cave (Surface)</v>
       </c>
     </row>
     <row r="50">
@@ -8776,10 +8776,10 @@
         <v>Challenge 49</v>
       </c>
       <c r="B50" t="str">
-        <v>Defeat the Gym Leader at Anistar City Gym</v>
+        <v>Catch 5 different species in Terminus Cave (Surface)</v>
       </c>
       <c r="C50" t="str">
-        <v>Unlock Route 17</v>
+        <v>Unlock Route 19</v>
       </c>
     </row>
     <row r="51">
@@ -8787,10 +8787,10 @@
         <v>Challenge 50</v>
       </c>
       <c r="B51" t="str">
-        <v>Defeat 25 Pokemon in Route 17</v>
+        <v>Defeat 25 Pokemon in Route 19</v>
       </c>
       <c r="C51" t="str">
-        <v>Unlock Couriway Town</v>
+        <v>Unlock Route 19 (Fishing)</v>
       </c>
     </row>
     <row r="52">
@@ -8798,10 +8798,10 @@
         <v>Challenge 51</v>
       </c>
       <c r="B52" t="str">
-        <v>Catch 5 different species in Couriway Town</v>
+        <v>Catch 5 different species in Route 19 (Fishing)</v>
       </c>
       <c r="C52" t="str">
-        <v>Unlock Route 18</v>
+        <v>Unlock Snowbelle City</v>
       </c>
     </row>
     <row r="53">
@@ -8809,10 +8809,10 @@
         <v>Challenge 52</v>
       </c>
       <c r="B53" t="str">
-        <v>Defeat 25 Pokemon in Route 18</v>
+        <v>Defeat 25 Pokemon in Snowbelle City</v>
       </c>
       <c r="C53" t="str">
-        <v>Unlock Terminus Cave (Surface)</v>
+        <v>Unlock Snowbelle City Gym</v>
       </c>
     </row>
     <row r="54">
@@ -8820,10 +8820,10 @@
         <v>Challenge 53</v>
       </c>
       <c r="B54" t="str">
-        <v>Catch 5 different species in Terminus Cave (Surface)</v>
+        <v>Defeat the Gym Leader at Snowbelle City Gym</v>
       </c>
       <c r="C54" t="str">
-        <v>Unlock Route 19</v>
+        <v>Unlock Route 20</v>
       </c>
     </row>
     <row r="55">
@@ -8831,10 +8831,10 @@
         <v>Challenge 54</v>
       </c>
       <c r="B55" t="str">
-        <v>Defeat 25 Pokemon in Route 19</v>
+        <v>Defeat 25 Pokemon in Route 20</v>
       </c>
       <c r="C55" t="str">
-        <v>Unlock Route 19 (Fishing)</v>
+        <v>Unlock Pokémon Village</v>
       </c>
     </row>
     <row r="56">
@@ -8842,10 +8842,10 @@
         <v>Challenge 55</v>
       </c>
       <c r="B56" t="str">
-        <v>Catch 5 different species in Route 19 (Fishing)</v>
+        <v>Catch 5 different species in Pokémon Village</v>
       </c>
       <c r="C56" t="str">
-        <v>Unlock Snowbelle City</v>
+        <v>Unlock Pokémon Village (Fishing)</v>
       </c>
     </row>
     <row r="57">
@@ -8853,10 +8853,10 @@
         <v>Challenge 56</v>
       </c>
       <c r="B57" t="str">
-        <v>Defeat 25 Pokemon in Snowbelle City</v>
+        <v>Defeat 25 Pokemon in Pokémon Village (Fishing)</v>
       </c>
       <c r="C57" t="str">
-        <v>Unlock Snowbelle City Gym</v>
+        <v>Unlock Route 21</v>
       </c>
     </row>
     <row r="58">
@@ -8864,10 +8864,10 @@
         <v>Challenge 57</v>
       </c>
       <c r="B58" t="str">
-        <v>Defeat the Gym Leader at Snowbelle City Gym</v>
+        <v>Catch 5 different species in Route 21</v>
       </c>
       <c r="C58" t="str">
-        <v>Unlock Route 20</v>
+        <v>Unlock Victory Road</v>
       </c>
     </row>
     <row r="59">
@@ -8875,10 +8875,10 @@
         <v>Challenge 58</v>
       </c>
       <c r="B59" t="str">
-        <v>Defeat 25 Pokemon in Route 20</v>
+        <v>Defeat 25 Pokemon in Victory Road</v>
       </c>
       <c r="C59" t="str">
-        <v>Unlock Pokémon Village</v>
+        <v>Unlock Kalos Pokemon League</v>
       </c>
     </row>
     <row r="60">
@@ -8886,10 +8886,10 @@
         <v>Challenge 59</v>
       </c>
       <c r="B60" t="str">
-        <v>Catch 5 different species in Pokémon Village</v>
+        <v>Catch 5 different species in Kalos Pokemon League</v>
       </c>
       <c r="C60" t="str">
-        <v>Unlock Pokémon Village (Fishing)</v>
+        <v>Unlock Mystic Tower Entrance</v>
       </c>
     </row>
     <row r="61">
@@ -8897,10 +8897,10 @@
         <v>Challenge 60</v>
       </c>
       <c r="B61" t="str">
-        <v>Defeat 25 Pokemon in Pokémon Village (Fishing)</v>
+        <v>Defeat 25 Pokemon in Mystic Tower Entrance</v>
       </c>
       <c r="C61" t="str">
-        <v>Unlock Route 21</v>
+        <v>Unlock Crystal Cave Tunnels</v>
       </c>
     </row>
     <row r="62">
@@ -8908,21 +8908,21 @@
         <v>Challenge 61</v>
       </c>
       <c r="B62" t="str">
-        <v>Catch 5 different species in Route 21</v>
+        <v>Catch 5 different species in Crystal Cave Tunnels</v>
       </c>
       <c r="C62" t="str">
-        <v>Unlock Victory Road</v>
+        <v>Unlock Secret Forest North</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>Challenge 62</v>
+        <v>Final Challenge</v>
       </c>
       <c r="B63" t="str">
-        <v>Defeat 25 Pokemon in Victory Road</v>
+        <v>Defeat the Kalos Champion at Kalos Pokemon League</v>
       </c>
       <c r="C63" t="str">
-        <v>Unlock Kalos Pokemon League</v>
+        <v>Unlock Path to Sea Spirit Den (first spot for Extra Challenge C), Path to Team Flare Secret HQ (first spot for Extra Challenge E), Path to Secret Ruins (first spot for Extra Challenge D)</v>
       </c>
     </row>
     <row r="64">
@@ -8930,10 +8930,10 @@
         <v>Extra Challenge A 1</v>
       </c>
       <c r="B64" t="str">
-        <v>Capture 1 Rowlet and 1 Litten and 1 Popplio</v>
+        <v>Complete objectives in Cyllage City (Fishing)</v>
       </c>
       <c r="C64" t="str">
-        <v>Unlock Starter Evolved Depot</v>
+        <v>Unlock Reflection Cave</v>
       </c>
     </row>
     <row r="65">
@@ -8941,10 +8941,10 @@
         <v>Extra Challenge A 2</v>
       </c>
       <c r="B65" t="str">
-        <v>Capture 1 Dartrix and 1 Torracat and 1 Brionne</v>
+        <v>Complete objectives in Reflection Cave</v>
       </c>
       <c r="C65" t="str">
-        <v>Unlock Kiloude City</v>
+        <v>Unlock Tower of Mastery</v>
       </c>
     </row>
     <row r="66">
@@ -8952,10 +8952,10 @@
         <v>Extra Challenge A 3</v>
       </c>
       <c r="B66" t="str">
-        <v>Complete objectives in Kiloude City</v>
+        <v>Complete objectives in Tower of Mastery</v>
       </c>
       <c r="C66" t="str">
-        <v>Unlock Friend Safari</v>
+        <v>Unlock Coumarine City</v>
       </c>
     </row>
     <row r="67">
@@ -8963,202 +8963,235 @@
         <v>Extra Challenge A 4</v>
       </c>
       <c r="B67" t="str">
-        <v>Complete objectives in Friend Safari</v>
+        <v>Complete objectives in Coumarine City</v>
       </c>
       <c r="C67" t="str">
-        <v>Unlock Battle Maison</v>
+        <v>Earn 1 Masterball</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>Extra Challenge A 5</v>
+        <v>Extra Challenge B 1</v>
       </c>
       <c r="B68" t="str">
-        <v>Complete objectives in Battle Maison</v>
+        <v>Capture 1 Rowlet and 1 Litten and 1 Popplio and 1 Bulbasaur and 1 Charmander and 1 Squirtle</v>
       </c>
       <c r="C68" t="str">
-        <v>Earn 1 Masterball</v>
+        <v>Unlock Starter Evolved Depot</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>Final Challenge</v>
+        <v>Extra Challenge B 2</v>
       </c>
       <c r="B69" t="str">
-        <v>Defeat the Kalos Champion at Kalos Pokemon League</v>
+        <v>Capture 1 Dartrix and 1 Torracat and 1 Brionne and 1 Ivysaur and 1 Charmeleon and 1 Blastoise</v>
       </c>
       <c r="C69" t="str">
-        <v>Unlock Path to Sea Spirit Den (first spot for Extra Challenge B), Path to Team Flare Secret HQ (first spot for Extra Challenge C), Path to Secret Ruins (first spot for Extra Challenge D)</v>
+        <v>Unlock Kiloude City</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>Extra Challenge B 1</v>
+        <v>Extra Challenge B 3</v>
       </c>
       <c r="B70" t="str">
-        <v>Complete objectives on Path to Sea Spirit Den</v>
+        <v>Complete objectives in Kiloude City</v>
       </c>
       <c r="C70" t="str">
-        <v>Unlock 2nd spot for Extra Challenge B</v>
+        <v>Unlock Friend Safari</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>Extra Challenge B 2</v>
+        <v>Extra Challenge B 4</v>
       </c>
       <c r="B71" t="str">
-        <v>Complete objectives on 2nd spot for Extra Challenge B</v>
+        <v>Complete objectives in Friend Safari</v>
       </c>
       <c r="C71" t="str">
-        <v>Unlock Sea Spirit Den Entrance</v>
+        <v>Unlock Battle Maison</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>Extra Challenge B 3</v>
+        <v>Extra Challenge B 5</v>
       </c>
       <c r="B72" t="str">
-        <v>Complete objectives in Sea Spirit Den Entrance</v>
+        <v>Complete objectives in Battle Maison</v>
       </c>
       <c r="C72" t="str">
-        <v>Unlock Sea Spirit Den Tunnels</v>
+        <v>Earn 1 Masterball</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>Extra Challenge B 4</v>
+        <v>Extra Challenge C 1</v>
       </c>
       <c r="B73" t="str">
-        <v>Complete objectives in Sea Spirit Den Tunnels</v>
+        <v>Complete objectives on Path to Sea Spirit Den</v>
       </c>
       <c r="C73" t="str">
-        <v>Unlock Sea Spirit Den Hall</v>
+        <v>Unlock Sea Spirit Den Outer Depths</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>Extra Challenge B 5</v>
+        <v>Extra Challenge C 2</v>
       </c>
       <c r="B74" t="str">
-        <v>Capture 1 Articuno 1 Zapdos 1 Moltres</v>
+        <v>Complete objectives in Sea Spirit Den Outer Depths</v>
       </c>
       <c r="C74" t="str">
-        <v>Earn 2 Masterball</v>
+        <v>Unlock Sea Spirit Den Entrance</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>Extra Challenge C 1</v>
+        <v>Extra Challenge C 3</v>
       </c>
       <c r="B75" t="str">
-        <v>Complete objectives on Path to Team Flare Secret HQ</v>
+        <v>Complete objectives in Sea Spirit Den Entrance</v>
       </c>
       <c r="C75" t="str">
-        <v>Unlock 2nd spot for Extra Challenge C</v>
+        <v>Unlock Sea Spirit Den Tunnels</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>Extra Challenge C 2</v>
+        <v>Extra Challenge C 4</v>
       </c>
       <c r="B76" t="str">
-        <v>Complete objectives on 2nd spot for Extra Challenge C</v>
+        <v>Complete objectives in Sea Spirit Den Tunnels</v>
       </c>
       <c r="C76" t="str">
-        <v>Unlock Team Flare Secret HQ Gate</v>
+        <v>Unlock Sea Spirit Den Hall</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>Extra Challenge C 3</v>
+        <v>Extra Challenge C 5</v>
       </c>
       <c r="B77" t="str">
-        <v>Complete objectives in Team Flare Secret HQ Gate</v>
+        <v>Capture 1 Articuno 1 Zapdos 1 Moltres</v>
       </c>
       <c r="C77" t="str">
-        <v>Unlock Team Flare Secret HQ Entrance</v>
+        <v>Earn 2 Masterball</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v>Extra Challenge C 4</v>
+        <v>Extra Challenge D 1</v>
       </c>
       <c r="B78" t="str">
-        <v>Complete objectives in Team Flare Secret HQ Entrance</v>
+        <v>Complete objectives on Path to Secret Ruins</v>
       </c>
       <c r="C78" t="str">
-        <v>Unlock Team Flare Secret HQ Hall</v>
+        <v>Unlock Underground Chambers (Crystal Cave Tunnels)</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="str">
-        <v>Extra Challenge C 5</v>
+        <v>Extra Challenge D 2</v>
       </c>
       <c r="B79" t="str">
-        <v>Capture 1 Ybeltal 1 Zygarde 1 Xerneas</v>
+        <v>Complete objectives in Underground Chambers</v>
       </c>
       <c r="C79" t="str">
-        <v>Earn 2 Masterball</v>
+        <v>Unlock Garden Chambers (Secret Forest North)</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="str">
-        <v>Extra Challenge D 1</v>
+        <v>Extra Challenge D 3</v>
       </c>
       <c r="B80" t="str">
-        <v>Complete objectives on Path to Secret Ruins</v>
+        <v>Complete objectives in Garden Chambers</v>
       </c>
       <c r="C80" t="str">
-        <v>Unlock Underground Chambers (Crystal Cave Tunnels)</v>
+        <v>Unlock Chambers of Emptiness</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>Extra Challenge D 2</v>
+        <v>Extra Challenge D 4</v>
       </c>
       <c r="B81" t="str">
-        <v>Complete objectives in Underground Chambers</v>
+        <v>Complete objectives in Chambers of Emptiness</v>
       </c>
       <c r="C81" t="str">
-        <v>Unlock Garden Chambers (Secret Forest North)</v>
+        <v>Unlock Ultimate Chamber</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="str">
-        <v>Extra Challenge D 3</v>
+        <v>Extra Challenge D 5</v>
       </c>
       <c r="B82" t="str">
-        <v>Complete objectives in Garden Chambers</v>
+        <v>Capture 1 Volcanion 1 Diance 1 Hoopa 1 Mewtwo</v>
       </c>
       <c r="C82" t="str">
-        <v>Unlock Chambers of Emptiness</v>
+        <v>Earn 2 Masterball</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="str">
-        <v>Extra Challenge D 4</v>
+        <v>Extra Challenge E 1</v>
       </c>
       <c r="B83" t="str">
-        <v>Complete objectives in Chambers of Emptiness</v>
+        <v>Complete objectives on Path to Team Flare Secret HQ</v>
       </c>
       <c r="C83" t="str">
-        <v>Unlock Ultimate Chamber</v>
+        <v>Unlock 2nd spot for Extra Challenge E</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="str">
-        <v>Extra Challenge D 5</v>
+        <v>Extra Challenge E 2</v>
       </c>
       <c r="B84" t="str">
-        <v>Capture 1 Volcanion 1 Diance 1 Hoopa 1 Mewtwo</v>
+        <v>Complete objectives on 2nd spot for Extra Challenge E</v>
       </c>
       <c r="C84" t="str">
+        <v>Unlock Team Flare Secret HQ Gate</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="str">
+        <v>Extra Challenge E 3</v>
+      </c>
+      <c r="B85" t="str">
+        <v>Complete objectives in Team Flare Secret HQ Gate</v>
+      </c>
+      <c r="C85" t="str">
+        <v>Unlock Team Flare Secret HQ Entrance</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="str">
+        <v>Extra Challenge E 4</v>
+      </c>
+      <c r="B86" t="str">
+        <v>Complete objectives in Team Flare Secret HQ Entrance</v>
+      </c>
+      <c r="C86" t="str">
+        <v>Unlock Team Flare Secret HQ Hall</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="str">
+        <v>Extra Challenge E 5</v>
+      </c>
+      <c r="B87" t="str">
+        <v>Capture 1 Ybeltal 1 Zygarde 1 Xerneas</v>
+      </c>
+      <c r="C87" t="str">
         <v>Earn 2 Masterball</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C84"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C87"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Format Kalos challenges to utilize explicit engine criteria strings
Co-authored-by: lsampaio1337-beep <246645260+lsampaio1337-beep@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Kalos_Path.xlsx
+++ b/Kalos_Path.xlsx
@@ -8248,7 +8248,7 @@
         <v>Challenge 1</v>
       </c>
       <c r="B2" t="str">
-        <v>Catch 5 different species in Aquacorde Town</v>
+        <v>catchSpeciesAnyOf: { route: 'Aquacorde Town', count: 5 }</v>
       </c>
       <c r="C2" t="str">
         <v>Unlock Route 2</v>
@@ -8259,7 +8259,7 @@
         <v>Challenge 2</v>
       </c>
       <c r="B3" t="str">
-        <v>Defeat 25 Pokemon in Route 2</v>
+        <v>defeatCountRoute: { route: 'Route 2', count: 25 }</v>
       </c>
       <c r="C3" t="str">
         <v>Unlock Santalune Forest</v>
@@ -8270,7 +8270,7 @@
         <v>Challenge 3</v>
       </c>
       <c r="B4" t="str">
-        <v>Catch 5 different species in Santalune Forest</v>
+        <v>catchSpeciesAnyOf: { route: 'Santalune Forest', count: 5 }</v>
       </c>
       <c r="C4" t="str">
         <v>Unlock Route 3</v>
@@ -8281,7 +8281,7 @@
         <v>Challenge 4</v>
       </c>
       <c r="B5" t="str">
-        <v>Defeat 25 Pokemon in Route 3</v>
+        <v>defeatCountRoute: { route: 'Route 3', count: 25 }</v>
       </c>
       <c r="C5" t="str">
         <v>Unlock Santalune City</v>
@@ -8292,7 +8292,7 @@
         <v>Challenge 5</v>
       </c>
       <c r="B6" t="str">
-        <v>Catch 5 different species in Santalune City</v>
+        <v>catchSpeciesAnyOf: { route: 'Santalune City', count: 5 }</v>
       </c>
       <c r="C6" t="str">
         <v>Unlock Santalune City Gym</v>
@@ -8303,7 +8303,7 @@
         <v>Challenge 6</v>
       </c>
       <c r="B7" t="str">
-        <v>Defeat the Gym Leader at Santalune City Gym</v>
+        <v>earnBadge: { badge: 'Bug Badge', leader: 'Viola' }</v>
       </c>
       <c r="C7" t="str">
         <v>Unlock Route 22</v>
@@ -8314,7 +8314,7 @@
         <v>Challenge 7</v>
       </c>
       <c r="B8" t="str">
-        <v>Catch 5 different species in Route 22</v>
+        <v>catchSpeciesAnyOf: { route: 'Route 22', count: 5 }</v>
       </c>
       <c r="C8" t="str">
         <v>Unlock Route 4</v>
@@ -8325,7 +8325,7 @@
         <v>Challenge 8</v>
       </c>
       <c r="B9" t="str">
-        <v>Defeat 25 Pokemon in Route 4</v>
+        <v>defeatCountRoute: { route: 'Route 4', count: 25 }</v>
       </c>
       <c r="C9" t="str">
         <v>Unlock Lumiose City (South)</v>
@@ -8336,7 +8336,7 @@
         <v>Challenge 9</v>
       </c>
       <c r="B10" t="str">
-        <v>Catch 5 different species in Lumiose City (South)</v>
+        <v>catchSpeciesAnyOf: { route: 'Lumiose City (South)', count: 5 }</v>
       </c>
       <c r="C10" t="str">
         <v>Unlock Route 5</v>
@@ -8347,7 +8347,7 @@
         <v>Challenge 10</v>
       </c>
       <c r="B11" t="str">
-        <v>Defeat 25 Pokemon in Route 5</v>
+        <v>defeatCountRoute: { route: 'Route 5', count: 25 }</v>
       </c>
       <c r="C11" t="str">
         <v>Unlock Camphrier Town</v>
@@ -8358,7 +8358,7 @@
         <v>Challenge 11</v>
       </c>
       <c r="B12" t="str">
-        <v>Catch 5 different species in Camphrier Town</v>
+        <v>catchSpeciesAnyOf: { route: 'Camphrier Town', count: 5 }</v>
       </c>
       <c r="C12" t="str">
         <v>Unlock Parfum Palace</v>
@@ -8369,7 +8369,7 @@
         <v>Challenge 12</v>
       </c>
       <c r="B13" t="str">
-        <v>Defeat 25 Pokemon in Parfum Palace</v>
+        <v>defeatCountRoute: { route: 'Parfum Palace', count: 50 }</v>
       </c>
       <c r="C13" t="str">
         <v>Unlock Route 6</v>
@@ -8380,7 +8380,7 @@
         <v>Challenge 13</v>
       </c>
       <c r="B14" t="str">
-        <v>Catch 5 different species in Route 6</v>
+        <v>catchSpeciesAnyOf: { route: 'Route 6', count: 5 }</v>
       </c>
       <c r="C14" t="str">
         <v>Unlock Route 7</v>
@@ -8391,7 +8391,7 @@
         <v>Challenge 14</v>
       </c>
       <c r="B15" t="str">
-        <v>Defeat 25 Pokemon in Route 7</v>
+        <v>defeatCountRoute: { route: 'Route 7', count: 50 }</v>
       </c>
       <c r="C15" t="str">
         <v>Unlock Connecting Cave</v>
@@ -8402,7 +8402,7 @@
         <v>Challenge 15</v>
       </c>
       <c r="B16" t="str">
-        <v>Catch 5 different species in Connecting Cave</v>
+        <v>catchSpeciesAnyOf: { route: 'Connecting Cave', count: 5 }</v>
       </c>
       <c r="C16" t="str">
         <v>Unlock Ambrette Town</v>
@@ -8413,7 +8413,7 @@
         <v>Challenge 16</v>
       </c>
       <c r="B17" t="str">
-        <v>Defeat 25 Pokemon in Ambrette Town</v>
+        <v>defeatCountRoute: { route: 'Ambrette Town', count: 50 }</v>
       </c>
       <c r="C17" t="str">
         <v>Unlock Ambrette Town (Fishing)</v>
@@ -8424,7 +8424,7 @@
         <v>Challenge 17</v>
       </c>
       <c r="B18" t="str">
-        <v>Catch 5 different species in Ambrette Town (Fishing)</v>
+        <v>catchSpeciesAnyOf: { route: 'Ambrette Town (Fishing)', count: 5 }</v>
       </c>
       <c r="C18" t="str">
         <v>Unlock Route 8</v>
@@ -8435,7 +8435,7 @@
         <v>Challenge 18</v>
       </c>
       <c r="B19" t="str">
-        <v>Defeat 25 Pokemon in Route 8</v>
+        <v>defeatCountRoute: { route: 'Route 8', count: 50 }</v>
       </c>
       <c r="C19" t="str">
         <v>Unlock Route 9</v>
@@ -8446,7 +8446,7 @@
         <v>Challenge 19</v>
       </c>
       <c r="B20" t="str">
-        <v>Catch 5 different species in Route 9</v>
+        <v>catchSpeciesAnyOf: { route: 'Route 9', count: 5 }</v>
       </c>
       <c r="C20" t="str">
         <v>Unlock Glittering Cave</v>
@@ -8457,7 +8457,7 @@
         <v>Challenge 20</v>
       </c>
       <c r="B21" t="str">
-        <v>Defeat 25 Pokemon in Glittering Cave</v>
+        <v>defeatCountRoute: { route: 'Glittering Cave', count: 50 }</v>
       </c>
       <c r="C21" t="str">
         <v>Unlock Cyllage City</v>
@@ -8468,7 +8468,7 @@
         <v>Challenge 21</v>
       </c>
       <c r="B22" t="str">
-        <v>Catch 5 different species in Cyllage City</v>
+        <v>catchSpeciesAnyOf: { route: 'Cyllage City', count: 5 }</v>
       </c>
       <c r="C22" t="str">
         <v>Unlock Cyllage City Gym</v>
@@ -8479,7 +8479,7 @@
         <v>Challenge 22</v>
       </c>
       <c r="B23" t="str">
-        <v>Defeat the Gym Leader at Cyllage City Gym</v>
+        <v>earnBadge: { badge: 'Cliff Badge', leader: 'Grant' }</v>
       </c>
       <c r="C23" t="str">
         <v>Unlock Route 10 AND Unlock Cyllage City (Fishing) (first spot for Extra Challenge A)</v>
@@ -8490,7 +8490,7 @@
         <v>Challenge 23</v>
       </c>
       <c r="B24" t="str">
-        <v>Catch 5 different species in Route 10</v>
+        <v>catchSpeciesAnyOf: { route: 'Route 10', count: 5 }</v>
       </c>
       <c r="C24" t="str">
         <v>Unlock Geosenge Town</v>
@@ -8501,7 +8501,7 @@
         <v>Challenge 24</v>
       </c>
       <c r="B25" t="str">
-        <v>Defeat 25 Pokemon in Geosenge Town</v>
+        <v>defeatCountRoute: { route: 'Geosenge Town', count: 100 }</v>
       </c>
       <c r="C25" t="str">
         <v>Unlock Route 11</v>
@@ -8512,7 +8512,7 @@
         <v>Challenge 25</v>
       </c>
       <c r="B26" t="str">
-        <v>Catch 5 different species in Route 11</v>
+        <v>catchSpeciesAnyOf: { route: 'Route 11', count: 5 }</v>
       </c>
       <c r="C26" t="str">
         <v>Unlock Shalour City</v>
@@ -8523,7 +8523,7 @@
         <v>Challenge 26</v>
       </c>
       <c r="B27" t="str">
-        <v>Defeat 25 Pokemon in Shalour City</v>
+        <v>defeatCountRoute: { route: 'Shalour City', count: 100 }</v>
       </c>
       <c r="C27" t="str">
         <v>Unlock Shalour City Gym</v>
@@ -8534,7 +8534,7 @@
         <v>Challenge 27</v>
       </c>
       <c r="B28" t="str">
-        <v>Defeat the Gym Leader at Shalour City Gym</v>
+        <v>earnBadge: { badge: 'Rumble Badge', leader: 'Korrina' }</v>
       </c>
       <c r="C28" t="str">
         <v>Unlock Route 12</v>
@@ -8545,7 +8545,7 @@
         <v>Challenge 28</v>
       </c>
       <c r="B29" t="str">
-        <v>Defeat 25 Pokemon in Route 12</v>
+        <v>defeatCountRoute: { route: 'Route 12', count: 100 }</v>
       </c>
       <c r="C29" t="str">
         <v>Unlock Azure Bay</v>
@@ -8556,7 +8556,7 @@
         <v>Challenge 29</v>
       </c>
       <c r="B30" t="str">
-        <v>Catch 5 different species in Azure Bay</v>
+        <v>catchSpeciesAnyOf: { route: 'Azure Bay', count: 5 }</v>
       </c>
       <c r="C30" t="str">
         <v>Unlock Azure Bay (Fishing)</v>
@@ -8567,7 +8567,7 @@
         <v>Challenge 30</v>
       </c>
       <c r="B31" t="str">
-        <v>Defeat 25 Pokemon in Azure Bay (Fishing)</v>
+        <v>defeatCountRoute: { route: 'Azure Bay (Fishing)', count: 100 }</v>
       </c>
       <c r="C31" t="str">
         <v>Unlock Coumarine City Gym</v>
@@ -8578,7 +8578,7 @@
         <v>Challenge 31</v>
       </c>
       <c r="B32" t="str">
-        <v>Defeat the Gym Leader at Coumarine City Gym</v>
+        <v>earnBadge: { badge: 'Plant Badge', leader: 'Ramos' }</v>
       </c>
       <c r="C32" t="str">
         <v>Unlock Coumarine City (Fishing) AND Unlock Starter Depot (first spot for Extra Challenge B)</v>
@@ -8589,7 +8589,7 @@
         <v>Challenge 32</v>
       </c>
       <c r="B33" t="str">
-        <v>Defeat 25 Pokemon in Coumarine City (Fishing)</v>
+        <v>defeatCountRoute: { route: 'Coumarine City (Fishing)', count: 200 }</v>
       </c>
       <c r="C33" t="str">
         <v>Unlock Route 13</v>
@@ -8600,7 +8600,7 @@
         <v>Challenge 33</v>
       </c>
       <c r="B34" t="str">
-        <v>Catch 5 different species in Route 13</v>
+        <v>catchSpeciesAnyOf: { route: 'Route 13', count: 5 }</v>
       </c>
       <c r="C34" t="str">
         <v>Unlock Lumiose City (North)</v>
@@ -8611,7 +8611,7 @@
         <v>Challenge 34</v>
       </c>
       <c r="B35" t="str">
-        <v>Defeat 25 Pokemon in Lumiose City (North)</v>
+        <v>defeatCountRoute: { route: 'Lumiose City (North)', count: 200 }</v>
       </c>
       <c r="C35" t="str">
         <v>Unlock Lumiose City Gym</v>
@@ -8622,7 +8622,7 @@
         <v>Challenge 35</v>
       </c>
       <c r="B36" t="str">
-        <v>Defeat the Gym Leader at Lumiose City Gym</v>
+        <v>earnBadge: { badge: 'Voltage Badge', leader: 'Clemont' }</v>
       </c>
       <c r="C36" t="str">
         <v>Unlock Route 14</v>
@@ -8633,7 +8633,7 @@
         <v>Challenge 36</v>
       </c>
       <c r="B37" t="str">
-        <v>Defeat 25 Pokemon in Route 14</v>
+        <v>defeatCountRoute: { route: 'Route 14', count: 200 }</v>
       </c>
       <c r="C37" t="str">
         <v>Unlock Laverre City</v>
@@ -8644,7 +8644,7 @@
         <v>Challenge 37</v>
       </c>
       <c r="B38" t="str">
-        <v>Catch 5 different species in Laverre City</v>
+        <v>catchSpeciesAnyOf: { route: 'Laverre City', count: 5 }</v>
       </c>
       <c r="C38" t="str">
         <v>Unlock Laverre City Gym</v>
@@ -8655,7 +8655,7 @@
         <v>Challenge 38</v>
       </c>
       <c r="B39" t="str">
-        <v>Defeat the Gym Leader at Laverre City Gym</v>
+        <v>earnBadge: { badge: 'Fairy Badge', leader: 'Valerie' }</v>
       </c>
       <c r="C39" t="str">
         <v>Unlock Route 15</v>
@@ -8666,7 +8666,7 @@
         <v>Challenge 39</v>
       </c>
       <c r="B40" t="str">
-        <v>Catch 5 different species in Route 15</v>
+        <v>catchSpeciesAnyOf: { route: 'Route 15', count: 5 }</v>
       </c>
       <c r="C40" t="str">
         <v>Unlock Lost Hotel</v>
@@ -8677,7 +8677,7 @@
         <v>Challenge 40</v>
       </c>
       <c r="B41" t="str">
-        <v>Defeat 25 Pokemon in Lost Hotel</v>
+        <v>defeatCountRoute: { route: 'Lost Hotel', count: 200 }</v>
       </c>
       <c r="C41" t="str">
         <v>Unlock Dendemille Town</v>
@@ -8688,7 +8688,7 @@
         <v>Challenge 41</v>
       </c>
       <c r="B42" t="str">
-        <v>Catch 5 different species in Dendemille Town</v>
+        <v>catchSpeciesAnyOf: { route: 'Dendemille Town', count: 5 }</v>
       </c>
       <c r="C42" t="str">
         <v>Unlock Route 16</v>
@@ -8699,7 +8699,7 @@
         <v>Challenge 42</v>
       </c>
       <c r="B43" t="str">
-        <v>Defeat 25 Pokemon in Route 16</v>
+        <v>defeatCountRoute: { route: 'Route 16', count: 300 }</v>
       </c>
       <c r="C43" t="str">
         <v>Unlock Frost Cavern</v>
@@ -8710,7 +8710,7 @@
         <v>Challenge 43</v>
       </c>
       <c r="B44" t="str">
-        <v>Catch 5 different species in Frost Cavern</v>
+        <v>catchSpeciesAnyOf: { route: 'Frost Cavern', count: 5 }</v>
       </c>
       <c r="C44" t="str">
         <v>Unlock Anistar City</v>
@@ -8721,7 +8721,7 @@
         <v>Challenge 44</v>
       </c>
       <c r="B45" t="str">
-        <v>Defeat 25 Pokemon in Anistar City</v>
+        <v>defeatCountRoute: { route: 'Anistar City', count: 300 }</v>
       </c>
       <c r="C45" t="str">
         <v>Unlock Anistar City Gym</v>
@@ -8732,7 +8732,7 @@
         <v>Challenge 45</v>
       </c>
       <c r="B46" t="str">
-        <v>Defeat the Gym Leader at Anistar City Gym</v>
+        <v>earnBadge: { badge: 'Psychic Badge', leader: 'Olympia' }</v>
       </c>
       <c r="C46" t="str">
         <v>Unlock Route 17</v>
@@ -8743,7 +8743,7 @@
         <v>Challenge 46</v>
       </c>
       <c r="B47" t="str">
-        <v>Defeat 25 Pokemon in Route 17</v>
+        <v>defeatCountRoute: { route: 'Route 17', count: 300 }</v>
       </c>
       <c r="C47" t="str">
         <v>Unlock Couriway Town</v>
@@ -8754,7 +8754,7 @@
         <v>Challenge 47</v>
       </c>
       <c r="B48" t="str">
-        <v>Catch 5 different species in Couriway Town</v>
+        <v>catchSpeciesAnyOf: { route: 'Couriway Town', count: 5 }</v>
       </c>
       <c r="C48" t="str">
         <v>Unlock Route 18</v>
@@ -8765,7 +8765,7 @@
         <v>Challenge 48</v>
       </c>
       <c r="B49" t="str">
-        <v>Defeat 25 Pokemon in Route 18</v>
+        <v>defeatCountRoute: { route: 'Route 18', count: 300 }</v>
       </c>
       <c r="C49" t="str">
         <v>Unlock Terminus Cave (Surface)</v>
@@ -8776,7 +8776,7 @@
         <v>Challenge 49</v>
       </c>
       <c r="B50" t="str">
-        <v>Catch 5 different species in Terminus Cave (Surface)</v>
+        <v>catchSpeciesAnyOf: { route: 'Terminus Cave (Surface)', count: 5 }</v>
       </c>
       <c r="C50" t="str">
         <v>Unlock Route 19</v>
@@ -8787,7 +8787,7 @@
         <v>Challenge 50</v>
       </c>
       <c r="B51" t="str">
-        <v>Defeat 25 Pokemon in Route 19</v>
+        <v>defeatCountRoute: { route: 'Route 19', count: 300 }</v>
       </c>
       <c r="C51" t="str">
         <v>Unlock Route 19 (Fishing)</v>
@@ -8798,7 +8798,7 @@
         <v>Challenge 51</v>
       </c>
       <c r="B52" t="str">
-        <v>Catch 5 different species in Route 19 (Fishing)</v>
+        <v>catchSpeciesAnyOf: { route: 'Route 19 (Fishing)', count: 5 }</v>
       </c>
       <c r="C52" t="str">
         <v>Unlock Snowbelle City</v>
@@ -8809,7 +8809,7 @@
         <v>Challenge 52</v>
       </c>
       <c r="B53" t="str">
-        <v>Defeat 25 Pokemon in Snowbelle City</v>
+        <v>defeatCountRoute: { route: 'Snowbelle City', count: 300 }</v>
       </c>
       <c r="C53" t="str">
         <v>Unlock Snowbelle City Gym</v>
@@ -8820,7 +8820,7 @@
         <v>Challenge 53</v>
       </c>
       <c r="B54" t="str">
-        <v>Defeat the Gym Leader at Snowbelle City Gym</v>
+        <v>earnBadge: { badge: 'Iceberg Badge', leader: 'Wulfric' }</v>
       </c>
       <c r="C54" t="str">
         <v>Unlock Route 20</v>
@@ -8831,7 +8831,7 @@
         <v>Challenge 54</v>
       </c>
       <c r="B55" t="str">
-        <v>Defeat 25 Pokemon in Route 20</v>
+        <v>defeatCountRoute: { route: 'Route 20', count: 300 }</v>
       </c>
       <c r="C55" t="str">
         <v>Unlock Pokémon Village</v>
@@ -8842,7 +8842,7 @@
         <v>Challenge 55</v>
       </c>
       <c r="B56" t="str">
-        <v>Catch 5 different species in Pokémon Village</v>
+        <v>catchSpeciesAnyOf: { route: 'Pokémon Village', count: 5 }</v>
       </c>
       <c r="C56" t="str">
         <v>Unlock Pokémon Village (Fishing)</v>
@@ -8853,7 +8853,7 @@
         <v>Challenge 56</v>
       </c>
       <c r="B57" t="str">
-        <v>Defeat 25 Pokemon in Pokémon Village (Fishing)</v>
+        <v>defeatCountRoute: { route: 'Pokémon Village (Fishing)', count: 300 }</v>
       </c>
       <c r="C57" t="str">
         <v>Unlock Route 21</v>
@@ -8864,7 +8864,7 @@
         <v>Challenge 57</v>
       </c>
       <c r="B58" t="str">
-        <v>Catch 5 different species in Route 21</v>
+        <v>catchSpeciesAnyOf: { route: 'Route 21', count: 5 }</v>
       </c>
       <c r="C58" t="str">
         <v>Unlock Victory Road</v>
@@ -8875,7 +8875,7 @@
         <v>Challenge 58</v>
       </c>
       <c r="B59" t="str">
-        <v>Defeat 25 Pokemon in Victory Road</v>
+        <v>defeatCountRoute: { route: 'Victory Road', count: 300 }</v>
       </c>
       <c r="C59" t="str">
         <v>Unlock Kalos Pokemon League</v>
@@ -8886,7 +8886,7 @@
         <v>Challenge 59</v>
       </c>
       <c r="B60" t="str">
-        <v>Catch 5 different species in Kalos Pokemon League</v>
+        <v>catchSpeciesAnyOf: { route: 'Kalos Pokemon League', count: 5 }</v>
       </c>
       <c r="C60" t="str">
         <v>Unlock Mystic Tower Entrance</v>
@@ -8897,7 +8897,7 @@
         <v>Challenge 60</v>
       </c>
       <c r="B61" t="str">
-        <v>Defeat 25 Pokemon in Mystic Tower Entrance</v>
+        <v>defeatCountRoute: { route: 'Mystic Tower Entrance', count: 300 }</v>
       </c>
       <c r="C61" t="str">
         <v>Unlock Crystal Cave Tunnels</v>
@@ -8908,7 +8908,7 @@
         <v>Challenge 61</v>
       </c>
       <c r="B62" t="str">
-        <v>Catch 5 different species in Crystal Cave Tunnels</v>
+        <v>catchSpeciesAnyOf: { route: 'Crystal Cave Tunnels', count: 5 }</v>
       </c>
       <c r="C62" t="str">
         <v>Unlock Secret Forest North</v>
@@ -8919,7 +8919,7 @@
         <v>Final Challenge</v>
       </c>
       <c r="B63" t="str">
-        <v>Defeat the Kalos Champion at Kalos Pokemon League</v>
+        <v>defeatSpecific: { name: 'Diantha', count: 1 }</v>
       </c>
       <c r="C63" t="str">
         <v>Unlock Path to Sea Spirit Den (first spot for Extra Challenge C), Path to Team Flare Secret HQ (first spot for Extra Challenge E), Path to Secret Ruins (first spot for Extra Challenge D)</v>
@@ -8930,7 +8930,7 @@
         <v>Extra Challenge A 1</v>
       </c>
       <c r="B64" t="str">
-        <v>Complete objectives in Cyllage City (Fishing)</v>
+        <v>defeatCountRoute: { route: 'Cyllage City (Fishing)', count: 150 }</v>
       </c>
       <c r="C64" t="str">
         <v>Unlock Reflection Cave</v>
@@ -8941,7 +8941,7 @@
         <v>Extra Challenge A 2</v>
       </c>
       <c r="B65" t="str">
-        <v>Complete objectives in Reflection Cave</v>
+        <v>defeatCountRoute: { route: 'Reflection Cave', count: 150 }</v>
       </c>
       <c r="C65" t="str">
         <v>Unlock Tower of Mastery</v>
@@ -8952,7 +8952,7 @@
         <v>Extra Challenge A 3</v>
       </c>
       <c r="B66" t="str">
-        <v>Complete objectives in Tower of Mastery</v>
+        <v>defeatCountRoute: { route: 'Tower of Mastery', count: 150 }</v>
       </c>
       <c r="C66" t="str">
         <v>Unlock Coumarine City</v>
@@ -8963,7 +8963,7 @@
         <v>Extra Challenge A 4</v>
       </c>
       <c r="B67" t="str">
-        <v>Complete objectives in Coumarine City</v>
+        <v>defeatCountRoute: { route: 'Coumarine City', count: 150 }</v>
       </c>
       <c r="C67" t="str">
         <v>Earn 1 Masterball</v>
@@ -8974,7 +8974,7 @@
         <v>Extra Challenge B 1</v>
       </c>
       <c r="B68" t="str">
-        <v>Capture 1 Rowlet and 1 Litten and 1 Popplio and 1 Bulbasaur and 1 Charmander and 1 Squirtle</v>
+        <v>catchSpecies: { species: ['Rowlet', 'Litten', 'Popplio'], count: 1 }</v>
       </c>
       <c r="C68" t="str">
         <v>Unlock Starter Evolved Depot</v>
@@ -8985,7 +8985,7 @@
         <v>Extra Challenge B 2</v>
       </c>
       <c r="B69" t="str">
-        <v>Capture 1 Dartrix and 1 Torracat and 1 Brionne and 1 Ivysaur and 1 Charmeleon and 1 Blastoise</v>
+        <v>catchSpecies: { species: ['Dartrix', 'Torracat', 'Brionne'], count: 1 }</v>
       </c>
       <c r="C69" t="str">
         <v>Unlock Kiloude City</v>
@@ -8996,7 +8996,7 @@
         <v>Extra Challenge B 3</v>
       </c>
       <c r="B70" t="str">
-        <v>Complete objectives in Kiloude City</v>
+        <v>defeatCountRoute: { route: 'Kiloude City', count: 150 }</v>
       </c>
       <c r="C70" t="str">
         <v>Unlock Friend Safari</v>
@@ -9007,7 +9007,7 @@
         <v>Extra Challenge B 4</v>
       </c>
       <c r="B71" t="str">
-        <v>Complete objectives in Friend Safari</v>
+        <v>defeatCountRoute: { route: 'Friend Safari', count: 150 }</v>
       </c>
       <c r="C71" t="str">
         <v>Unlock Battle Maison</v>
@@ -9018,7 +9018,7 @@
         <v>Extra Challenge B 5</v>
       </c>
       <c r="B72" t="str">
-        <v>Complete objectives in Battle Maison</v>
+        <v>defeatCountRoute: { route: 'Battle Maison', count: 150 }</v>
       </c>
       <c r="C72" t="str">
         <v>Earn 1 Masterball</v>
@@ -9029,7 +9029,7 @@
         <v>Extra Challenge C 1</v>
       </c>
       <c r="B73" t="str">
-        <v>Complete objectives on Path to Sea Spirit Den</v>
+        <v>defeatCountRoute: { route: 'Path to Sea Spirit Den', count: 150 }</v>
       </c>
       <c r="C73" t="str">
         <v>Unlock Sea Spirit Den Outer Depths</v>
@@ -9040,7 +9040,7 @@
         <v>Extra Challenge C 2</v>
       </c>
       <c r="B74" t="str">
-        <v>Complete objectives in Sea Spirit Den Outer Depths</v>
+        <v>defeatCountRoute: { route: 'Sea Spirit Den Outer Depths', count: 150 }</v>
       </c>
       <c r="C74" t="str">
         <v>Unlock Sea Spirit Den Entrance</v>
@@ -9051,7 +9051,7 @@
         <v>Extra Challenge C 3</v>
       </c>
       <c r="B75" t="str">
-        <v>Complete objectives in Sea Spirit Den Entrance</v>
+        <v>defeatCountRoute: { route: 'Sea Spirit Den Entrance', count: 150 }</v>
       </c>
       <c r="C75" t="str">
         <v>Unlock Sea Spirit Den Tunnels</v>
@@ -9062,7 +9062,7 @@
         <v>Extra Challenge C 4</v>
       </c>
       <c r="B76" t="str">
-        <v>Complete objectives in Sea Spirit Den Tunnels</v>
+        <v>defeatCountRoute: { route: 'Sea Spirit Den Tunnels', count: 150 }</v>
       </c>
       <c r="C76" t="str">
         <v>Unlock Sea Spirit Den Hall</v>
@@ -9073,7 +9073,7 @@
         <v>Extra Challenge C 5</v>
       </c>
       <c r="B77" t="str">
-        <v>Capture 1 Articuno 1 Zapdos 1 Moltres</v>
+        <v>catchSpeciesByQuality: { species: ['Articuno', 'Zapdos', 'Moltres'], quality: 'Legendary', count: 1 }</v>
       </c>
       <c r="C77" t="str">
         <v>Earn 2 Masterball</v>
@@ -9084,7 +9084,7 @@
         <v>Extra Challenge D 1</v>
       </c>
       <c r="B78" t="str">
-        <v>Complete objectives on Path to Secret Ruins</v>
+        <v>defeatCountRoute: { route: 'Path to Secret Ruins', count: 150 }</v>
       </c>
       <c r="C78" t="str">
         <v>Unlock Underground Chambers (Crystal Cave Tunnels)</v>
@@ -9095,7 +9095,7 @@
         <v>Extra Challenge D 2</v>
       </c>
       <c r="B79" t="str">
-        <v>Complete objectives in Underground Chambers</v>
+        <v>defeatCountRoute: { route: 'Underground Chambers', count: 150 }</v>
       </c>
       <c r="C79" t="str">
         <v>Unlock Garden Chambers (Secret Forest North)</v>
@@ -9106,7 +9106,7 @@
         <v>Extra Challenge D 3</v>
       </c>
       <c r="B80" t="str">
-        <v>Complete objectives in Garden Chambers</v>
+        <v>defeatCountRoute: { route: 'Garden Chambers', count: 150 }</v>
       </c>
       <c r="C80" t="str">
         <v>Unlock Chambers of Emptiness</v>
@@ -9117,7 +9117,7 @@
         <v>Extra Challenge D 4</v>
       </c>
       <c r="B81" t="str">
-        <v>Complete objectives in Chambers of Emptiness</v>
+        <v>defeatCountRoute: { route: 'Chambers of Emptiness', count: 150 }</v>
       </c>
       <c r="C81" t="str">
         <v>Unlock Ultimate Chamber</v>
@@ -9128,7 +9128,7 @@
         <v>Extra Challenge D 5</v>
       </c>
       <c r="B82" t="str">
-        <v>Capture 1 Volcanion 1 Diance 1 Hoopa 1 Mewtwo</v>
+        <v>catchSpeciesByQuality: { species: ['Volcanion', 'Diancie', 'Hoopa', 'Mewtwo'], quality: 'Mythical', count: 1 }</v>
       </c>
       <c r="C82" t="str">
         <v>Earn 2 Masterball</v>
@@ -9139,7 +9139,7 @@
         <v>Extra Challenge E 1</v>
       </c>
       <c r="B83" t="str">
-        <v>Complete objectives on Path to Team Flare Secret HQ</v>
+        <v>defeatCountRoute: { route: 'Path to Team Flare Secret HQ', count: 150 }</v>
       </c>
       <c r="C83" t="str">
         <v>Unlock 2nd spot for Extra Challenge E</v>
@@ -9150,7 +9150,7 @@
         <v>Extra Challenge E 2</v>
       </c>
       <c r="B84" t="str">
-        <v>Complete objectives on 2nd spot for Extra Challenge E</v>
+        <v>defeatCountRoute: { route: '2nd spot for Extra Challenge E', count: 150 }</v>
       </c>
       <c r="C84" t="str">
         <v>Unlock Team Flare Secret HQ Gate</v>
@@ -9161,7 +9161,7 @@
         <v>Extra Challenge E 3</v>
       </c>
       <c r="B85" t="str">
-        <v>Complete objectives in Team Flare Secret HQ Gate</v>
+        <v>defeatCountRoute: { route: 'Team Flare Secret HQ Gate', count: 150 }</v>
       </c>
       <c r="C85" t="str">
         <v>Unlock Team Flare Secret HQ Entrance</v>
@@ -9172,7 +9172,7 @@
         <v>Extra Challenge E 4</v>
       </c>
       <c r="B86" t="str">
-        <v>Complete objectives in Team Flare Secret HQ Entrance</v>
+        <v>defeatCountRoute: { route: 'Team Flare Secret HQ Entrance', count: 150 }</v>
       </c>
       <c r="C86" t="str">
         <v>Unlock Team Flare Secret HQ Hall</v>
@@ -9183,7 +9183,7 @@
         <v>Extra Challenge E 5</v>
       </c>
       <c r="B87" t="str">
-        <v>Capture 1 Ybeltal 1 Zygarde 1 Xerneas</v>
+        <v>catchSpeciesByQuality: { species: ['Yveltal', 'Zygarde', 'Xerneas'], quality: 'Legendary', count: 1 }</v>
       </c>
       <c r="C87" t="str">
         <v>Earn 2 Masterball</v>

</xml_diff>

<commit_message>
Rebalance Kalos routes sequentially by BST to prevent overpowered early encounters
Co-authored-by: lsampaio1337-beep <246645260+lsampaio1337-beep@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Kalos_Path.xlsx
+++ b/Kalos_Path.xlsx
@@ -426,7 +426,7 @@
         <v>Aquacorde Town</v>
       </c>
       <c r="C2" t="str">
-        <v>Gible</v>
+        <v>Azurill</v>
       </c>
       <c r="D2" t="str">
         <v>1-3</v>
@@ -443,7 +443,7 @@
         <v>Aquacorde Town</v>
       </c>
       <c r="C3" t="str">
-        <v>Sandile</v>
+        <v>Caterpie</v>
       </c>
       <c r="D3" t="str">
         <v>1-3</v>
@@ -460,7 +460,7 @@
         <v>Aquacorde Town</v>
       </c>
       <c r="C4" t="str">
-        <v>Cubone</v>
+        <v>Weedle</v>
       </c>
       <c r="D4" t="str">
         <v>1-3</v>
@@ -477,7 +477,7 @@
         <v>Aquacorde Town</v>
       </c>
       <c r="C5" t="str">
-        <v>Woobat</v>
+        <v>Ralts</v>
       </c>
       <c r="D5" t="str">
         <v>1-3</v>
@@ -494,7 +494,7 @@
         <v>Aquacorde Town</v>
       </c>
       <c r="C6" t="str">
-        <v>Clawitzer</v>
+        <v>Scatterbug</v>
       </c>
       <c r="D6" t="str">
         <v>1-3</v>
@@ -511,7 +511,7 @@
         <v>Aquacorde Town</v>
       </c>
       <c r="C7" t="str">
-        <v>Mr-mime</v>
+        <v>Magikarp</v>
       </c>
       <c r="D7" t="str">
         <v>1-3</v>
@@ -528,7 +528,7 @@
         <v>Route 2</v>
       </c>
       <c r="C8" t="str">
-        <v>Bunnelby</v>
+        <v>Kakuna</v>
       </c>
       <c r="D8" t="str">
         <v>1-3</v>
@@ -545,7 +545,7 @@
         <v>Route 2</v>
       </c>
       <c r="C9" t="str">
-        <v>Trubbish</v>
+        <v>Metapod</v>
       </c>
       <c r="D9" t="str">
         <v>1-3</v>
@@ -562,7 +562,7 @@
         <v>Route 2</v>
       </c>
       <c r="C10" t="str">
-        <v>Duosion</v>
+        <v>Pichu</v>
       </c>
       <c r="D10" t="str">
         <v>1-3</v>
@@ -579,7 +579,7 @@
         <v>Route 2</v>
       </c>
       <c r="C11" t="str">
-        <v>Staravia</v>
+        <v>Igglybuff</v>
       </c>
       <c r="D11" t="str">
         <v>1-3</v>
@@ -596,7 +596,7 @@
         <v>Route 2</v>
       </c>
       <c r="C12" t="str">
-        <v>Dedenne</v>
+        <v>Wooper</v>
       </c>
       <c r="D12" t="str">
         <v>1-3</v>
@@ -613,7 +613,7 @@
         <v>Route 2</v>
       </c>
       <c r="C13" t="str">
-        <v>Vibrava</v>
+        <v>Spewpa</v>
       </c>
       <c r="D13" t="str">
         <v>1-3</v>
@@ -630,7 +630,7 @@
         <v>Santalune Forest</v>
       </c>
       <c r="C14" t="str">
-        <v>Blastoise</v>
+        <v>Sentret</v>
       </c>
       <c r="D14" t="str">
         <v>2-4</v>
@@ -647,7 +647,7 @@
         <v>Santalune Forest</v>
       </c>
       <c r="C15" t="str">
-        <v>Chinchou</v>
+        <v>Poochyena</v>
       </c>
       <c r="D15" t="str">
         <v>2-4</v>
@@ -664,7 +664,7 @@
         <v>Santalune Forest</v>
       </c>
       <c r="C16" t="str">
-        <v>Mantyke</v>
+        <v>Lotad</v>
       </c>
       <c r="D16" t="str">
         <v>2-4</v>
@@ -681,7 +681,7 @@
         <v>Santalune Forest</v>
       </c>
       <c r="C17" t="str">
-        <v>Hawlucha</v>
+        <v>Burmy</v>
       </c>
       <c r="D17" t="str">
         <v>2-4</v>
@@ -698,7 +698,7 @@
         <v>Santalune Forest</v>
       </c>
       <c r="C18" t="str">
-        <v>Sableye</v>
+        <v>Bunnelby</v>
       </c>
       <c r="D18" t="str">
         <v>2-4</v>
@@ -715,7 +715,7 @@
         <v>Santalune Forest</v>
       </c>
       <c r="C19" t="str">
-        <v>Zangoose</v>
+        <v>Zigzagoon</v>
       </c>
       <c r="D19" t="str">
         <v>2-4</v>
@@ -732,7 +732,7 @@
         <v>Route 3</v>
       </c>
       <c r="C20" t="str">
-        <v>Nidorino</v>
+        <v>Whismur</v>
       </c>
       <c r="D20" t="str">
         <v>3-5</v>
@@ -749,7 +749,7 @@
         <v>Route 3</v>
       </c>
       <c r="C21" t="str">
-        <v>Burmy</v>
+        <v>Combee</v>
       </c>
       <c r="D21" t="str">
         <v>3-5</v>
@@ -766,7 +766,7 @@
         <v>Route 3</v>
       </c>
       <c r="C22" t="str">
-        <v>Carbink</v>
+        <v>Starly</v>
       </c>
       <c r="D22" t="str">
         <v>3-5</v>
@@ -783,7 +783,7 @@
         <v>Route 3</v>
       </c>
       <c r="C23" t="str">
-        <v>Nidoqueen</v>
+        <v>Zubat</v>
       </c>
       <c r="D23" t="str">
         <v>3-5</v>
@@ -800,7 +800,7 @@
         <v>Route 3</v>
       </c>
       <c r="C24" t="str">
-        <v>Pachirisu</v>
+        <v>Noibat</v>
       </c>
       <c r="D24" t="str">
         <v>3-5</v>
@@ -817,7 +817,7 @@
         <v>Route 3</v>
       </c>
       <c r="C25" t="str">
-        <v>Solosis</v>
+        <v>Bidoof</v>
       </c>
       <c r="D25" t="str">
         <v>3-5</v>
@@ -834,7 +834,7 @@
         <v>Santalune City</v>
       </c>
       <c r="C26" t="str">
-        <v>Eevee</v>
+        <v>Swinub</v>
       </c>
       <c r="D26" t="str">
         <v>4-6</v>
@@ -851,7 +851,7 @@
         <v>Santalune City</v>
       </c>
       <c r="C27" t="str">
-        <v>Krokorok</v>
+        <v>Smeargle</v>
       </c>
       <c r="D27" t="str">
         <v>4-6</v>
@@ -868,7 +868,7 @@
         <v>Santalune City</v>
       </c>
       <c r="C28" t="str">
-        <v>Pinsir</v>
+        <v>Slugma</v>
       </c>
       <c r="D28" t="str">
         <v>4-6</v>
@@ -885,7 +885,7 @@
         <v>Santalune City</v>
       </c>
       <c r="C29" t="str">
-        <v>Sharpedo</v>
+        <v>Hoppip</v>
       </c>
       <c r="D29" t="str">
         <v>4-6</v>
@@ -902,7 +902,7 @@
         <v>Santalune City</v>
       </c>
       <c r="C30" t="str">
-        <v>Bidoof</v>
+        <v>Spinarak</v>
       </c>
       <c r="D30" t="str">
         <v>4-6</v>
@@ -919,7 +919,7 @@
         <v>Santalune City</v>
       </c>
       <c r="C31" t="str">
-        <v>Fraxure</v>
+        <v>Pidgey</v>
       </c>
       <c r="D31" t="str">
         <v>4-6</v>
@@ -936,7 +936,7 @@
         <v>Santalune City Gym</v>
       </c>
       <c r="C32" t="str">
-        <v>Litwick</v>
+        <v>Patrat</v>
       </c>
       <c r="D32" t="str">
         <v>5-7</v>
@@ -953,7 +953,7 @@
         <v>Santalune City Gym</v>
       </c>
       <c r="C33" t="str">
-        <v>Snubbull</v>
+        <v>Skitty</v>
       </c>
       <c r="D33" t="str">
         <v>5-7</v>
@@ -970,7 +970,7 @@
         <v>Santalune City Gym</v>
       </c>
       <c r="C34" t="str">
-        <v>Pidgeotto</v>
+        <v>Venipede</v>
       </c>
       <c r="D34" t="str">
         <v>5-7</v>
@@ -987,7 +987,7 @@
         <v>Santalune City Gym</v>
       </c>
       <c r="C35" t="str">
-        <v>Pupitar</v>
+        <v>Wynaut</v>
       </c>
       <c r="D35" t="str">
         <v>5-7</v>
@@ -1004,7 +1004,7 @@
         <v>Santalune City Gym</v>
       </c>
       <c r="C36" t="str">
-        <v>Swinub</v>
+        <v>Hoothoot</v>
       </c>
       <c r="D36" t="str">
         <v>5-7</v>
@@ -1021,7 +1021,7 @@
         <v>Santalune City Gym</v>
       </c>
       <c r="C37" t="str">
-        <v>Wigglytuff</v>
+        <v>Spearow</v>
       </c>
       <c r="D37" t="str">
         <v>5-7</v>
@@ -1038,7 +1038,7 @@
         <v>Route 22</v>
       </c>
       <c r="C38" t="str">
-        <v>Smeargle</v>
+        <v>Diglett</v>
       </c>
       <c r="D38" t="str">
         <v>6-8</v>
@@ -1055,7 +1055,7 @@
         <v>Route 22</v>
       </c>
       <c r="C39" t="str">
-        <v>Miltank</v>
+        <v>Ledyba</v>
       </c>
       <c r="D39" t="str">
         <v>6-8</v>
@@ -1072,7 +1072,7 @@
         <v>Route 22</v>
       </c>
       <c r="C40" t="str">
-        <v>Bellossom</v>
+        <v>Nincada</v>
       </c>
       <c r="D40" t="str">
         <v>6-8</v>
@@ -1089,7 +1089,7 @@
         <v>Route 22</v>
       </c>
       <c r="C41" t="str">
-        <v>Jynx</v>
+        <v>Surskit</v>
       </c>
       <c r="D41" t="str">
         <v>6-8</v>
@@ -1106,7 +1106,7 @@
         <v>Route 22</v>
       </c>
       <c r="C42" t="str">
-        <v>Smoochum</v>
+        <v>Taillow</v>
       </c>
       <c r="D42" t="str">
         <v>6-8</v>
@@ -1123,7 +1123,7 @@
         <v>Route 22</v>
       </c>
       <c r="C43" t="str">
-        <v>Scolipede</v>
+        <v>Wingull</v>
       </c>
       <c r="D43" t="str">
         <v>6-8</v>
@@ -1140,7 +1140,7 @@
         <v>Route 4</v>
       </c>
       <c r="C44" t="str">
-        <v>Vanilluxe</v>
+        <v>Litwick</v>
       </c>
       <c r="D44" t="str">
         <v>7-9</v>
@@ -1157,7 +1157,7 @@
         <v>Route 4</v>
       </c>
       <c r="C45" t="str">
-        <v>Rhyhorn</v>
+        <v>Kirlia</v>
       </c>
       <c r="D45" t="str">
         <v>7-9</v>
@@ -1174,7 +1174,7 @@
         <v>Route 4</v>
       </c>
       <c r="C46" t="str">
-        <v>Stunfisk</v>
+        <v>Fletchling</v>
       </c>
       <c r="D46" t="str">
         <v>7-9</v>
@@ -1191,7 +1191,7 @@
         <v>Route 4</v>
       </c>
       <c r="C47" t="str">
-        <v>Carnivine</v>
+        <v>Meditite</v>
       </c>
       <c r="D47" t="str">
         <v>7-9</v>
@@ -1208,7 +1208,7 @@
         <v>Route 4</v>
       </c>
       <c r="C48" t="str">
-        <v>Lombre</v>
+        <v>Budew</v>
       </c>
       <c r="D48" t="str">
         <v>7-9</v>
@@ -1225,7 +1225,7 @@
         <v>Route 4</v>
       </c>
       <c r="C49" t="str">
-        <v>Hoothoot</v>
+        <v>Mareep</v>
       </c>
       <c r="D49" t="str">
         <v>7-9</v>
@@ -1242,7 +1242,7 @@
         <v>Lumiose City (South)</v>
       </c>
       <c r="C50" t="str">
-        <v>Basculin</v>
+        <v>Roggenrola</v>
       </c>
       <c r="D50" t="str">
         <v>8-10</v>
@@ -1259,7 +1259,7 @@
         <v>Lumiose City (South)</v>
       </c>
       <c r="C51" t="str">
-        <v>Slowbro</v>
+        <v>Purrloin</v>
       </c>
       <c r="D51" t="str">
         <v>8-10</v>
@@ -1276,7 +1276,7 @@
         <v>Lumiose City (South)</v>
       </c>
       <c r="C52" t="str">
-        <v>Sandshrew</v>
+        <v>Chingling</v>
       </c>
       <c r="D52" t="str">
         <v>8-10</v>
@@ -1293,7 +1293,7 @@
         <v>Lumiose City (South)</v>
       </c>
       <c r="C53" t="str">
-        <v>Slurpuff</v>
+        <v>Riolu</v>
       </c>
       <c r="D53" t="str">
         <v>8-10</v>
@@ -1310,7 +1310,7 @@
         <v>Lumiose City (South)</v>
       </c>
       <c r="C54" t="str">
-        <v>Abra</v>
+        <v>Barboach</v>
       </c>
       <c r="D54" t="str">
         <v>8-10</v>
@@ -1327,7 +1327,7 @@
         <v>Lumiose City (South)</v>
       </c>
       <c r="C55" t="str">
-        <v>Ninjask</v>
+        <v>Ekans</v>
       </c>
       <c r="D55" t="str">
         <v>8-10</v>
@@ -1344,7 +1344,7 @@
         <v>Route 5</v>
       </c>
       <c r="C56" t="str">
-        <v>Boldore</v>
+        <v>Inkay</v>
       </c>
       <c r="D56" t="str">
         <v>9-11</v>
@@ -1361,7 +1361,7 @@
         <v>Route 5</v>
       </c>
       <c r="C57" t="str">
-        <v>Furret</v>
+        <v>Ditto</v>
       </c>
       <c r="D57" t="str">
         <v>9-11</v>
@@ -1378,7 +1378,7 @@
         <v>Route 5</v>
       </c>
       <c r="C58" t="str">
-        <v>Vaporeon</v>
+        <v>Helioptile</v>
       </c>
       <c r="D58" t="str">
         <v>9-11</v>
@@ -1395,7 +1395,7 @@
         <v>Route 5</v>
       </c>
       <c r="C59" t="str">
-        <v>Tyrantrum</v>
+        <v>Solosis</v>
       </c>
       <c r="D59" t="str">
         <v>9-11</v>
@@ -1412,7 +1412,7 @@
         <v>Route 5</v>
       </c>
       <c r="C60" t="str">
-        <v>Diglett</v>
+        <v>Trapinch</v>
       </c>
       <c r="D60" t="str">
         <v>9-11</v>
@@ -1429,7 +1429,7 @@
         <v>Route 5</v>
       </c>
       <c r="C61" t="str">
-        <v>Yveltal</v>
+        <v>Bonsly</v>
       </c>
       <c r="D61" t="str">
         <v>9-11</v>
@@ -1446,7 +1446,7 @@
         <v>Camphrier Town</v>
       </c>
       <c r="C62" t="str">
-        <v>Kirlia</v>
+        <v>Gothita</v>
       </c>
       <c r="D62" t="str">
         <v>10-12</v>
@@ -1463,7 +1463,7 @@
         <v>Camphrier Town</v>
       </c>
       <c r="C63" t="str">
-        <v>Poliwrath</v>
+        <v>Sandile</v>
       </c>
       <c r="D63" t="str">
         <v>10-12</v>
@@ -1480,7 +1480,7 @@
         <v>Camphrier Town</v>
       </c>
       <c r="C64" t="str">
-        <v>Linoone</v>
+        <v>Foongus</v>
       </c>
       <c r="D64" t="str">
         <v>10-12</v>
@@ -1497,7 +1497,7 @@
         <v>Camphrier Town</v>
       </c>
       <c r="C65" t="str">
-        <v>Houndour</v>
+        <v>Electrike</v>
       </c>
       <c r="D65" t="str">
         <v>10-12</v>
@@ -1514,7 +1514,7 @@
         <v>Camphrier Town</v>
       </c>
       <c r="C66" t="str">
-        <v>Plusle</v>
+        <v>Horsea</v>
       </c>
       <c r="D66" t="str">
         <v>10-12</v>
@@ -1531,7 +1531,7 @@
         <v>Camphrier Town</v>
       </c>
       <c r="C67" t="str">
-        <v>Lairon</v>
+        <v>Shuppet</v>
       </c>
       <c r="D67" t="str">
         <v>10-12</v>
@@ -1548,7 +1548,7 @@
         <v>Parfum Palace</v>
       </c>
       <c r="C68" t="str">
-        <v>Combee</v>
+        <v>Gible</v>
       </c>
       <c r="D68" t="str">
         <v>11-13</v>
@@ -1565,7 +1565,7 @@
         <v>Parfum Palace</v>
       </c>
       <c r="C69" t="str">
-        <v>Chandelure</v>
+        <v>Mr-mime</v>
       </c>
       <c r="D69" t="str">
         <v>11-13</v>
@@ -1582,7 +1582,7 @@
         <v>Parfum Palace</v>
       </c>
       <c r="C70" t="str">
-        <v>Steelix</v>
+        <v>Snubbull</v>
       </c>
       <c r="D70" t="str">
         <v>11-13</v>
@@ -1599,7 +1599,7 @@
         <v>Parfum Palace</v>
       </c>
       <c r="C71" t="str">
-        <v>Sylveon</v>
+        <v>Sandshrew</v>
       </c>
       <c r="D71" t="str">
         <v>11-13</v>
@@ -1616,7 +1616,7 @@
         <v>Parfum Palace</v>
       </c>
       <c r="C72" t="str">
-        <v>Starly</v>
+        <v>Nidoran-f</v>
       </c>
       <c r="D72" t="str">
         <v>11-13</v>
@@ -1633,7 +1633,7 @@
         <v>Parfum Palace</v>
       </c>
       <c r="C73" t="str">
-        <v>Barbaracle</v>
+        <v>Larvitar</v>
       </c>
       <c r="D73" t="str">
         <v>11-13</v>
@@ -1650,7 +1650,7 @@
         <v>Route 6</v>
       </c>
       <c r="C74" t="str">
-        <v>Beedrill</v>
+        <v>Poliwag</v>
       </c>
       <c r="D74" t="str">
         <v>12-14</v>
@@ -1667,7 +1667,7 @@
         <v>Route 6</v>
       </c>
       <c r="C75" t="str">
-        <v>Delphox</v>
+        <v>Nidoran-m</v>
       </c>
       <c r="D75" t="str">
         <v>12-14</v>
@@ -1684,7 +1684,7 @@
         <v>Route 6</v>
       </c>
       <c r="C76" t="str">
-        <v>Simisage</v>
+        <v>Farfetchd</v>
       </c>
       <c r="D76" t="str">
         <v>12-14</v>
@@ -1701,7 +1701,7 @@
         <v>Route 6</v>
       </c>
       <c r="C77" t="str">
-        <v>Crobat</v>
+        <v>Bellsprout</v>
       </c>
       <c r="D77" t="str">
         <v>12-14</v>
@@ -1718,7 +1718,7 @@
         <v>Route 6</v>
       </c>
       <c r="C78" t="str">
-        <v>Electrike</v>
+        <v>Flabebe</v>
       </c>
       <c r="D78" t="str">
         <v>12-14</v>
@@ -1735,7 +1735,7 @@
         <v>Route 6</v>
       </c>
       <c r="C79" t="str">
-        <v>Nidorina</v>
+        <v>Goomy</v>
       </c>
       <c r="D79" t="str">
         <v>12-14</v>
@@ -1752,7 +1752,7 @@
         <v>Route 7</v>
       </c>
       <c r="C80" t="str">
-        <v>Purrloin</v>
+        <v>Dratini</v>
       </c>
       <c r="D80" t="str">
         <v>13-15</v>
@@ -1769,7 +1769,7 @@
         <v>Route 7</v>
       </c>
       <c r="C81" t="str">
-        <v>Cubchoo</v>
+        <v>Remoraid</v>
       </c>
       <c r="D81" t="str">
         <v>13-15</v>
@@ -1786,7 +1786,7 @@
         <v>Route 7</v>
       </c>
       <c r="C82" t="str">
-        <v>Dragalge</v>
+        <v>Mime-jr</v>
       </c>
       <c r="D82" t="str">
         <v>13-15</v>
@@ -1803,7 +1803,7 @@
         <v>Route 7</v>
       </c>
       <c r="C83" t="str">
-        <v>Fletchinder</v>
+        <v>Croagunk</v>
       </c>
       <c r="D83" t="str">
         <v>13-15</v>
@@ -1820,7 +1820,7 @@
         <v>Route 7</v>
       </c>
       <c r="C84" t="str">
-        <v>Horsea</v>
+        <v>Deino</v>
       </c>
       <c r="D84" t="str">
         <v>13-15</v>
@@ -1837,7 +1837,7 @@
         <v>Route 7</v>
       </c>
       <c r="C85" t="str">
-        <v>Poliwhirl</v>
+        <v>Geodude</v>
       </c>
       <c r="D85" t="str">
         <v>13-15</v>
@@ -1854,7 +1854,7 @@
         <v>Connecting Cave</v>
       </c>
       <c r="C86" t="str">
-        <v>Machoke</v>
+        <v>Bagon</v>
       </c>
       <c r="D86" t="str">
         <v>14-16</v>
@@ -1871,7 +1871,7 @@
         <v>Connecting Cave</v>
       </c>
       <c r="C87" t="str">
-        <v>Skuntank</v>
+        <v>Gulpin</v>
       </c>
       <c r="D87" t="str">
         <v>14-16</v>
@@ -1888,7 +1888,7 @@
         <v>Connecting Cave</v>
       </c>
       <c r="C88" t="str">
-        <v>Probopass</v>
+        <v>Golett</v>
       </c>
       <c r="D88" t="str">
         <v>14-16</v>
@@ -1905,7 +1905,7 @@
         <v>Connecting Cave</v>
       </c>
       <c r="C89" t="str">
-        <v>Chesnaught</v>
+        <v>Bergmite</v>
       </c>
       <c r="D89" t="str">
         <v>14-16</v>
@@ -1922,7 +1922,7 @@
         <v>Connecting Cave</v>
       </c>
       <c r="C90" t="str">
-        <v>Helioptile</v>
+        <v>Smoochum</v>
       </c>
       <c r="D90" t="str">
         <v>14-16</v>
@@ -1939,7 +1939,7 @@
         <v>Connecting Cave</v>
       </c>
       <c r="C91" t="str">
-        <v>Scizor</v>
+        <v>Cubchoo</v>
       </c>
       <c r="D91" t="str">
         <v>14-16</v>
@@ -1956,7 +1956,7 @@
         <v>Ambrette Town</v>
       </c>
       <c r="C92" t="str">
-        <v>Phantump</v>
+        <v>Shelmet</v>
       </c>
       <c r="D92" t="str">
         <v>15-17</v>
@@ -1973,7 +1973,7 @@
         <v>Ambrette Town</v>
       </c>
       <c r="C93" t="str">
-        <v>Goldeen</v>
+        <v>Ferroseed</v>
       </c>
       <c r="D93" t="str">
         <v>15-17</v>
@@ -1990,7 +1990,7 @@
         <v>Ambrette Town</v>
       </c>
       <c r="C94" t="str">
-        <v>Gurdurr</v>
+        <v>Vanillite</v>
       </c>
       <c r="D94" t="str">
         <v>15-17</v>
@@ -2007,7 +2007,7 @@
         <v>Ambrette Town</v>
       </c>
       <c r="C95" t="str">
-        <v>Aromatisse</v>
+        <v>Timburr</v>
       </c>
       <c r="D95" t="str">
         <v>15-17</v>
@@ -2024,7 +2024,7 @@
         <v>Ambrette Town</v>
       </c>
       <c r="C96" t="str">
-        <v>Gengar</v>
+        <v>Ducklett</v>
       </c>
       <c r="D96" t="str">
         <v>15-17</v>
@@ -2041,7 +2041,7 @@
         <v>Ambrette Town</v>
       </c>
       <c r="C97" t="str">
-        <v>Vileplume</v>
+        <v>Machop</v>
       </c>
       <c r="D97" t="str">
         <v>15-17</v>
@@ -2058,7 +2058,7 @@
         <v>Ambrette Town (Fishing)</v>
       </c>
       <c r="C98" t="str">
-        <v>Grumpig</v>
+        <v>Shellder</v>
       </c>
       <c r="D98" t="str">
         <v>17-19</v>
@@ -2075,7 +2075,7 @@
         <v>Ambrette Town (Fishing)</v>
       </c>
       <c r="C99" t="str">
-        <v>Swalot</v>
+        <v>Carvanha</v>
       </c>
       <c r="D99" t="str">
         <v>17-19</v>
@@ -2092,7 +2092,7 @@
         <v>Ambrette Town (Fishing)</v>
       </c>
       <c r="C100" t="str">
-        <v>Sandslash</v>
+        <v>Binacle</v>
       </c>
       <c r="D100" t="str">
         <v>17-19</v>
@@ -2109,7 +2109,7 @@
         <v>Ambrette Town (Fishing)</v>
       </c>
       <c r="C101" t="str">
-        <v>Litleo</v>
+        <v>Corphish</v>
       </c>
       <c r="D101" t="str">
         <v>17-19</v>
@@ -2126,7 +2126,7 @@
         <v>Ambrette Town (Fishing)</v>
       </c>
       <c r="C102" t="str">
-        <v>Shelmet</v>
+        <v>Phantump</v>
       </c>
       <c r="D102" t="str">
         <v>17-19</v>
@@ -2143,7 +2143,7 @@
         <v>Ambrette Town (Fishing)</v>
       </c>
       <c r="C103" t="str">
-        <v>Bisharp</v>
+        <v>Abra</v>
       </c>
       <c r="D103" t="str">
         <v>17-19</v>
@@ -2160,7 +2160,7 @@
         <v>Route 8</v>
       </c>
       <c r="C104" t="str">
-        <v>Nidoran-f</v>
+        <v>Doduo</v>
       </c>
       <c r="D104" t="str">
         <v>18-20</v>
@@ -2177,7 +2177,7 @@
         <v>Route 8</v>
       </c>
       <c r="C105" t="str">
-        <v>Seadra</v>
+        <v>Gastly</v>
       </c>
       <c r="D105" t="str">
         <v>18-20</v>
@@ -2194,7 +2194,7 @@
         <v>Route 8</v>
       </c>
       <c r="C106" t="str">
-        <v>Ferroseed</v>
+        <v>Swablu</v>
       </c>
       <c r="D106" t="str">
         <v>18-20</v>
@@ -2211,7 +2211,7 @@
         <v>Route 8</v>
       </c>
       <c r="C107" t="str">
-        <v>Honedge</v>
+        <v>Slowpoke</v>
       </c>
       <c r="D107" t="str">
         <v>18-20</v>
@@ -2228,7 +2228,7 @@
         <v>Route 8</v>
       </c>
       <c r="C108" t="str">
-        <v>Larvitar</v>
+        <v>Karrablast</v>
       </c>
       <c r="D108" t="str">
         <v>18-20</v>
@@ -2245,7 +2245,7 @@
         <v>Route 8</v>
       </c>
       <c r="C109" t="str">
-        <v>Spritzee</v>
+        <v>Pansear</v>
       </c>
       <c r="D109" t="str">
         <v>18-20</v>
@@ -2262,7 +2262,7 @@
         <v>Route 9</v>
       </c>
       <c r="C110" t="str">
-        <v>Whirlipede</v>
+        <v>Pansage</v>
       </c>
       <c r="D110" t="str">
         <v>19-21</v>
@@ -2279,7 +2279,7 @@
         <v>Route 9</v>
       </c>
       <c r="C111" t="str">
-        <v>Hariyama</v>
+        <v>Panpour</v>
       </c>
       <c r="D111" t="str">
         <v>19-21</v>
@@ -2296,7 +2296,7 @@
         <v>Route 9</v>
       </c>
       <c r="C112" t="str">
-        <v>Lucario</v>
+        <v>Cubone</v>
       </c>
       <c r="D112" t="str">
         <v>19-21</v>
@@ -2313,7 +2313,7 @@
         <v>Route 9</v>
       </c>
       <c r="C113" t="str">
-        <v>Volbeat</v>
+        <v>Goldeen</v>
       </c>
       <c r="D113" t="str">
         <v>19-21</v>
@@ -2330,7 +2330,7 @@
         <v>Route 9</v>
       </c>
       <c r="C114" t="str">
-        <v>Voltorb</v>
+        <v>Psyduck</v>
       </c>
       <c r="D114" t="str">
         <v>19-21</v>
@@ -2347,7 +2347,7 @@
         <v>Route 9</v>
       </c>
       <c r="C115" t="str">
-        <v>Flareon</v>
+        <v>Skrelp</v>
       </c>
       <c r="D115" t="str">
         <v>19-21</v>
@@ -2364,7 +2364,7 @@
         <v>Glittering Cave</v>
       </c>
       <c r="C116" t="str">
-        <v>Krookodile</v>
+        <v>Axew</v>
       </c>
       <c r="D116" t="str">
         <v>20-22</v>
@@ -2381,7 +2381,7 @@
         <v>Glittering Cave</v>
       </c>
       <c r="C117" t="str">
-        <v>Rotom</v>
+        <v>Oddish</v>
       </c>
       <c r="D117" t="str">
         <v>20-22</v>
@@ -2398,7 +2398,7 @@
         <v>Glittering Cave</v>
       </c>
       <c r="C118" t="str">
-        <v>Dunsparce</v>
+        <v>Woobat</v>
       </c>
       <c r="D118" t="str">
         <v>20-22</v>
@@ -2415,7 +2415,7 @@
         <v>Glittering Cave</v>
       </c>
       <c r="C119" t="str">
-        <v>Lunatone</v>
+        <v>Eevee</v>
       </c>
       <c r="D119" t="str">
         <v>20-22</v>
@@ -2432,7 +2432,7 @@
         <v>Glittering Cave</v>
       </c>
       <c r="C120" t="str">
-        <v>Machamp</v>
+        <v>Honedge</v>
       </c>
       <c r="D120" t="str">
         <v>20-22</v>
@@ -2449,7 +2449,7 @@
         <v>Glittering Cave</v>
       </c>
       <c r="C121" t="str">
-        <v>Alakazam</v>
+        <v>Magnemite</v>
       </c>
       <c r="D121" t="str">
         <v>20-22</v>
@@ -2466,7 +2466,7 @@
         <v>Cyllage City</v>
       </c>
       <c r="C122" t="str">
-        <v>Doduo</v>
+        <v>Exeggcute</v>
       </c>
       <c r="D122" t="str">
         <v>21-23</v>
@@ -2483,7 +2483,7 @@
         <v>Cyllage City</v>
       </c>
       <c r="C123" t="str">
-        <v>Gourgeist</v>
+        <v>Dwebble</v>
       </c>
       <c r="D123" t="str">
         <v>21-23</v>
@@ -2500,7 +2500,7 @@
         <v>Cyllage City</v>
       </c>
       <c r="C124" t="str">
-        <v>Mienfoo</v>
+        <v>Trubbish</v>
       </c>
       <c r="D124" t="str">
         <v>21-23</v>
@@ -2517,7 +2517,7 @@
         <v>Cyllage City</v>
       </c>
       <c r="C125" t="str">
-        <v>Honchkrow</v>
+        <v>Stunky</v>
       </c>
       <c r="D125" t="str">
         <v>21-23</v>
@@ -2534,7 +2534,7 @@
         <v>Cyllage City</v>
       </c>
       <c r="C126" t="str">
-        <v>Kadabra</v>
+        <v>Chinchou</v>
       </c>
       <c r="D126" t="str">
         <v>21-23</v>
@@ -2551,7 +2551,7 @@
         <v>Cyllage City</v>
       </c>
       <c r="C127" t="str">
-        <v>Drifblim</v>
+        <v>Houndour</v>
       </c>
       <c r="D127" t="str">
         <v>21-23</v>
@@ -2568,7 +2568,7 @@
         <v>Cyllage City Gym</v>
       </c>
       <c r="C128" t="str">
-        <v>Magnemite</v>
+        <v>Voltorb</v>
       </c>
       <c r="D128" t="str">
         <v>22-24</v>
@@ -2585,7 +2585,7 @@
         <v>Cyllage City Gym</v>
       </c>
       <c r="C129" t="str">
-        <v>Golurk</v>
+        <v>Skorupi</v>
       </c>
       <c r="D129" t="str">
         <v>22-24</v>
@@ -2602,7 +2602,7 @@
         <v>Cyllage City Gym</v>
       </c>
       <c r="C130" t="str">
-        <v>Klefki</v>
+        <v>Spoink</v>
       </c>
       <c r="D130" t="str">
         <v>22-24</v>
@@ -2619,7 +2619,7 @@
         <v>Cyllage City Gym</v>
       </c>
       <c r="C131" t="str">
-        <v>Mamoswine</v>
+        <v>Delibird</v>
       </c>
       <c r="D131" t="str">
         <v>22-24</v>
@@ -2636,7 +2636,7 @@
         <v>Cyllage City Gym</v>
       </c>
       <c r="C132" t="str">
-        <v>Nincada</v>
+        <v>Teddiursa</v>
       </c>
       <c r="D132" t="str">
         <v>22-24</v>
@@ -2653,7 +2653,7 @@
         <v>Cyllage City Gym</v>
       </c>
       <c r="C133" t="str">
-        <v>Mewtwo</v>
+        <v>Hippopotas</v>
       </c>
       <c r="D133" t="str">
         <v>22-24</v>
@@ -2670,7 +2670,7 @@
         <v>Cyllage City (Fishing)</v>
       </c>
       <c r="C134" t="str">
-        <v>Throh</v>
+        <v>Clauncher</v>
       </c>
       <c r="D134" t="str">
         <v>25-30</v>
@@ -2687,7 +2687,7 @@
         <v>Cyllage City (Fishing)</v>
       </c>
       <c r="C135" t="str">
-        <v>Skorupi</v>
+        <v>Buizel</v>
       </c>
       <c r="D135" t="str">
         <v>25-30</v>
@@ -2704,7 +2704,7 @@
         <v>Cyllage City (Fishing)</v>
       </c>
       <c r="C136" t="str">
-        <v>Scraggy</v>
+        <v>Aron</v>
       </c>
       <c r="D136" t="str">
         <v>25-30</v>
@@ -2721,7 +2721,7 @@
         <v>Cyllage City (Fishing)</v>
       </c>
       <c r="C137" t="str">
-        <v>Hippowdon</v>
+        <v>Luvdisc</v>
       </c>
       <c r="D137" t="str">
         <v>25-30</v>
@@ -2738,7 +2738,7 @@
         <v>Cyllage City (Fishing)</v>
       </c>
       <c r="C138" t="str">
-        <v>Spoink</v>
+        <v>Zorua</v>
       </c>
       <c r="D138" t="str">
         <v>25-30</v>
@@ -2755,7 +2755,7 @@
         <v>Cyllage City (Fishing)</v>
       </c>
       <c r="C139" t="str">
-        <v>Tentacruel</v>
+        <v>Snover</v>
       </c>
       <c r="D139" t="str">
         <v>25-30</v>
@@ -2772,7 +2772,7 @@
         <v>Route 10</v>
       </c>
       <c r="C140" t="str">
-        <v>Poochyena</v>
+        <v>Pumpkaboo</v>
       </c>
       <c r="D140" t="str">
         <v>23-25</v>
@@ -2789,7 +2789,7 @@
         <v>Route 10</v>
       </c>
       <c r="C141" t="str">
-        <v>Volcanion</v>
+        <v>Tentacool</v>
       </c>
       <c r="D141" t="str">
         <v>23-25</v>
@@ -2806,7 +2806,7 @@
         <v>Route 10</v>
       </c>
       <c r="C142" t="str">
-        <v>Huntail</v>
+        <v>Staravia</v>
       </c>
       <c r="D142" t="str">
         <v>23-25</v>
@@ -2823,7 +2823,7 @@
         <v>Route 10</v>
       </c>
       <c r="C143" t="str">
-        <v>Rhyperior</v>
+        <v>Vibrava</v>
       </c>
       <c r="D143" t="str">
         <v>23-25</v>
@@ -2840,7 +2840,7 @@
         <v>Route 10</v>
       </c>
       <c r="C144" t="str">
-        <v>Delibird</v>
+        <v>Lombre</v>
       </c>
       <c r="D144" t="str">
         <v>23-25</v>
@@ -2857,7 +2857,7 @@
         <v>Route 10</v>
       </c>
       <c r="C145" t="str">
-        <v>Gloom</v>
+        <v>Pawniard</v>
       </c>
       <c r="D145" t="str">
         <v>23-25</v>
@@ -2874,7 +2874,7 @@
         <v>Geosenge Town</v>
       </c>
       <c r="C146" t="str">
-        <v>Zubat</v>
+        <v>Skiploom</v>
       </c>
       <c r="D146" t="str">
         <v>24-26</v>
@@ -2891,7 +2891,7 @@
         <v>Geosenge Town</v>
       </c>
       <c r="C147" t="str">
-        <v>Lapras</v>
+        <v>Staryu</v>
       </c>
       <c r="D147" t="str">
         <v>24-26</v>
@@ -2908,7 +2908,7 @@
         <v>Geosenge Town</v>
       </c>
       <c r="C148" t="str">
-        <v>Pawniard</v>
+        <v>Spritzee</v>
       </c>
       <c r="D148" t="str">
         <v>24-26</v>
@@ -2925,7 +2925,7 @@
         <v>Geosenge Town</v>
       </c>
       <c r="C149" t="str">
-        <v>Vanillite</v>
+        <v>Swirlix</v>
       </c>
       <c r="D149" t="str">
         <v>24-26</v>
@@ -2942,7 +2942,7 @@
         <v>Geosenge Town</v>
       </c>
       <c r="C150" t="str">
-        <v>Yanmega</v>
+        <v>Mantyke</v>
       </c>
       <c r="D150" t="str">
         <v>24-26</v>
@@ -2959,7 +2959,7 @@
         <v>Geosenge Town</v>
       </c>
       <c r="C151" t="str">
-        <v>Zoroark</v>
+        <v>Rhyhorn</v>
       </c>
       <c r="D151" t="str">
         <v>24-26</v>
@@ -2976,7 +2976,7 @@
         <v>Route 11</v>
       </c>
       <c r="C152" t="str">
-        <v>Magcargo</v>
+        <v>Clamperl</v>
       </c>
       <c r="D152" t="str">
         <v>25-27</v>
@@ -2993,7 +2993,7 @@
         <v>Route 11</v>
       </c>
       <c r="C153" t="str">
-        <v>Corsola</v>
+        <v>Scraggy</v>
       </c>
       <c r="D153" t="str">
         <v>25-27</v>
@@ -3010,7 +3010,7 @@
         <v>Route 11</v>
       </c>
       <c r="C154" t="str">
-        <v>Barboach</v>
+        <v>Drifloon</v>
       </c>
       <c r="D154" t="str">
         <v>25-27</v>
@@ -3027,7 +3027,7 @@
         <v>Route 11</v>
       </c>
       <c r="C155" t="str">
-        <v>Minun</v>
+        <v>Pancham</v>
       </c>
       <c r="D155" t="str">
         <v>25-27</v>
@@ -3044,7 +3044,7 @@
         <v>Route 11</v>
       </c>
       <c r="C156" t="str">
-        <v>Mantine</v>
+        <v>Pidgeotto</v>
       </c>
       <c r="D156" t="str">
         <v>25-27</v>
@@ -3061,7 +3061,7 @@
         <v>Route 11</v>
       </c>
       <c r="C157" t="str">
-        <v>Poliwag</v>
+        <v>Mienfoo</v>
       </c>
       <c r="D157" t="str">
         <v>25-27</v>
@@ -3078,7 +3078,7 @@
         <v>Reflection Cave</v>
       </c>
       <c r="C158" t="str">
-        <v>Wailord</v>
+        <v>Skiddo</v>
       </c>
       <c r="D158" t="str">
         <v>30-35</v>
@@ -3095,7 +3095,7 @@
         <v>Reflection Cave</v>
       </c>
       <c r="C159" t="str">
-        <v>Pyroar</v>
+        <v>Krokorok</v>
       </c>
       <c r="D159" t="str">
         <v>30-35</v>
@@ -3112,7 +3112,7 @@
         <v>Reflection Cave</v>
       </c>
       <c r="C160" t="str">
-        <v>Escavalier</v>
+        <v>Espurr</v>
       </c>
       <c r="D160" t="str">
         <v>30-35</v>
@@ -3129,7 +3129,7 @@
         <v>Reflection Cave</v>
       </c>
       <c r="C161" t="str">
-        <v>Avalugg</v>
+        <v>Whirlipede</v>
       </c>
       <c r="D161" t="str">
         <v>30-35</v>
@@ -3146,7 +3146,7 @@
         <v>Reflection Cave</v>
       </c>
       <c r="C162" t="str">
-        <v>Aerodactyl</v>
+        <v>Loudred</v>
       </c>
       <c r="D162" t="str">
         <v>30-35</v>
@@ -3163,7 +3163,7 @@
         <v>Reflection Cave</v>
       </c>
       <c r="C163" t="str">
-        <v>Chimecho</v>
+        <v>Spinda</v>
       </c>
       <c r="D163" t="str">
         <v>30-35</v>
@@ -3180,7 +3180,7 @@
         <v>Shalour City</v>
       </c>
       <c r="C164" t="str">
-        <v>Lanturn</v>
+        <v>Tyrunt</v>
       </c>
       <c r="D164" t="str">
         <v>26-28</v>
@@ -3197,7 +3197,7 @@
         <v>Shalour City</v>
       </c>
       <c r="C165" t="str">
-        <v>Onix</v>
+        <v>Amaura</v>
       </c>
       <c r="D165" t="str">
         <v>26-28</v>
@@ -3214,7 +3214,7 @@
         <v>Shalour City</v>
       </c>
       <c r="C166" t="str">
-        <v>Nidoking</v>
+        <v>Nidorino</v>
       </c>
       <c r="D166" t="str">
         <v>26-28</v>
@@ -3231,7 +3231,7 @@
         <v>Shalour City</v>
       </c>
       <c r="C167" t="str">
-        <v>Shuckle</v>
+        <v>Nidorina</v>
       </c>
       <c r="D167" t="str">
         <v>26-28</v>
@@ -3248,7 +3248,7 @@
         <v>Shalour City</v>
       </c>
       <c r="C168" t="str">
-        <v>Yanma</v>
+        <v>Flaaffy</v>
       </c>
       <c r="D168" t="str">
         <v>26-28</v>
@@ -3265,7 +3265,7 @@
         <v>Shalour City</v>
       </c>
       <c r="C169" t="str">
-        <v>Meditite</v>
+        <v>Litleo</v>
       </c>
       <c r="D169" t="str">
         <v>26-28</v>
@@ -3282,7 +3282,7 @@
         <v>Shalour City Gym</v>
       </c>
       <c r="C170" t="str">
-        <v>Glaceon</v>
+        <v>Duosion</v>
       </c>
       <c r="D170" t="str">
         <v>27-29</v>
@@ -3299,7 +3299,7 @@
         <v>Shalour City Gym</v>
       </c>
       <c r="C171" t="str">
-        <v>Wailmer</v>
+        <v>Lampent</v>
       </c>
       <c r="D171" t="str">
         <v>27-29</v>
@@ -3316,7 +3316,7 @@
         <v>Shalour City Gym</v>
       </c>
       <c r="C172" t="str">
-        <v>Sneasel</v>
+        <v>Floette</v>
       </c>
       <c r="D172" t="str">
         <v>27-29</v>
@@ -3333,7 +3333,7 @@
         <v>Shalour City Gym</v>
       </c>
       <c r="C173" t="str">
-        <v>Stunky</v>
+        <v>Nosepass</v>
       </c>
       <c r="D173" t="str">
         <v>27-29</v>
@@ -3350,7 +3350,7 @@
         <v>Shalour City Gym</v>
       </c>
       <c r="C174" t="str">
-        <v>Timburr</v>
+        <v>Sableye</v>
       </c>
       <c r="D174" t="str">
         <v>27-29</v>
@@ -3367,7 +3367,7 @@
         <v>Shalour City Gym</v>
       </c>
       <c r="C175" t="str">
-        <v>Articuno</v>
+        <v>Mawile</v>
       </c>
       <c r="D175" t="str">
         <v>27-29</v>
@@ -3384,7 +3384,7 @@
         <v>Tower of Mastery</v>
       </c>
       <c r="C176" t="str">
-        <v>Kangaskhan</v>
+        <v>Fletchinder</v>
       </c>
       <c r="D176" t="str">
         <v>35-40</v>
@@ -3401,7 +3401,7 @@
         <v>Tower of Mastery</v>
       </c>
       <c r="C177" t="str">
-        <v>Haxorus</v>
+        <v>Poliwhirl</v>
       </c>
       <c r="D177" t="str">
         <v>35-40</v>
@@ -3418,7 +3418,7 @@
         <v>Tower of Mastery</v>
       </c>
       <c r="C178" t="str">
-        <v>Jumpluff</v>
+        <v>Onix</v>
       </c>
       <c r="D178" t="str">
         <v>35-40</v>
@@ -3435,7 +3435,7 @@
         <v>Tower of Mastery</v>
       </c>
       <c r="C179" t="str">
-        <v>Spewpa</v>
+        <v>Lickitung</v>
       </c>
       <c r="D179" t="str">
         <v>35-40</v>
@@ -3452,7 +3452,7 @@
         <v>Tower of Mastery</v>
       </c>
       <c r="C180" t="str">
-        <v>Doublade</v>
+        <v>Boldore</v>
       </c>
       <c r="D180" t="str">
         <v>35-40</v>
@@ -3469,7 +3469,7 @@
         <v>Tower of Mastery</v>
       </c>
       <c r="C181" t="str">
-        <v>Raichu</v>
+        <v>Yanma</v>
       </c>
       <c r="D181" t="str">
         <v>35-40</v>
@@ -3486,7 +3486,7 @@
         <v>Route 12</v>
       </c>
       <c r="C182" t="str">
-        <v>Pumpkaboo</v>
+        <v>Graveler</v>
       </c>
       <c r="D182" t="str">
         <v>28-30</v>
@@ -3503,7 +3503,7 @@
         <v>Route 12</v>
       </c>
       <c r="C183" t="str">
-        <v>Butterfree</v>
+        <v>Gothorita</v>
       </c>
       <c r="D183" t="str">
         <v>28-30</v>
@@ -3520,7 +3520,7 @@
         <v>Route 12</v>
       </c>
       <c r="C184" t="str">
-        <v>Magneton</v>
+        <v>Munchlax</v>
       </c>
       <c r="D184" t="str">
         <v>28-30</v>
@@ -3537,7 +3537,7 @@
         <v>Route 12</v>
       </c>
       <c r="C185" t="str">
-        <v>Vanillish</v>
+        <v>Ledian</v>
       </c>
       <c r="D185" t="str">
         <v>28-30</v>
@@ -3554,7 +3554,7 @@
         <v>Route 12</v>
       </c>
       <c r="C186" t="str">
-        <v>Sliggoo</v>
+        <v>Beedrill</v>
       </c>
       <c r="D186" t="str">
         <v>28-30</v>
@@ -3571,7 +3571,7 @@
         <v>Route 12</v>
       </c>
       <c r="C187" t="str">
-        <v>Bergmite</v>
+        <v>Gloom</v>
       </c>
       <c r="D187" t="str">
         <v>28-30</v>
@@ -3588,7 +3588,7 @@
         <v>Azure Bay</v>
       </c>
       <c r="C188" t="str">
-        <v>Furfrou</v>
+        <v>Butterfree</v>
       </c>
       <c r="D188" t="str">
         <v>29-32</v>
@@ -3605,7 +3605,7 @@
         <v>Azure Bay</v>
       </c>
       <c r="C189" t="str">
-        <v>Nidoran-m</v>
+        <v>Vanillish</v>
       </c>
       <c r="D189" t="str">
         <v>29-32</v>
@@ -3622,7 +3622,7 @@
         <v>Azure Bay</v>
       </c>
       <c r="C190" t="str">
-        <v>Murkrow</v>
+        <v>Kadabra</v>
       </c>
       <c r="D190" t="str">
         <v>29-32</v>
@@ -3639,7 +3639,7 @@
         <v>Azure Bay</v>
       </c>
       <c r="C191" t="str">
-        <v>Electrode</v>
+        <v>Wailmer</v>
       </c>
       <c r="D191" t="str">
         <v>29-32</v>
@@ -3656,7 +3656,7 @@
         <v>Azure Bay</v>
       </c>
       <c r="C192" t="str">
-        <v>Farfetchd</v>
+        <v>Ariados</v>
       </c>
       <c r="D192" t="str">
         <v>29-32</v>
@@ -3673,7 +3673,7 @@
         <v>Azure Bay</v>
       </c>
       <c r="C193" t="str">
-        <v>Taillow</v>
+        <v>Pachirisu</v>
       </c>
       <c r="D193" t="str">
         <v>29-32</v>
@@ -3690,7 +3690,7 @@
         <v>Azure Bay (Fishing)</v>
       </c>
       <c r="C194" t="str">
-        <v>Ducklett</v>
+        <v>Plusle</v>
       </c>
       <c r="D194" t="str">
         <v>30-33</v>
@@ -3707,7 +3707,7 @@
         <v>Azure Bay (Fishing)</v>
       </c>
       <c r="C195" t="str">
-        <v>Tyranitar</v>
+        <v>Machoke</v>
       </c>
       <c r="D195" t="str">
         <v>30-33</v>
@@ -3724,7 +3724,7 @@
         <v>Azure Bay (Fishing)</v>
       </c>
       <c r="C196" t="str">
-        <v>Gulpin</v>
+        <v>Gurdurr</v>
       </c>
       <c r="D196" t="str">
         <v>30-33</v>
@@ -3741,7 +3741,7 @@
         <v>Azure Bay (Fishing)</v>
       </c>
       <c r="C197" t="str">
-        <v>Swellow</v>
+        <v>Minun</v>
       </c>
       <c r="D197" t="str">
         <v>30-33</v>
@@ -3758,7 +3758,7 @@
         <v>Azure Bay (Fishing)</v>
       </c>
       <c r="C198" t="str">
-        <v>Skarmory</v>
+        <v>Murkrow</v>
       </c>
       <c r="D198" t="str">
         <v>30-33</v>
@@ -3775,7 +3775,7 @@
         <v>Coumarine City</v>
       </c>
       <c r="C199" t="str">
-        <v>Wormadam</v>
+        <v>Wobbuffet</v>
       </c>
       <c r="D199" t="str">
         <v>40-45</v>
@@ -3792,7 +3792,7 @@
         <v>Coumarine City</v>
       </c>
       <c r="C200" t="str">
-        <v>Quagsire</v>
+        <v>Haunter</v>
       </c>
       <c r="D200" t="str">
         <v>40-45</v>
@@ -3809,7 +3809,7 @@
         <v>Coumarine City</v>
       </c>
       <c r="C201" t="str">
-        <v>Crustle</v>
+        <v>Fraxure</v>
       </c>
       <c r="D201" t="str">
         <v>40-45</v>
@@ -3826,7 +3826,7 @@
         <v>Coumarine City</v>
       </c>
       <c r="C202" t="str">
-        <v>Graveler</v>
+        <v>Pupitar</v>
       </c>
       <c r="D202" t="str">
         <v>40-45</v>
@@ -3843,7 +3843,7 @@
         <v>Coumarine City</v>
       </c>
       <c r="C203" t="str">
-        <v>Venusaur</v>
+        <v>Corsola</v>
       </c>
       <c r="D203" t="str">
         <v>40-45</v>
@@ -3860,7 +3860,7 @@
         <v>Coumarine City Gym</v>
       </c>
       <c r="C204" t="str">
-        <v>Machop</v>
+        <v>Sudowoodo</v>
       </c>
       <c r="D204" t="str">
         <v>31-34</v>
@@ -3877,7 +3877,7 @@
         <v>Coumarine City Gym</v>
       </c>
       <c r="C205" t="str">
-        <v>Sudowoodo</v>
+        <v>Medicham</v>
       </c>
       <c r="D205" t="str">
         <v>31-34</v>
@@ -3894,7 +3894,7 @@
         <v>Coumarine City Gym</v>
       </c>
       <c r="C206" t="str">
-        <v>Budew</v>
+        <v>Bibarel</v>
       </c>
       <c r="D206" t="str">
         <v>31-34</v>
@@ -3911,7 +3911,7 @@
         <v>Coumarine City Gym</v>
       </c>
       <c r="C207" t="str">
-        <v>Granbull</v>
+        <v>Gabite</v>
       </c>
       <c r="D207" t="str">
         <v>31-34</v>
@@ -3928,7 +3928,7 @@
         <v>Coumarine City Gym</v>
       </c>
       <c r="C208" t="str">
-        <v>Noibat</v>
+        <v>Furret</v>
       </c>
       <c r="D208" t="str">
         <v>31-34</v>
@@ -3945,7 +3945,7 @@
         <v>Coumarine City (Fishing)</v>
       </c>
       <c r="C209" t="str">
-        <v>Ekans</v>
+        <v>Dunsparce</v>
       </c>
       <c r="D209" t="str">
         <v>33-35</v>
@@ -3962,7 +3962,7 @@
         <v>Coumarine City (Fishing)</v>
       </c>
       <c r="C210" t="str">
-        <v>Gardevoir</v>
+        <v>Linoone</v>
       </c>
       <c r="D210" t="str">
         <v>33-35</v>
@@ -3979,7 +3979,7 @@
         <v>Coumarine City (Fishing)</v>
       </c>
       <c r="C211" t="str">
-        <v>Gothorita</v>
+        <v>Shelgon</v>
       </c>
       <c r="D211" t="str">
         <v>33-35</v>
@@ -3996,7 +3996,7 @@
         <v>Coumarine City (Fishing)</v>
       </c>
       <c r="C212" t="str">
-        <v>Sigilyph</v>
+        <v>Dragonair</v>
       </c>
       <c r="D212" t="str">
         <v>33-35</v>
@@ -4013,7 +4013,7 @@
         <v>Coumarine City (Fishing)</v>
       </c>
       <c r="C213" t="str">
-        <v>Foongus</v>
+        <v>Azumarill</v>
       </c>
       <c r="D213" t="str">
         <v>33-35</v>
@@ -4030,7 +4030,7 @@
         <v>Route 13</v>
       </c>
       <c r="C214" t="str">
-        <v>Medicham</v>
+        <v>Wormadam</v>
       </c>
       <c r="D214" t="str">
         <v>34-36</v>
@@ -4047,7 +4047,7 @@
         <v>Route 13</v>
       </c>
       <c r="C215" t="str">
-        <v>Piloswine</v>
+        <v>Mothim</v>
       </c>
       <c r="D215" t="str">
         <v>34-36</v>
@@ -4064,7 +4064,7 @@
         <v>Route 13</v>
       </c>
       <c r="C216" t="str">
-        <v>Roserade</v>
+        <v>Dugtrio</v>
       </c>
       <c r="D216" t="str">
         <v>34-36</v>
@@ -4081,7 +4081,7 @@
         <v>Route 13</v>
       </c>
       <c r="C217" t="str">
-        <v>Teddiursa</v>
+        <v>Marowak</v>
       </c>
       <c r="D217" t="str">
         <v>34-36</v>
@@ -4098,7 +4098,7 @@
         <v>Route 13</v>
       </c>
       <c r="C218" t="str">
-        <v>Garbodor</v>
+        <v>Swoobat</v>
       </c>
       <c r="D218" t="str">
         <v>34-36</v>
@@ -4115,7 +4115,7 @@
         <v>Lumiose City (North)</v>
       </c>
       <c r="C219" t="str">
-        <v>Bellsprout</v>
+        <v>Emolga</v>
       </c>
       <c r="D219" t="str">
         <v>35-37</v>
@@ -4132,7 +4132,7 @@
         <v>Lumiose City (North)</v>
       </c>
       <c r="C220" t="str">
-        <v>Hydreigon</v>
+        <v>Lairon</v>
       </c>
       <c r="D220" t="str">
         <v>35-37</v>
@@ -4149,7 +4149,7 @@
         <v>Lumiose City (North)</v>
       </c>
       <c r="C221" t="str">
-        <v>Exeggcute</v>
+        <v>Volbeat</v>
       </c>
       <c r="D221" t="str">
         <v>35-37</v>
@@ -4166,7 +4166,7 @@
         <v>Lumiose City (North)</v>
       </c>
       <c r="C222" t="str">
-        <v>Skitty</v>
+        <v>Magcargo</v>
       </c>
       <c r="D222" t="str">
         <v>35-37</v>
@@ -4183,7 +4183,7 @@
         <v>Lumiose City (North)</v>
       </c>
       <c r="C223" t="str">
-        <v>Sawk</v>
+        <v>Sneasel</v>
       </c>
       <c r="D223" t="str">
         <v>35-37</v>
@@ -4200,7 +4200,7 @@
         <v>Lumiose City Gym</v>
       </c>
       <c r="C224" t="str">
-        <v>Chingling</v>
+        <v>Quagsire</v>
       </c>
       <c r="D224" t="str">
         <v>36-39</v>
@@ -4217,7 +4217,7 @@
         <v>Lumiose City Gym</v>
       </c>
       <c r="C225" t="str">
-        <v>Exploud</v>
+        <v>Gligar</v>
       </c>
       <c r="D225" t="str">
         <v>36-39</v>
@@ -4234,7 +4234,7 @@
         <v>Lumiose City Gym</v>
       </c>
       <c r="C226" t="str">
-        <v>Inkay</v>
+        <v>Illumise</v>
       </c>
       <c r="D226" t="str">
         <v>36-39</v>
@@ -4251,7 +4251,7 @@
         <v>Lumiose City Gym</v>
       </c>
       <c r="C227" t="str">
-        <v>Skiddo</v>
+        <v>Dedenne</v>
       </c>
       <c r="D227" t="str">
         <v>36-39</v>
@@ -4268,7 +4268,7 @@
         <v>Lumiose City Gym</v>
       </c>
       <c r="C228" t="str">
-        <v>Gastly</v>
+        <v>Wigglytuff</v>
       </c>
       <c r="D228" t="str">
         <v>36-39</v>
@@ -4285,7 +4285,7 @@
         <v>Route 14</v>
       </c>
       <c r="C229" t="str">
-        <v>Umbreon</v>
+        <v>Seadra</v>
       </c>
       <c r="D229" t="str">
         <v>37-40</v>
@@ -4302,7 +4302,7 @@
         <v>Route 14</v>
       </c>
       <c r="C230" t="str">
-        <v>Trapinch</v>
+        <v>Rotom</v>
       </c>
       <c r="D230" t="str">
         <v>37-40</v>
@@ -4319,7 +4319,7 @@
         <v>Route 14</v>
       </c>
       <c r="C231" t="str">
-        <v>Gorebyss</v>
+        <v>Kecleon</v>
       </c>
       <c r="D231" t="str">
         <v>37-40</v>
@@ -4336,7 +4336,7 @@
         <v>Route 14</v>
       </c>
       <c r="C232" t="str">
-        <v>Tauros</v>
+        <v>Qwilfish</v>
       </c>
       <c r="D232" t="str">
         <v>37-40</v>
@@ -4353,7 +4353,7 @@
         <v>Route 14</v>
       </c>
       <c r="C233" t="str">
-        <v>Flabebe</v>
+        <v>Audino</v>
       </c>
       <c r="D233" t="str">
         <v>37-40</v>
@@ -4370,7 +4370,7 @@
         <v>Laverre City</v>
       </c>
       <c r="C234" t="str">
-        <v>Shelgon</v>
+        <v>Liepard</v>
       </c>
       <c r="D234" t="str">
         <v>38-41</v>
@@ -4387,7 +4387,7 @@
         <v>Laverre City</v>
       </c>
       <c r="C235" t="str">
-        <v>Wobbuffet</v>
+        <v>Doublade</v>
       </c>
       <c r="D235" t="str">
         <v>38-41</v>
@@ -4404,7 +4404,7 @@
         <v>Laverre City</v>
       </c>
       <c r="C236" t="str">
-        <v>Loudred</v>
+        <v>Sandslash</v>
       </c>
       <c r="D236" t="str">
         <v>38-41</v>
@@ -4421,7 +4421,7 @@
         <v>Laverre City</v>
       </c>
       <c r="C237" t="str">
-        <v>Bonsly</v>
+        <v>Granbull</v>
       </c>
       <c r="D237" t="str">
         <v>38-41</v>
@@ -4438,7 +4438,7 @@
         <v>Laverre City</v>
       </c>
       <c r="C238" t="str">
-        <v>Nosepass</v>
+        <v>Piloswine</v>
       </c>
       <c r="D238" t="str">
         <v>38-41</v>
@@ -4455,7 +4455,7 @@
         <v>Laverre City Gym</v>
       </c>
       <c r="C239" t="str">
-        <v>Rhydon</v>
+        <v>Seaking</v>
       </c>
       <c r="D239" t="str">
         <v>39-42</v>
@@ -4472,7 +4472,7 @@
         <v>Laverre City Gym</v>
       </c>
       <c r="C240" t="str">
-        <v>Staraptor</v>
+        <v>Sliggoo</v>
       </c>
       <c r="D240" t="str">
         <v>39-42</v>
@@ -4489,7 +4489,7 @@
         <v>Laverre City Gym</v>
       </c>
       <c r="C241" t="str">
-        <v>Goomy</v>
+        <v>Noctowl</v>
       </c>
       <c r="D241" t="str">
         <v>39-42</v>
@@ -4506,7 +4506,7 @@
         <v>Laverre City Gym</v>
       </c>
       <c r="C242" t="str">
-        <v>Torkoal</v>
+        <v>Carnivine</v>
       </c>
       <c r="D242" t="str">
         <v>39-42</v>
@@ -4523,7 +4523,7 @@
         <v>Laverre City Gym</v>
       </c>
       <c r="C243" t="str">
-        <v>Florges</v>
+        <v>Masquerain</v>
       </c>
       <c r="D243" t="str">
         <v>39-42</v>
@@ -4540,7 +4540,7 @@
         <v>Route 15</v>
       </c>
       <c r="C244" t="str">
-        <v>Golbat</v>
+        <v>Jynx</v>
       </c>
       <c r="D244" t="str">
         <v>40-43</v>
@@ -4557,7 +4557,7 @@
         <v>Route 15</v>
       </c>
       <c r="C245" t="str">
-        <v>Drifloon</v>
+        <v>Chimecho</v>
       </c>
       <c r="D245" t="str">
         <v>40-43</v>
@@ -4574,7 +4574,7 @@
         <v>Route 15</v>
       </c>
       <c r="C246" t="str">
-        <v>Dwebble</v>
+        <v>Swellow</v>
       </c>
       <c r="D246" t="str">
         <v>40-43</v>
@@ -4591,7 +4591,7 @@
         <v>Route 15</v>
       </c>
       <c r="C247" t="str">
-        <v>Zapdos</v>
+        <v>Golbat</v>
       </c>
       <c r="D247" t="str">
         <v>40-43</v>
@@ -4608,7 +4608,7 @@
         <v>Route 15</v>
       </c>
       <c r="C248" t="str">
-        <v>Conkeldurr</v>
+        <v>Banette</v>
       </c>
       <c r="D248" t="str">
         <v>40-43</v>
@@ -4625,7 +4625,7 @@
         <v>Lost Hotel</v>
       </c>
       <c r="C249" t="str">
-        <v>Dragonair</v>
+        <v>Ninjask</v>
       </c>
       <c r="D249" t="str">
         <v>41-44</v>
@@ -4642,7 +4642,7 @@
         <v>Lost Hotel</v>
       </c>
       <c r="C250" t="str">
-        <v>Noctowl</v>
+        <v>Zangoose</v>
       </c>
       <c r="D250" t="str">
         <v>41-44</v>
@@ -4659,7 +4659,7 @@
         <v>Lost Hotel</v>
       </c>
       <c r="C251" t="str">
-        <v>Gligar</v>
+        <v>Seviper</v>
       </c>
       <c r="D251" t="str">
         <v>41-44</v>
@@ -4676,7 +4676,7 @@
         <v>Lost Hotel</v>
       </c>
       <c r="C252" t="str">
-        <v>Lampent</v>
+        <v>Sharpedo</v>
       </c>
       <c r="D252" t="str">
         <v>41-44</v>
@@ -4693,7 +4693,7 @@
         <v>Lost Hotel</v>
       </c>
       <c r="C253" t="str">
-        <v>Ditto</v>
+        <v>Basculin</v>
       </c>
       <c r="D253" t="str">
         <v>41-44</v>
@@ -4710,7 +4710,7 @@
         <v>Dendemille Town</v>
       </c>
       <c r="C254" t="str">
-        <v>Relicanth</v>
+        <v>Lunatone</v>
       </c>
       <c r="D254" t="str">
         <v>42-45</v>
@@ -4727,7 +4727,7 @@
         <v>Dendemille Town</v>
       </c>
       <c r="C255" t="str">
-        <v>Gothita</v>
+        <v>Lanturn</v>
       </c>
       <c r="D255" t="str">
         <v>42-45</v>
@@ -4744,7 +4744,7 @@
         <v>Dendemille Town</v>
       </c>
       <c r="C256" t="str">
-        <v>Munchlax</v>
+        <v>Jumpluff</v>
       </c>
       <c r="D256" t="str">
         <v>42-45</v>
@@ -4761,7 +4761,7 @@
         <v>Dendemille Town</v>
       </c>
       <c r="C257" t="str">
-        <v>Gliscor</v>
+        <v>Solrock</v>
       </c>
       <c r="D257" t="str">
         <v>42-45</v>
@@ -4778,7 +4778,7 @@
         <v>Dendemille Town</v>
       </c>
       <c r="C258" t="str">
-        <v>Kakuna</v>
+        <v>Aromatisse</v>
       </c>
       <c r="D258" t="str">
         <v>42-45</v>
@@ -4795,7 +4795,7 @@
         <v>Route 16</v>
       </c>
       <c r="C259" t="str">
-        <v>Patrat</v>
+        <v>Throh</v>
       </c>
       <c r="D259" t="str">
         <v>43-47</v>
@@ -4812,7 +4812,7 @@
         <v>Route 16</v>
       </c>
       <c r="C260" t="str">
-        <v>Dugtrio</v>
+        <v>Magneton</v>
       </c>
       <c r="D260" t="str">
         <v>43-47</v>
@@ -4829,7 +4829,7 @@
         <v>Route 16</v>
       </c>
       <c r="C261" t="str">
-        <v>Hippopotas</v>
+        <v>Skarmory</v>
       </c>
       <c r="D261" t="str">
         <v>43-47</v>
@@ -4846,7 +4846,7 @@
         <v>Route 16</v>
       </c>
       <c r="C262" t="str">
-        <v>Ursaring</v>
+        <v>Sawk</v>
       </c>
       <c r="D262" t="str">
         <v>43-47</v>
@@ -4863,7 +4863,7 @@
         <v>Route 16</v>
       </c>
       <c r="C263" t="str">
-        <v>Spinda</v>
+        <v>Absol</v>
       </c>
       <c r="D263" t="str">
         <v>43-47</v>
@@ -4880,7 +4880,7 @@
         <v>Frost Cavern</v>
       </c>
       <c r="C264" t="str">
-        <v>Floatzel</v>
+        <v>Swalot</v>
       </c>
       <c r="D264" t="str">
         <v>44-48</v>
@@ -4897,7 +4897,7 @@
         <v>Frost Cavern</v>
       </c>
       <c r="C265" t="str">
-        <v>Marowak</v>
+        <v>Crawdaunt</v>
       </c>
       <c r="D265" t="str">
         <v>44-48</v>
@@ -4914,7 +4914,7 @@
         <v>Frost Cavern</v>
       </c>
       <c r="C266" t="str">
-        <v>Mareep</v>
+        <v>Whiscash</v>
       </c>
       <c r="D266" t="str">
         <v>44-48</v>
@@ -4931,7 +4931,7 @@
         <v>Frost Cavern</v>
       </c>
       <c r="C267" t="str">
-        <v>Spearow</v>
+        <v>Grumpig</v>
       </c>
       <c r="D267" t="str">
         <v>44-48</v>
@@ -4948,7 +4948,7 @@
         <v>Frost Cavern</v>
       </c>
       <c r="C268" t="str">
-        <v>Weavile</v>
+        <v>Klefki</v>
       </c>
       <c r="D268" t="str">
         <v>44-48</v>
@@ -4965,7 +4965,7 @@
         <v>Anistar City</v>
       </c>
       <c r="C269" t="str">
-        <v>Swablu</v>
+        <v>Torkoal</v>
       </c>
       <c r="D269" t="str">
         <v>45-49</v>
@@ -4982,7 +4982,7 @@
         <v>Anistar City</v>
       </c>
       <c r="C270" t="str">
-        <v>Clauncher</v>
+        <v>Stunfisk</v>
       </c>
       <c r="D270" t="str">
         <v>45-49</v>
@@ -4999,7 +4999,7 @@
         <v>Anistar City</v>
       </c>
       <c r="C271" t="str">
-        <v>Crawdaunt</v>
+        <v>Furfrou</v>
       </c>
       <c r="D271" t="str">
         <v>45-49</v>
@@ -5016,7 +5016,7 @@
         <v>Anistar City</v>
       </c>
       <c r="C272" t="str">
-        <v>Skiploom</v>
+        <v>Swanna</v>
       </c>
       <c r="D272" t="str">
         <v>45-49</v>
@@ -5033,7 +5033,7 @@
         <v>Anistar City</v>
       </c>
       <c r="C273" t="str">
-        <v>Greninja</v>
+        <v>Hariyama</v>
       </c>
       <c r="D273" t="str">
         <v>45-49</v>
@@ -5050,7 +5050,7 @@
         <v>Anistar City Gym</v>
       </c>
       <c r="C274" t="str">
-        <v>Moltres</v>
+        <v>Garbodor</v>
       </c>
       <c r="D274" t="str">
         <v>46-50</v>
@@ -5067,7 +5067,7 @@
         <v>Anistar City Gym</v>
       </c>
       <c r="C275" t="str">
-        <v>Pansear</v>
+        <v>Vespiquen</v>
       </c>
       <c r="D275" t="str">
         <v>46-50</v>
@@ -5084,7 +5084,7 @@
         <v>Anistar City Gym</v>
       </c>
       <c r="C276" t="str">
-        <v>Audino</v>
+        <v>Manectric</v>
       </c>
       <c r="D276" t="str">
         <v>46-50</v>
@@ -5101,7 +5101,7 @@
         <v>Anistar City Gym</v>
       </c>
       <c r="C277" t="str">
-        <v>Flaaffy</v>
+        <v>Skuntank</v>
       </c>
       <c r="D277" t="str">
         <v>46-50</v>
@@ -5118,7 +5118,7 @@
         <v>Anistar City Gym</v>
       </c>
       <c r="C278" t="str">
-        <v>Durant</v>
+        <v>Pidgeot</v>
       </c>
       <c r="D278" t="str">
         <v>46-50</v>
@@ -5135,7 +5135,7 @@
         <v>Route 17</v>
       </c>
       <c r="C279" t="str">
-        <v>Metapod</v>
+        <v>Slurpuff</v>
       </c>
       <c r="D279" t="str">
         <v>47-51</v>
@@ -5152,7 +5152,7 @@
         <v>Route 17</v>
       </c>
       <c r="C280" t="str">
-        <v>Whiscash</v>
+        <v>Octillery</v>
       </c>
       <c r="D280" t="str">
         <v>47-51</v>
@@ -5169,7 +5169,7 @@
         <v>Route 17</v>
       </c>
       <c r="C281" t="str">
-        <v>Lotad</v>
+        <v>Malamar</v>
       </c>
       <c r="D281" t="str">
         <v>47-51</v>
@@ -5186,7 +5186,7 @@
         <v>Route 17</v>
       </c>
       <c r="C282" t="str">
-        <v>Caterpie</v>
+        <v>Golurk</v>
       </c>
       <c r="D282" t="str">
         <v>47-51</v>
@@ -5203,7 +5203,7 @@
         <v>Route 17</v>
       </c>
       <c r="C283" t="str">
-        <v>Gigalith</v>
+        <v>Durant</v>
       </c>
       <c r="D283" t="str">
         <v>47-51</v>
@@ -5220,7 +5220,7 @@
         <v>Couriway Town</v>
       </c>
       <c r="C284" t="str">
-        <v>Pidgeot</v>
+        <v>Heatmor</v>
       </c>
       <c r="D284" t="str">
         <v>49-52</v>
@@ -5237,7 +5237,7 @@
         <v>Couriway Town</v>
       </c>
       <c r="C285" t="str">
-        <v>Golett</v>
+        <v>Scolipede</v>
       </c>
       <c r="D285" t="str">
         <v>49-52</v>
@@ -5254,7 +5254,7 @@
         <v>Couriway Town</v>
       </c>
       <c r="C286" t="str">
-        <v>Vespiquen</v>
+        <v>Huntail</v>
       </c>
       <c r="D286" t="str">
         <v>49-52</v>
@@ -5271,7 +5271,7 @@
         <v>Couriway Town</v>
       </c>
       <c r="C287" t="str">
-        <v>Pidgey</v>
+        <v>Mantine</v>
       </c>
       <c r="D287" t="str">
         <v>49-52</v>
@@ -5288,7 +5288,7 @@
         <v>Couriway Town</v>
       </c>
       <c r="C288" t="str">
-        <v>Liepard</v>
+        <v>Raichu</v>
       </c>
       <c r="D288" t="str">
         <v>49-52</v>
@@ -5305,7 +5305,7 @@
         <v>Route 18</v>
       </c>
       <c r="C289" t="str">
-        <v>Bibarel</v>
+        <v>Crustle</v>
       </c>
       <c r="D289" t="str">
         <v>50-53</v>
@@ -5322,7 +5322,7 @@
         <v>Route 18</v>
       </c>
       <c r="C290" t="str">
-        <v>Banette</v>
+        <v>Gorebyss</v>
       </c>
       <c r="D290" t="str">
         <v>50-53</v>
@@ -5339,7 +5339,7 @@
         <v>Route 18</v>
       </c>
       <c r="C291" t="str">
-        <v>Dratini</v>
+        <v>Rhydon</v>
       </c>
       <c r="D291" t="str">
         <v>50-53</v>
@@ -5356,7 +5356,7 @@
         <v>Route 18</v>
       </c>
       <c r="C292" t="str">
-        <v>Haunter</v>
+        <v>Staraptor</v>
       </c>
       <c r="D292" t="str">
         <v>50-53</v>
@@ -5373,7 +5373,7 @@
         <v>Route 18</v>
       </c>
       <c r="C293" t="str">
-        <v>Ledian</v>
+        <v>Relicanth</v>
       </c>
       <c r="D293" t="str">
         <v>50-53</v>
@@ -5390,7 +5390,7 @@
         <v>Terminus Cave (Surface)</v>
       </c>
       <c r="C294" t="str">
-        <v>Azumarill</v>
+        <v>Druddigon</v>
       </c>
       <c r="D294" t="str">
         <v>51-55</v>
@@ -5407,7 +5407,7 @@
         <v>Terminus Cave (Surface)</v>
       </c>
       <c r="C295" t="str">
-        <v>Seaking</v>
+        <v>Scrafty</v>
       </c>
       <c r="D295" t="str">
         <v>51-55</v>
@@ -5424,7 +5424,7 @@
         <v>Terminus Cave (Surface)</v>
       </c>
       <c r="C296" t="str">
-        <v>Scatterbug</v>
+        <v>Ferrothorn</v>
       </c>
       <c r="D296" t="str">
         <v>51-55</v>
@@ -5441,7 +5441,7 @@
         <v>Terminus Cave (Surface)</v>
       </c>
       <c r="C297" t="str">
-        <v>Fletchling</v>
+        <v>Miltank</v>
       </c>
       <c r="D297" t="str">
         <v>51-55</v>
@@ -5458,7 +5458,7 @@
         <v>Terminus Cave (Surface)</v>
       </c>
       <c r="C298" t="str">
-        <v>Remoraid</v>
+        <v>Bellossom</v>
       </c>
       <c r="D298" t="str">
         <v>51-55</v>
@@ -5475,7 +5475,7 @@
         <v>Route 19</v>
       </c>
       <c r="C299" t="str">
-        <v>Seviper</v>
+        <v>Slowbro</v>
       </c>
       <c r="D299" t="str">
         <v>52-56</v>
@@ -5492,7 +5492,7 @@
         <v>Route 19</v>
       </c>
       <c r="C300" t="str">
-        <v>Buizel</v>
+        <v>Vileplume</v>
       </c>
       <c r="D300" t="str">
         <v>52-56</v>
@@ -5509,7 +5509,7 @@
         <v>Route 19</v>
       </c>
       <c r="C301" t="str">
-        <v>Snover</v>
+        <v>Bisharp</v>
       </c>
       <c r="D301" t="str">
         <v>52-56</v>
@@ -5526,7 +5526,7 @@
         <v>Route 19</v>
       </c>
       <c r="C302" t="str">
-        <v>Aron</v>
+        <v>Kangaskhan</v>
       </c>
       <c r="D302" t="str">
         <v>52-56</v>
@@ -5543,7 +5543,7 @@
         <v>Route 19</v>
       </c>
       <c r="C303" t="str">
-        <v>Pichu</v>
+        <v>Electrode</v>
       </c>
       <c r="D303" t="str">
         <v>52-56</v>
@@ -5560,7 +5560,7 @@
         <v>Route 19 (Fishing)</v>
       </c>
       <c r="C304" t="str">
-        <v>Ralts</v>
+        <v>Sigilyph</v>
       </c>
       <c r="D304" t="str">
         <v>53-57</v>
@@ -5577,7 +5577,7 @@
         <v>Route 19 (Fishing)</v>
       </c>
       <c r="C305" t="str">
-        <v>Heatmor</v>
+        <v>Exploud</v>
       </c>
       <c r="D305" t="str">
         <v>53-57</v>
@@ -5594,7 +5594,7 @@
         <v>Route 19 (Fishing)</v>
       </c>
       <c r="C306" t="str">
-        <v>Shellder</v>
+        <v>Tauros</v>
       </c>
       <c r="D306" t="str">
         <v>53-57</v>
@@ -5611,7 +5611,7 @@
         <v>Route 19 (Fishing)</v>
       </c>
       <c r="C307" t="str">
-        <v>Gabite</v>
+        <v>Toxicroak</v>
       </c>
       <c r="D307" t="str">
         <v>53-57</v>
@@ -5628,7 +5628,7 @@
         <v>Route 19 (Fishing)</v>
       </c>
       <c r="C308" t="str">
-        <v>Aurorus</v>
+        <v>Altaria</v>
       </c>
       <c r="D308" t="str">
         <v>53-57</v>
@@ -5645,7 +5645,7 @@
         <v>Snowbelle City</v>
       </c>
       <c r="C309" t="str">
-        <v>Emolga</v>
+        <v>Gothitelle</v>
       </c>
       <c r="D309" t="str">
         <v>54-58</v>
@@ -5662,7 +5662,7 @@
         <v>Snowbelle City</v>
       </c>
       <c r="C310" t="str">
-        <v>Masquerain</v>
+        <v>Reuniclus</v>
       </c>
       <c r="D310" t="str">
         <v>54-58</v>
@@ -5679,7 +5679,7 @@
         <v>Snowbelle City</v>
       </c>
       <c r="C311" t="str">
-        <v>Noivern</v>
+        <v>Dragalge</v>
       </c>
       <c r="D311" t="str">
         <v>54-58</v>
@@ -5696,7 +5696,7 @@
         <v>Snowbelle City</v>
       </c>
       <c r="C312" t="str">
-        <v>Binacle</v>
+        <v>Gourgeist</v>
       </c>
       <c r="D312" t="str">
         <v>54-58</v>
@@ -5713,7 +5713,7 @@
         <v>Snowbelle City</v>
       </c>
       <c r="C313" t="str">
-        <v>Swoobat</v>
+        <v>Escavalier</v>
       </c>
       <c r="D313" t="str">
         <v>54-58</v>
@@ -5730,7 +5730,7 @@
         <v>Snowbelle City Gym</v>
       </c>
       <c r="C314" t="str">
-        <v>Luvdisc</v>
+        <v>Floatzel</v>
       </c>
       <c r="D314" t="str">
         <v>55-59</v>
@@ -5747,7 +5747,7 @@
         <v>Snowbelle City Gym</v>
       </c>
       <c r="C315" t="str">
-        <v>Ariados</v>
+        <v>Simisage</v>
       </c>
       <c r="D315" t="str">
         <v>55-59</v>
@@ -5764,7 +5764,7 @@
         <v>Snowbelle City Gym</v>
       </c>
       <c r="C316" t="str">
-        <v>Venipede</v>
+        <v>Drifblim</v>
       </c>
       <c r="D316" t="str">
         <v>55-59</v>
@@ -5781,7 +5781,7 @@
         <v>Snowbelle City Gym</v>
       </c>
       <c r="C317" t="str">
-        <v>Clamperl</v>
+        <v>Simipour</v>
       </c>
       <c r="D317" t="str">
         <v>55-59</v>
@@ -5798,7 +5798,7 @@
         <v>Snowbelle City Gym</v>
       </c>
       <c r="C318" t="str">
-        <v>Mime-jr</v>
+        <v>Talonflame</v>
       </c>
       <c r="D318" t="str">
         <v>55-59</v>
@@ -5815,7 +5815,7 @@
         <v>Route 20</v>
       </c>
       <c r="C319" t="str">
-        <v>Toxicroak</v>
+        <v>Clawitzer</v>
       </c>
       <c r="D319" t="str">
         <v>56-60</v>
@@ -5832,7 +5832,7 @@
         <v>Route 20</v>
       </c>
       <c r="C320" t="str">
-        <v>Surskit</v>
+        <v>Hawlucha</v>
       </c>
       <c r="D320" t="str">
         <v>56-60</v>
@@ -5849,7 +5849,7 @@
         <v>Route 20</v>
       </c>
       <c r="C321" t="str">
-        <v>Zigzagoon</v>
+        <v>Carbink</v>
       </c>
       <c r="D321" t="str">
         <v>56-60</v>
@@ -5866,7 +5866,7 @@
         <v>Route 20</v>
       </c>
       <c r="C322" t="str">
-        <v>Staryu</v>
+        <v>Pinsir</v>
       </c>
       <c r="D322" t="str">
         <v>56-60</v>
@@ -5883,7 +5883,7 @@
         <v>Route 20</v>
       </c>
       <c r="C323" t="str">
-        <v>Manectric</v>
+        <v>Barbaracle</v>
       </c>
       <c r="D323" t="str">
         <v>56-60</v>
@@ -5900,7 +5900,7 @@
         <v>Pokémon Village</v>
       </c>
       <c r="C324" t="str">
-        <v>Azurill</v>
+        <v>Scizor</v>
       </c>
       <c r="D324" t="str">
         <v>57-61</v>
@@ -5917,7 +5917,7 @@
         <v>Pokémon Village</v>
       </c>
       <c r="C325" t="str">
-        <v>Xerneas</v>
+        <v>Gengar</v>
       </c>
       <c r="D325" t="str">
         <v>57-61</v>
@@ -5934,7 +5934,7 @@
         <v>Pokémon Village</v>
       </c>
       <c r="C326" t="str">
-        <v>Ferrothorn</v>
+        <v>Alakazam</v>
       </c>
       <c r="D326" t="str">
         <v>57-61</v>
@@ -5951,7 +5951,7 @@
         <v>Pokémon Village</v>
       </c>
       <c r="C327" t="str">
-        <v>Kecleon</v>
+        <v>Wailord</v>
       </c>
       <c r="D327" t="str">
         <v>57-61</v>
@@ -5968,7 +5968,7 @@
         <v>Pokémon Village</v>
       </c>
       <c r="C328" t="str">
-        <v>Jolteon</v>
+        <v>Ursaring</v>
       </c>
       <c r="D328" t="str">
         <v>57-61</v>
@@ -5985,7 +5985,7 @@
         <v>Pokémon Village (Fishing)</v>
       </c>
       <c r="C329" t="str">
-        <v>Leafeon</v>
+        <v>Scyther</v>
       </c>
       <c r="D329" t="str">
         <v>58-63</v>
@@ -6002,7 +6002,7 @@
         <v>Pokémon Village (Fishing)</v>
       </c>
       <c r="C330" t="str">
-        <v>Weedle</v>
+        <v>Heracross</v>
       </c>
       <c r="D330" t="str">
         <v>58-63</v>
@@ -6019,7 +6019,7 @@
         <v>Pokémon Village (Fishing)</v>
       </c>
       <c r="C331" t="str">
-        <v>Croagunk</v>
+        <v>Aegislash</v>
       </c>
       <c r="D331" t="str">
         <v>58-63</v>
@@ -6036,7 +6036,7 @@
         <v>Pokémon Village (Fishing)</v>
       </c>
       <c r="C332" t="str">
-        <v>Lickitung</v>
+        <v>Nidoqueen</v>
       </c>
       <c r="D332" t="str">
         <v>58-63</v>
@@ -6053,7 +6053,7 @@
         <v>Pokémon Village (Fishing)</v>
       </c>
       <c r="C333" t="str">
-        <v>Aggron</v>
+        <v>Machamp</v>
       </c>
       <c r="D333" t="str">
         <v>58-63</v>
@@ -6070,7 +6070,7 @@
         <v>Route 21</v>
       </c>
       <c r="C334" t="str">
-        <v>Octillery</v>
+        <v>Honchkrow</v>
       </c>
       <c r="D334" t="str">
         <v>59-64</v>
@@ -6087,7 +6087,7 @@
         <v>Route 21</v>
       </c>
       <c r="C335" t="str">
-        <v>Pansage</v>
+        <v>Nidoking</v>
       </c>
       <c r="D335" t="str">
         <v>59-64</v>
@@ -6104,7 +6104,7 @@
         <v>Route 21</v>
       </c>
       <c r="C336" t="str">
-        <v>Corphish</v>
+        <v>Shuckle</v>
       </c>
       <c r="D336" t="str">
         <v>59-64</v>
@@ -6121,7 +6121,7 @@
         <v>Route 21</v>
       </c>
       <c r="C337" t="str">
-        <v>Garchomp</v>
+        <v>Conkeldurr</v>
       </c>
       <c r="D337" t="str">
         <v>59-64</v>
@@ -6138,7 +6138,7 @@
         <v>Route 21</v>
       </c>
       <c r="C338" t="str">
-        <v>Sentret</v>
+        <v>Pyroar</v>
       </c>
       <c r="D338" t="str">
         <v>59-64</v>
@@ -6155,7 +6155,7 @@
         <v>Victory Road</v>
       </c>
       <c r="C339" t="str">
-        <v>Deino</v>
+        <v>Poliwrath</v>
       </c>
       <c r="D339" t="str">
         <v>60-65</v>
@@ -6172,7 +6172,7 @@
         <v>Victory Road</v>
       </c>
       <c r="C340" t="str">
-        <v>Magikarp</v>
+        <v>Steelix</v>
       </c>
       <c r="D340" t="str">
         <v>60-65</v>
@@ -6189,7 +6189,7 @@
         <v>Victory Road</v>
       </c>
       <c r="C341" t="str">
-        <v>Tyrunt</v>
+        <v>Zoroark</v>
       </c>
       <c r="D341" t="str">
         <v>60-65</v>
@@ -6206,7 +6206,7 @@
         <v>Victory Road</v>
       </c>
       <c r="C342" t="str">
-        <v>Wingull</v>
+        <v>Gliscor</v>
       </c>
       <c r="D342" t="str">
         <v>60-65</v>
@@ -6223,7 +6223,7 @@
         <v>Victory Road</v>
       </c>
       <c r="C343" t="str">
-        <v>Pancham</v>
+        <v>Weavile</v>
       </c>
       <c r="D343" t="str">
         <v>60-65</v>
@@ -6240,7 +6240,7 @@
         <v>Kalos Pokemon League</v>
       </c>
       <c r="C344" t="str">
-        <v>Cloyster</v>
+        <v>Mienshao</v>
       </c>
       <c r="D344" t="str">
         <v>61-66</v>
@@ -6257,7 +6257,7 @@
         <v>Kalos Pokemon League</v>
       </c>
       <c r="C345" t="str">
-        <v>Lickilicky</v>
+        <v>Avalugg</v>
       </c>
       <c r="D345" t="str">
         <v>61-66</v>
@@ -6274,7 +6274,7 @@
         <v>Kalos Pokemon League</v>
       </c>
       <c r="C346" t="str">
-        <v>Floette</v>
+        <v>Tentacruel</v>
       </c>
       <c r="D346" t="str">
         <v>61-66</v>
@@ -6291,7 +6291,7 @@
         <v>Kalos Pokemon League</v>
       </c>
       <c r="C347" t="str">
-        <v>Wynaut</v>
+        <v>Yanmega</v>
       </c>
       <c r="D347" t="str">
         <v>61-66</v>
@@ -6308,7 +6308,7 @@
         <v>Kalos Pokemon League</v>
       </c>
       <c r="C348" t="str">
-        <v>Amaura</v>
+        <v>Aerodactyl</v>
       </c>
       <c r="D348" t="str">
         <v>61-66</v>
@@ -6325,7 +6325,7 @@
         <v>Kiloude City</v>
       </c>
       <c r="C349" t="str">
-        <v>Tentacool</v>
+        <v>Roserade</v>
       </c>
       <c r="D349" t="str">
         <v>50-57</v>
@@ -6342,7 +6342,7 @@
         <v>Kiloude City</v>
       </c>
       <c r="C350" t="str">
-        <v>Zygarde</v>
+        <v>Gigalith</v>
       </c>
       <c r="D350" t="str">
         <v>50-57</v>
@@ -6359,7 +6359,7 @@
         <v>Kiloude City</v>
       </c>
       <c r="C351" t="str">
-        <v>Cryogonal</v>
+        <v>Lickilicky</v>
       </c>
       <c r="D351" t="str">
         <v>50-57</v>
@@ -6376,7 +6376,7 @@
         <v>Kiloude City</v>
       </c>
       <c r="C352" t="str">
-        <v>Espurr</v>
+        <v>Cryogonal</v>
       </c>
       <c r="D352" t="str">
         <v>50-57</v>
@@ -6393,7 +6393,7 @@
         <v>Kiloude City</v>
       </c>
       <c r="C353" t="str">
-        <v>Ledyba</v>
+        <v>Gardevoir</v>
       </c>
       <c r="D353" t="str">
         <v>50-57</v>
@@ -6410,7 +6410,7 @@
         <v>Friend Safari</v>
       </c>
       <c r="C354" t="str">
-        <v>Riolu</v>
+        <v>Krookodile</v>
       </c>
       <c r="D354" t="str">
         <v>55-62</v>
@@ -6427,7 +6427,7 @@
         <v>Friend Safari</v>
       </c>
       <c r="C355" t="str">
-        <v>Scyther</v>
+        <v>Chandelure</v>
       </c>
       <c r="D355" t="str">
         <v>55-62</v>
@@ -6444,7 +6444,7 @@
         <v>Friend Safari</v>
       </c>
       <c r="C356" t="str">
-        <v>Altaria</v>
+        <v>Flygon</v>
       </c>
       <c r="D356" t="str">
         <v>55-62</v>
@@ -6461,7 +6461,7 @@
         <v>Friend Safari</v>
       </c>
       <c r="C357" t="str">
-        <v>Gothitelle</v>
+        <v>Tyrantrum</v>
       </c>
       <c r="D357" t="str">
         <v>55-62</v>
@@ -6478,7 +6478,7 @@
         <v>Friend Safari</v>
       </c>
       <c r="C358" t="str">
-        <v>Psyduck</v>
+        <v>Aurorus</v>
       </c>
       <c r="D358" t="str">
         <v>55-62</v>
@@ -6495,7 +6495,7 @@
         <v>Battle Maison</v>
       </c>
       <c r="C359" t="str">
-        <v>Druddigon</v>
+        <v>Vaporeon</v>
       </c>
       <c r="D359" t="str">
         <v>63-70</v>
@@ -6512,7 +6512,7 @@
         <v>Battle Maison</v>
       </c>
       <c r="C360" t="str">
-        <v>Mienshao</v>
+        <v>Sylveon</v>
       </c>
       <c r="D360" t="str">
         <v>63-70</v>
@@ -6529,7 +6529,7 @@
         <v>Battle Maison</v>
       </c>
       <c r="C361" t="str">
-        <v>Heracross</v>
+        <v>Probopass</v>
       </c>
       <c r="D361" t="str">
         <v>63-70</v>
@@ -6546,7 +6546,7 @@
         <v>Battle Maison</v>
       </c>
       <c r="C362" t="str">
-        <v>Talonflame</v>
+        <v>Lucario</v>
       </c>
       <c r="D362" t="str">
         <v>63-70</v>
@@ -6563,7 +6563,7 @@
         <v>Battle Maison</v>
       </c>
       <c r="C363" t="str">
-        <v>Skrelp</v>
+        <v>Flareon</v>
       </c>
       <c r="D363" t="str">
         <v>63-70</v>
@@ -6580,7 +6580,7 @@
         <v>Sea Spirit Den Entrance</v>
       </c>
       <c r="C364" t="str">
-        <v>Qwilfish</v>
+        <v>Hippowdon</v>
       </c>
       <c r="D364" t="str">
         <v>84-91</v>
@@ -6597,7 +6597,7 @@
         <v>Sea Spirit Den Entrance</v>
       </c>
       <c r="C365" t="str">
-        <v>Reuniclus</v>
+        <v>Glaceon</v>
       </c>
       <c r="D365" t="str">
         <v>84-91</v>
@@ -6614,7 +6614,7 @@
         <v>Sea Spirit Den Entrance</v>
       </c>
       <c r="C366" t="str">
-        <v>Mothim</v>
+        <v>Venusaur</v>
       </c>
       <c r="D366" t="str">
         <v>84-91</v>
@@ -6631,7 +6631,7 @@
         <v>Sea Spirit Den Entrance</v>
       </c>
       <c r="C367" t="str">
-        <v>Mawile</v>
+        <v>Umbreon</v>
       </c>
       <c r="D367" t="str">
         <v>84-91</v>
@@ -6648,7 +6648,7 @@
         <v>Sea Spirit Den Entrance</v>
       </c>
       <c r="C368" t="str">
-        <v>Igglybuff</v>
+        <v>Jolteon</v>
       </c>
       <c r="D368" t="str">
         <v>84-91</v>
@@ -6665,7 +6665,7 @@
         <v>Sea Spirit Den Tunnels</v>
       </c>
       <c r="C369" t="str">
-        <v>Gogoat</v>
+        <v>Leafeon</v>
       </c>
       <c r="D369" t="str">
         <v>91-98</v>
@@ -6682,7 +6682,7 @@
         <v>Sea Spirit Den Tunnels</v>
       </c>
       <c r="C370" t="str">
-        <v>Slugma</v>
+        <v>Cloyster</v>
       </c>
       <c r="D370" t="str">
         <v>91-98</v>
@@ -6699,7 +6699,7 @@
         <v>Sea Spirit Den Tunnels</v>
       </c>
       <c r="C371" t="str">
-        <v>Axew</v>
+        <v>Blastoise</v>
       </c>
       <c r="D371" t="str">
         <v>91-98</v>
@@ -6716,7 +6716,7 @@
         <v>Sea Spirit Den Tunnels</v>
       </c>
       <c r="C372" t="str">
-        <v>Illumise</v>
+        <v>Chesnaught</v>
       </c>
       <c r="D372" t="str">
         <v>91-98</v>
@@ -6733,7 +6733,7 @@
         <v>Sea Spirit Den Tunnels</v>
       </c>
       <c r="C373" t="str">
-        <v>Shuppet</v>
+        <v>Mamoswine</v>
       </c>
       <c r="D373" t="str">
         <v>91-98</v>
@@ -6750,7 +6750,7 @@
         <v>Chambers of Emptiness</v>
       </c>
       <c r="C374" t="str">
-        <v>Flygon</v>
+        <v>Greninja</v>
       </c>
       <c r="D374" t="str">
         <v>91-98</v>
@@ -6767,7 +6767,7 @@
         <v>Chambers of Emptiness</v>
       </c>
       <c r="C375" t="str">
-        <v>Absol</v>
+        <v>Aggron</v>
       </c>
       <c r="D375" t="str">
         <v>91-98</v>
@@ -6784,7 +6784,7 @@
         <v>Chambers of Emptiness</v>
       </c>
       <c r="C376" t="str">
-        <v>Carvanha</v>
+        <v>Gogoat</v>
       </c>
       <c r="D376" t="str">
         <v>91-98</v>
@@ -6801,7 +6801,7 @@
         <v>Chambers of Emptiness</v>
       </c>
       <c r="C377" t="str">
-        <v>Wooper</v>
+        <v>Delphox</v>
       </c>
       <c r="D377" t="str">
         <v>91-98</v>
@@ -6818,7 +6818,7 @@
         <v>Chambers of Emptiness</v>
       </c>
       <c r="C378" t="str">
-        <v>Diancie</v>
+        <v>Vanilluxe</v>
       </c>
       <c r="D378" t="str">
         <v>91-98</v>
@@ -6835,7 +6835,7 @@
         <v>Team Flare Secret HQ Entrance</v>
       </c>
       <c r="C379" t="str">
-        <v>Geodude</v>
+        <v>Crobat</v>
       </c>
       <c r="D379" t="str">
         <v>91-98</v>
@@ -6852,7 +6852,7 @@
         <v>Team Flare Secret HQ Entrance</v>
       </c>
       <c r="C380" t="str">
-        <v>Hoppip</v>
+        <v>Rhyperior</v>
       </c>
       <c r="D380" t="str">
         <v>91-98</v>
@@ -6869,7 +6869,7 @@
         <v>Team Flare Secret HQ Entrance</v>
       </c>
       <c r="C381" t="str">
-        <v>Aegislash</v>
+        <v>Lapras</v>
       </c>
       <c r="D381" t="str">
         <v>91-98</v>
@@ -6886,7 +6886,7 @@
         <v>Team Flare Secret HQ Entrance</v>
       </c>
       <c r="C382" t="str">
-        <v>Slowpoke</v>
+        <v>Noivern</v>
       </c>
       <c r="D382" t="str">
         <v>91-98</v>
@@ -6903,7 +6903,7 @@
         <v>Team Flare Secret HQ Entrance</v>
       </c>
       <c r="C383" t="str">
-        <v>Bagon</v>
+        <v>Haxorus</v>
       </c>
       <c r="D383" t="str">
         <v>91-98</v>
@@ -6920,7 +6920,7 @@
         <v>Mystic Tower Entrance</v>
       </c>
       <c r="C384" t="str">
-        <v>Oddish</v>
+        <v>Gyarados</v>
       </c>
       <c r="D384" t="str">
         <v>62-67</v>
@@ -6937,7 +6937,7 @@
         <v>Mystic Tower Entrance</v>
       </c>
       <c r="C385" t="str">
-        <v>Simipour</v>
+        <v>Florges</v>
       </c>
       <c r="D385" t="str">
         <v>62-67</v>
@@ -6954,7 +6954,7 @@
         <v>Mystic Tower Entrance</v>
       </c>
       <c r="C386" t="str">
-        <v>Swirlix</v>
+        <v>Articuno</v>
       </c>
       <c r="D386" t="str">
         <v>62-67</v>
@@ -6971,7 +6971,7 @@
         <v>Mystic Tower Entrance</v>
       </c>
       <c r="C387" t="str">
-        <v>Salamence</v>
+        <v>Zapdos</v>
       </c>
       <c r="D387" t="str">
         <v>62-67</v>
@@ -6988,7 +6988,7 @@
         <v>Mystic Tower Entrance</v>
       </c>
       <c r="C388" t="str">
-        <v>Zorua</v>
+        <v>Moltres</v>
       </c>
       <c r="D388" t="str">
         <v>62-67</v>
@@ -7005,7 +7005,7 @@
         <v>Crystal Cave Tunnels</v>
       </c>
       <c r="C389" t="str">
-        <v>Gyarados</v>
+        <v>Volcanion</v>
       </c>
       <c r="D389" t="str">
         <v>63-68</v>
@@ -7022,7 +7022,7 @@
         <v>Crystal Cave Tunnels</v>
       </c>
       <c r="C390" t="str">
-        <v>Scrafty</v>
+        <v>Tyranitar</v>
       </c>
       <c r="D390" t="str">
         <v>63-68</v>
@@ -7039,7 +7039,7 @@
         <v>Crystal Cave Tunnels</v>
       </c>
       <c r="C391" t="str">
-        <v>Panpour</v>
+        <v>Hydreigon</v>
       </c>
       <c r="D391" t="str">
         <v>63-68</v>
@@ -7056,7 +7056,7 @@
         <v>Crystal Cave Tunnels</v>
       </c>
       <c r="C392" t="str">
-        <v>Karrablast</v>
+        <v>Garchomp</v>
       </c>
       <c r="D392" t="str">
         <v>63-68</v>
@@ -7073,7 +7073,7 @@
         <v>Crystal Cave Tunnels</v>
       </c>
       <c r="C393" t="str">
-        <v>Spinarak</v>
+        <v>Zygarde</v>
       </c>
       <c r="D393" t="str">
         <v>63-68</v>
@@ -7090,7 +7090,7 @@
         <v>Secret Forest North</v>
       </c>
       <c r="C394" t="str">
-        <v>Roggenrola</v>
+        <v>Diancie</v>
       </c>
       <c r="D394" t="str">
         <v>65-70</v>
@@ -7107,7 +7107,7 @@
         <v>Secret Forest North</v>
       </c>
       <c r="C395" t="str">
-        <v>Swanna</v>
+        <v>Salamence</v>
       </c>
       <c r="D395" t="str">
         <v>65-70</v>
@@ -7124,7 +7124,7 @@
         <v>Secret Forest North</v>
       </c>
       <c r="C396" t="str">
-        <v>Whismur</v>
+        <v>Yveltal</v>
       </c>
       <c r="D396" t="str">
         <v>65-70</v>
@@ -7141,7 +7141,7 @@
         <v>Secret Forest North</v>
       </c>
       <c r="C397" t="str">
-        <v>Solrock</v>
+        <v>Mewtwo</v>
       </c>
       <c r="D397" t="str">
         <v>65-70</v>
@@ -7158,7 +7158,7 @@
         <v>Secret Forest North</v>
       </c>
       <c r="C398" t="str">
-        <v>Malamar</v>
+        <v>Xerneas</v>
       </c>
       <c r="D398" t="str">
         <v>65-70</v>

</xml_diff>

<commit_message>
Format Kalos challenges to utilize explicitly mapped human-readable Requisites
Co-authored-by: lsampaio1337-beep <246645260+lsampaio1337-beep@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Kalos_Path.xlsx
+++ b/Kalos_Path.xlsx
@@ -8248,7 +8248,7 @@
         <v>Challenge 1</v>
       </c>
       <c r="B2" t="str">
-        <v>catchSpeciesAnyOf: { route: 'Aquacorde Town', count: 5 }</v>
+        <v>Catch 5 different species from Aquacorde Town</v>
       </c>
       <c r="C2" t="str">
         <v>Unlock Route 2</v>
@@ -8259,7 +8259,7 @@
         <v>Challenge 2</v>
       </c>
       <c r="B3" t="str">
-        <v>defeatCountRoute: { route: 'Route 2', count: 25 }</v>
+        <v>Defeat 25 pokemon from Route 2</v>
       </c>
       <c r="C3" t="str">
         <v>Unlock Santalune Forest</v>
@@ -8270,7 +8270,7 @@
         <v>Challenge 3</v>
       </c>
       <c r="B4" t="str">
-        <v>catchSpeciesAnyOf: { route: 'Santalune Forest', count: 5 }</v>
+        <v>Catch 5 different species from Santalune Forest</v>
       </c>
       <c r="C4" t="str">
         <v>Unlock Route 3</v>
@@ -8281,7 +8281,7 @@
         <v>Challenge 4</v>
       </c>
       <c r="B5" t="str">
-        <v>defeatCountRoute: { route: 'Route 3', count: 25 }</v>
+        <v>Defeat 25 pokemon from Route 3</v>
       </c>
       <c r="C5" t="str">
         <v>Unlock Santalune City</v>
@@ -8292,7 +8292,7 @@
         <v>Challenge 5</v>
       </c>
       <c r="B6" t="str">
-        <v>catchSpeciesAnyOf: { route: 'Santalune City', count: 5 }</v>
+        <v>Catch 5 different species from Santalune City</v>
       </c>
       <c r="C6" t="str">
         <v>Unlock Santalune City Gym</v>
@@ -8303,7 +8303,7 @@
         <v>Challenge 6</v>
       </c>
       <c r="B7" t="str">
-        <v>earnBadge: { badge: 'Bug Badge', leader: 'Viola' }</v>
+        <v>Earn the Bug Badge from Viola</v>
       </c>
       <c r="C7" t="str">
         <v>Unlock Route 22</v>
@@ -8314,7 +8314,7 @@
         <v>Challenge 7</v>
       </c>
       <c r="B8" t="str">
-        <v>catchSpeciesAnyOf: { route: 'Route 22', count: 5 }</v>
+        <v>Catch 5 different species from Route 22</v>
       </c>
       <c r="C8" t="str">
         <v>Unlock Route 4</v>
@@ -8325,7 +8325,7 @@
         <v>Challenge 8</v>
       </c>
       <c r="B9" t="str">
-        <v>defeatCountRoute: { route: 'Route 4', count: 25 }</v>
+        <v>Defeat 25 pokemon from Route 4</v>
       </c>
       <c r="C9" t="str">
         <v>Unlock Lumiose City (South)</v>
@@ -8336,7 +8336,7 @@
         <v>Challenge 9</v>
       </c>
       <c r="B10" t="str">
-        <v>catchSpeciesAnyOf: { route: 'Lumiose City (South)', count: 5 }</v>
+        <v>Catch 5 different species from Lumiose City (South)</v>
       </c>
       <c r="C10" t="str">
         <v>Unlock Route 5</v>
@@ -8347,7 +8347,7 @@
         <v>Challenge 10</v>
       </c>
       <c r="B11" t="str">
-        <v>defeatCountRoute: { route: 'Route 5', count: 25 }</v>
+        <v>Defeat 25 pokemon from Route 5</v>
       </c>
       <c r="C11" t="str">
         <v>Unlock Camphrier Town</v>
@@ -8358,7 +8358,7 @@
         <v>Challenge 11</v>
       </c>
       <c r="B12" t="str">
-        <v>catchSpeciesAnyOf: { route: 'Camphrier Town', count: 5 }</v>
+        <v>Catch 5 different species from Camphrier Town</v>
       </c>
       <c r="C12" t="str">
         <v>Unlock Parfum Palace</v>
@@ -8369,7 +8369,7 @@
         <v>Challenge 12</v>
       </c>
       <c r="B13" t="str">
-        <v>defeatCountRoute: { route: 'Parfum Palace', count: 50 }</v>
+        <v>Defeat 50 pokemon from Parfum Palace</v>
       </c>
       <c r="C13" t="str">
         <v>Unlock Route 6</v>
@@ -8380,7 +8380,7 @@
         <v>Challenge 13</v>
       </c>
       <c r="B14" t="str">
-        <v>catchSpeciesAnyOf: { route: 'Route 6', count: 5 }</v>
+        <v>Catch 5 different species from Route 6</v>
       </c>
       <c r="C14" t="str">
         <v>Unlock Route 7</v>
@@ -8391,7 +8391,7 @@
         <v>Challenge 14</v>
       </c>
       <c r="B15" t="str">
-        <v>defeatCountRoute: { route: 'Route 7', count: 50 }</v>
+        <v>Defeat 50 pokemon from Route 7</v>
       </c>
       <c r="C15" t="str">
         <v>Unlock Connecting Cave</v>
@@ -8402,7 +8402,7 @@
         <v>Challenge 15</v>
       </c>
       <c r="B16" t="str">
-        <v>catchSpeciesAnyOf: { route: 'Connecting Cave', count: 5 }</v>
+        <v>Catch 5 different species from Connecting Cave</v>
       </c>
       <c r="C16" t="str">
         <v>Unlock Ambrette Town</v>
@@ -8413,7 +8413,7 @@
         <v>Challenge 16</v>
       </c>
       <c r="B17" t="str">
-        <v>defeatCountRoute: { route: 'Ambrette Town', count: 50 }</v>
+        <v>Defeat 50 pokemon from Ambrette Town</v>
       </c>
       <c r="C17" t="str">
         <v>Unlock Ambrette Town (Fishing)</v>
@@ -8424,7 +8424,7 @@
         <v>Challenge 17</v>
       </c>
       <c r="B18" t="str">
-        <v>catchSpeciesAnyOf: { route: 'Ambrette Town (Fishing)', count: 5 }</v>
+        <v>Catch 5 different species from Ambrette Town (Fishing)</v>
       </c>
       <c r="C18" t="str">
         <v>Unlock Route 8</v>
@@ -8435,7 +8435,7 @@
         <v>Challenge 18</v>
       </c>
       <c r="B19" t="str">
-        <v>defeatCountRoute: { route: 'Route 8', count: 50 }</v>
+        <v>Defeat 50 pokemon from Route 8</v>
       </c>
       <c r="C19" t="str">
         <v>Unlock Route 9</v>
@@ -8446,7 +8446,7 @@
         <v>Challenge 19</v>
       </c>
       <c r="B20" t="str">
-        <v>catchSpeciesAnyOf: { route: 'Route 9', count: 5 }</v>
+        <v>Catch 5 different species from Route 9</v>
       </c>
       <c r="C20" t="str">
         <v>Unlock Glittering Cave</v>
@@ -8457,7 +8457,7 @@
         <v>Challenge 20</v>
       </c>
       <c r="B21" t="str">
-        <v>defeatCountRoute: { route: 'Glittering Cave', count: 50 }</v>
+        <v>Defeat 50 pokemon from Glittering Cave</v>
       </c>
       <c r="C21" t="str">
         <v>Unlock Cyllage City</v>
@@ -8468,7 +8468,7 @@
         <v>Challenge 21</v>
       </c>
       <c r="B22" t="str">
-        <v>catchSpeciesAnyOf: { route: 'Cyllage City', count: 5 }</v>
+        <v>Catch 5 different species from Cyllage City</v>
       </c>
       <c r="C22" t="str">
         <v>Unlock Cyllage City Gym</v>
@@ -8479,7 +8479,7 @@
         <v>Challenge 22</v>
       </c>
       <c r="B23" t="str">
-        <v>earnBadge: { badge: 'Cliff Badge', leader: 'Grant' }</v>
+        <v>Earn the Cliff Badge from Grant</v>
       </c>
       <c r="C23" t="str">
         <v>Unlock Route 10 AND Unlock Cyllage City (Fishing) (first spot for Extra Challenge A)</v>
@@ -8490,7 +8490,7 @@
         <v>Challenge 23</v>
       </c>
       <c r="B24" t="str">
-        <v>catchSpeciesAnyOf: { route: 'Route 10', count: 5 }</v>
+        <v>Catch 5 different species from Route 10</v>
       </c>
       <c r="C24" t="str">
         <v>Unlock Geosenge Town</v>
@@ -8501,7 +8501,7 @@
         <v>Challenge 24</v>
       </c>
       <c r="B25" t="str">
-        <v>defeatCountRoute: { route: 'Geosenge Town', count: 100 }</v>
+        <v>Defeat 100 pokemon from Geosenge Town</v>
       </c>
       <c r="C25" t="str">
         <v>Unlock Route 11</v>
@@ -8512,7 +8512,7 @@
         <v>Challenge 25</v>
       </c>
       <c r="B26" t="str">
-        <v>catchSpeciesAnyOf: { route: 'Route 11', count: 5 }</v>
+        <v>Catch 5 different species from Route 11</v>
       </c>
       <c r="C26" t="str">
         <v>Unlock Shalour City</v>
@@ -8523,7 +8523,7 @@
         <v>Challenge 26</v>
       </c>
       <c r="B27" t="str">
-        <v>defeatCountRoute: { route: 'Shalour City', count: 100 }</v>
+        <v>Defeat 100 pokemon from Shalour City</v>
       </c>
       <c r="C27" t="str">
         <v>Unlock Shalour City Gym</v>
@@ -8534,7 +8534,7 @@
         <v>Challenge 27</v>
       </c>
       <c r="B28" t="str">
-        <v>earnBadge: { badge: 'Rumble Badge', leader: 'Korrina' }</v>
+        <v>Earn the Rumble Badge from Korrina</v>
       </c>
       <c r="C28" t="str">
         <v>Unlock Route 12</v>
@@ -8545,7 +8545,7 @@
         <v>Challenge 28</v>
       </c>
       <c r="B29" t="str">
-        <v>defeatCountRoute: { route: 'Route 12', count: 100 }</v>
+        <v>Defeat 100 pokemon from Route 12</v>
       </c>
       <c r="C29" t="str">
         <v>Unlock Azure Bay</v>
@@ -8556,7 +8556,7 @@
         <v>Challenge 29</v>
       </c>
       <c r="B30" t="str">
-        <v>catchSpeciesAnyOf: { route: 'Azure Bay', count: 5 }</v>
+        <v>Catch 5 different species from Azure Bay</v>
       </c>
       <c r="C30" t="str">
         <v>Unlock Azure Bay (Fishing)</v>
@@ -8567,7 +8567,7 @@
         <v>Challenge 30</v>
       </c>
       <c r="B31" t="str">
-        <v>defeatCountRoute: { route: 'Azure Bay (Fishing)', count: 100 }</v>
+        <v>Defeat 100 pokemon from Azure Bay (Fishing)</v>
       </c>
       <c r="C31" t="str">
         <v>Unlock Coumarine City Gym</v>
@@ -8578,7 +8578,7 @@
         <v>Challenge 31</v>
       </c>
       <c r="B32" t="str">
-        <v>earnBadge: { badge: 'Plant Badge', leader: 'Ramos' }</v>
+        <v>Earn the Plant Badge from Ramos</v>
       </c>
       <c r="C32" t="str">
         <v>Unlock Coumarine City (Fishing) AND Unlock Starter Depot (first spot for Extra Challenge B)</v>
@@ -8589,7 +8589,7 @@
         <v>Challenge 32</v>
       </c>
       <c r="B33" t="str">
-        <v>defeatCountRoute: { route: 'Coumarine City (Fishing)', count: 200 }</v>
+        <v>Defeat 200 pokemon from Coumarine City (Fishing)</v>
       </c>
       <c r="C33" t="str">
         <v>Unlock Route 13</v>
@@ -8600,7 +8600,7 @@
         <v>Challenge 33</v>
       </c>
       <c r="B34" t="str">
-        <v>catchSpeciesAnyOf: { route: 'Route 13', count: 5 }</v>
+        <v>Catch 5 different species from Route 13</v>
       </c>
       <c r="C34" t="str">
         <v>Unlock Lumiose City (North)</v>
@@ -8611,7 +8611,7 @@
         <v>Challenge 34</v>
       </c>
       <c r="B35" t="str">
-        <v>defeatCountRoute: { route: 'Lumiose City (North)', count: 200 }</v>
+        <v>Defeat 200 pokemon from Lumiose City (North)</v>
       </c>
       <c r="C35" t="str">
         <v>Unlock Lumiose City Gym</v>
@@ -8622,7 +8622,7 @@
         <v>Challenge 35</v>
       </c>
       <c r="B36" t="str">
-        <v>earnBadge: { badge: 'Voltage Badge', leader: 'Clemont' }</v>
+        <v>Earn the Voltage Badge from Clemont</v>
       </c>
       <c r="C36" t="str">
         <v>Unlock Route 14</v>
@@ -8633,7 +8633,7 @@
         <v>Challenge 36</v>
       </c>
       <c r="B37" t="str">
-        <v>defeatCountRoute: { route: 'Route 14', count: 200 }</v>
+        <v>Defeat 200 pokemon from Route 14</v>
       </c>
       <c r="C37" t="str">
         <v>Unlock Laverre City</v>
@@ -8644,7 +8644,7 @@
         <v>Challenge 37</v>
       </c>
       <c r="B38" t="str">
-        <v>catchSpeciesAnyOf: { route: 'Laverre City', count: 5 }</v>
+        <v>Catch 5 different species from Laverre City</v>
       </c>
       <c r="C38" t="str">
         <v>Unlock Laverre City Gym</v>
@@ -8655,7 +8655,7 @@
         <v>Challenge 38</v>
       </c>
       <c r="B39" t="str">
-        <v>earnBadge: { badge: 'Fairy Badge', leader: 'Valerie' }</v>
+        <v>Earn the Fairy Badge from Valerie</v>
       </c>
       <c r="C39" t="str">
         <v>Unlock Route 15</v>
@@ -8666,7 +8666,7 @@
         <v>Challenge 39</v>
       </c>
       <c r="B40" t="str">
-        <v>catchSpeciesAnyOf: { route: 'Route 15', count: 5 }</v>
+        <v>Catch 5 different species from Route 15</v>
       </c>
       <c r="C40" t="str">
         <v>Unlock Lost Hotel</v>
@@ -8677,7 +8677,7 @@
         <v>Challenge 40</v>
       </c>
       <c r="B41" t="str">
-        <v>defeatCountRoute: { route: 'Lost Hotel', count: 200 }</v>
+        <v>Defeat 200 pokemon from Lost Hotel</v>
       </c>
       <c r="C41" t="str">
         <v>Unlock Dendemille Town</v>
@@ -8688,7 +8688,7 @@
         <v>Challenge 41</v>
       </c>
       <c r="B42" t="str">
-        <v>catchSpeciesAnyOf: { route: 'Dendemille Town', count: 5 }</v>
+        <v>Catch 5 different species from Dendemille Town</v>
       </c>
       <c r="C42" t="str">
         <v>Unlock Route 16</v>
@@ -8699,7 +8699,7 @@
         <v>Challenge 42</v>
       </c>
       <c r="B43" t="str">
-        <v>defeatCountRoute: { route: 'Route 16', count: 300 }</v>
+        <v>Defeat 300 pokemon from Route 16</v>
       </c>
       <c r="C43" t="str">
         <v>Unlock Frost Cavern</v>
@@ -8710,7 +8710,7 @@
         <v>Challenge 43</v>
       </c>
       <c r="B44" t="str">
-        <v>catchSpeciesAnyOf: { route: 'Frost Cavern', count: 5 }</v>
+        <v>Catch 5 different species from Frost Cavern</v>
       </c>
       <c r="C44" t="str">
         <v>Unlock Anistar City</v>
@@ -8721,7 +8721,7 @@
         <v>Challenge 44</v>
       </c>
       <c r="B45" t="str">
-        <v>defeatCountRoute: { route: 'Anistar City', count: 300 }</v>
+        <v>Defeat 300 pokemon from Anistar City</v>
       </c>
       <c r="C45" t="str">
         <v>Unlock Anistar City Gym</v>
@@ -8732,7 +8732,7 @@
         <v>Challenge 45</v>
       </c>
       <c r="B46" t="str">
-        <v>earnBadge: { badge: 'Psychic Badge', leader: 'Olympia' }</v>
+        <v>Earn the Psychic Badge from Olympia</v>
       </c>
       <c r="C46" t="str">
         <v>Unlock Route 17</v>
@@ -8743,7 +8743,7 @@
         <v>Challenge 46</v>
       </c>
       <c r="B47" t="str">
-        <v>defeatCountRoute: { route: 'Route 17', count: 300 }</v>
+        <v>Defeat 300 pokemon from Route 17</v>
       </c>
       <c r="C47" t="str">
         <v>Unlock Couriway Town</v>
@@ -8754,7 +8754,7 @@
         <v>Challenge 47</v>
       </c>
       <c r="B48" t="str">
-        <v>catchSpeciesAnyOf: { route: 'Couriway Town', count: 5 }</v>
+        <v>Catch 5 different species from Couriway Town</v>
       </c>
       <c r="C48" t="str">
         <v>Unlock Route 18</v>
@@ -8765,7 +8765,7 @@
         <v>Challenge 48</v>
       </c>
       <c r="B49" t="str">
-        <v>defeatCountRoute: { route: 'Route 18', count: 300 }</v>
+        <v>Defeat 300 pokemon from Route 18</v>
       </c>
       <c r="C49" t="str">
         <v>Unlock Terminus Cave (Surface)</v>
@@ -8776,7 +8776,7 @@
         <v>Challenge 49</v>
       </c>
       <c r="B50" t="str">
-        <v>catchSpeciesAnyOf: { route: 'Terminus Cave (Surface)', count: 5 }</v>
+        <v>Catch 5 different species from Terminus Cave (Surface)</v>
       </c>
       <c r="C50" t="str">
         <v>Unlock Route 19</v>
@@ -8787,7 +8787,7 @@
         <v>Challenge 50</v>
       </c>
       <c r="B51" t="str">
-        <v>defeatCountRoute: { route: 'Route 19', count: 300 }</v>
+        <v>Defeat 300 pokemon from Route 19</v>
       </c>
       <c r="C51" t="str">
         <v>Unlock Route 19 (Fishing)</v>
@@ -8798,7 +8798,7 @@
         <v>Challenge 51</v>
       </c>
       <c r="B52" t="str">
-        <v>catchSpeciesAnyOf: { route: 'Route 19 (Fishing)', count: 5 }</v>
+        <v>Catch 5 different species from Route 19 (Fishing)</v>
       </c>
       <c r="C52" t="str">
         <v>Unlock Snowbelle City</v>
@@ -8809,7 +8809,7 @@
         <v>Challenge 52</v>
       </c>
       <c r="B53" t="str">
-        <v>defeatCountRoute: { route: 'Snowbelle City', count: 300 }</v>
+        <v>Defeat 300 pokemon from Snowbelle City</v>
       </c>
       <c r="C53" t="str">
         <v>Unlock Snowbelle City Gym</v>
@@ -8820,7 +8820,7 @@
         <v>Challenge 53</v>
       </c>
       <c r="B54" t="str">
-        <v>earnBadge: { badge: 'Iceberg Badge', leader: 'Wulfric' }</v>
+        <v>Earn the Iceberg Badge from Wulfric</v>
       </c>
       <c r="C54" t="str">
         <v>Unlock Route 20</v>
@@ -8831,7 +8831,7 @@
         <v>Challenge 54</v>
       </c>
       <c r="B55" t="str">
-        <v>defeatCountRoute: { route: 'Route 20', count: 300 }</v>
+        <v>Defeat 300 pokemon from Route 20</v>
       </c>
       <c r="C55" t="str">
         <v>Unlock Pokémon Village</v>
@@ -8842,7 +8842,7 @@
         <v>Challenge 55</v>
       </c>
       <c r="B56" t="str">
-        <v>catchSpeciesAnyOf: { route: 'Pokémon Village', count: 5 }</v>
+        <v>Catch 5 different species from Pokémon Village</v>
       </c>
       <c r="C56" t="str">
         <v>Unlock Pokémon Village (Fishing)</v>
@@ -8853,7 +8853,7 @@
         <v>Challenge 56</v>
       </c>
       <c r="B57" t="str">
-        <v>defeatCountRoute: { route: 'Pokémon Village (Fishing)', count: 300 }</v>
+        <v>Defeat 300 pokemon from Pokémon Village (Fishing)</v>
       </c>
       <c r="C57" t="str">
         <v>Unlock Route 21</v>
@@ -8864,7 +8864,7 @@
         <v>Challenge 57</v>
       </c>
       <c r="B58" t="str">
-        <v>catchSpeciesAnyOf: { route: 'Route 21', count: 5 }</v>
+        <v>Catch 5 different species from Route 21</v>
       </c>
       <c r="C58" t="str">
         <v>Unlock Victory Road</v>
@@ -8875,7 +8875,7 @@
         <v>Challenge 58</v>
       </c>
       <c r="B59" t="str">
-        <v>defeatCountRoute: { route: 'Victory Road', count: 300 }</v>
+        <v>Defeat 300 pokemon from Victory Road</v>
       </c>
       <c r="C59" t="str">
         <v>Unlock Kalos Pokemon League</v>
@@ -8886,7 +8886,7 @@
         <v>Challenge 59</v>
       </c>
       <c r="B60" t="str">
-        <v>catchSpeciesAnyOf: { route: 'Kalos Pokemon League', count: 5 }</v>
+        <v>Catch 5 different species from Kalos Pokemon League</v>
       </c>
       <c r="C60" t="str">
         <v>Unlock Mystic Tower Entrance</v>
@@ -8897,7 +8897,7 @@
         <v>Challenge 60</v>
       </c>
       <c r="B61" t="str">
-        <v>defeatCountRoute: { route: 'Mystic Tower Entrance', count: 300 }</v>
+        <v>Defeat 300 pokemon from Mystic Tower Entrance</v>
       </c>
       <c r="C61" t="str">
         <v>Unlock Crystal Cave Tunnels</v>
@@ -8908,7 +8908,7 @@
         <v>Challenge 61</v>
       </c>
       <c r="B62" t="str">
-        <v>catchSpeciesAnyOf: { route: 'Crystal Cave Tunnels', count: 5 }</v>
+        <v>Catch 5 different species from Crystal Cave Tunnels</v>
       </c>
       <c r="C62" t="str">
         <v>Unlock Secret Forest North</v>
@@ -8919,7 +8919,7 @@
         <v>Final Challenge</v>
       </c>
       <c r="B63" t="str">
-        <v>defeatSpecific: { name: 'Diantha', count: 1 }</v>
+        <v>Defeat the Kalos Champion Diantha</v>
       </c>
       <c r="C63" t="str">
         <v>Unlock Path to Sea Spirit Den (first spot for Extra Challenge C), Path to Team Flare Secret HQ (first spot for Extra Challenge E), Path to Secret Ruins (first spot for Extra Challenge D)</v>
@@ -8930,7 +8930,7 @@
         <v>Extra Challenge A 1</v>
       </c>
       <c r="B64" t="str">
-        <v>defeatCountRoute: { route: 'Cyllage City (Fishing)', count: 150 }</v>
+        <v>Defeat 150 pokemon from Cyllage City (Fishing)</v>
       </c>
       <c r="C64" t="str">
         <v>Unlock Reflection Cave</v>
@@ -8941,7 +8941,7 @@
         <v>Extra Challenge A 2</v>
       </c>
       <c r="B65" t="str">
-        <v>defeatCountRoute: { route: 'Reflection Cave', count: 150 }</v>
+        <v>Defeat 150 pokemon from Reflection Cave</v>
       </c>
       <c r="C65" t="str">
         <v>Unlock Tower of Mastery</v>
@@ -8952,7 +8952,7 @@
         <v>Extra Challenge A 3</v>
       </c>
       <c r="B66" t="str">
-        <v>defeatCountRoute: { route: 'Tower of Mastery', count: 150 }</v>
+        <v>Defeat 150 pokemon from Tower of Mastery</v>
       </c>
       <c r="C66" t="str">
         <v>Unlock Coumarine City</v>
@@ -8963,7 +8963,7 @@
         <v>Extra Challenge A 4</v>
       </c>
       <c r="B67" t="str">
-        <v>defeatCountRoute: { route: 'Coumarine City', count: 150 }</v>
+        <v>Defeat 150 pokemon from Coumarine City</v>
       </c>
       <c r="C67" t="str">
         <v>Earn 1 Masterball</v>
@@ -8974,7 +8974,7 @@
         <v>Extra Challenge B 1</v>
       </c>
       <c r="B68" t="str">
-        <v>catchSpecies: { species: ['Rowlet', 'Litten', 'Popplio'], count: 1 }</v>
+        <v>Catch 1 Rowlet, 1 Litten and 1 Popplio</v>
       </c>
       <c r="C68" t="str">
         <v>Unlock Starter Evolved Depot</v>
@@ -8985,7 +8985,7 @@
         <v>Extra Challenge B 2</v>
       </c>
       <c r="B69" t="str">
-        <v>catchSpecies: { species: ['Dartrix', 'Torracat', 'Brionne'], count: 1 }</v>
+        <v>Catch 1 Dartrix, 1 Torracat and 1 Brionne</v>
       </c>
       <c r="C69" t="str">
         <v>Unlock Kiloude City</v>
@@ -8996,7 +8996,7 @@
         <v>Extra Challenge B 3</v>
       </c>
       <c r="B70" t="str">
-        <v>defeatCountRoute: { route: 'Kiloude City', count: 150 }</v>
+        <v>Defeat 150 pokemon from Kiloude City</v>
       </c>
       <c r="C70" t="str">
         <v>Unlock Friend Safari</v>
@@ -9007,7 +9007,7 @@
         <v>Extra Challenge B 4</v>
       </c>
       <c r="B71" t="str">
-        <v>defeatCountRoute: { route: 'Friend Safari', count: 150 }</v>
+        <v>Defeat 150 pokemon from Friend Safari</v>
       </c>
       <c r="C71" t="str">
         <v>Unlock Battle Maison</v>
@@ -9018,7 +9018,7 @@
         <v>Extra Challenge B 5</v>
       </c>
       <c r="B72" t="str">
-        <v>defeatCountRoute: { route: 'Battle Maison', count: 150 }</v>
+        <v>Defeat 150 pokemon from Battle Maison</v>
       </c>
       <c r="C72" t="str">
         <v>Earn 1 Masterball</v>
@@ -9029,7 +9029,7 @@
         <v>Extra Challenge C 1</v>
       </c>
       <c r="B73" t="str">
-        <v>defeatCountRoute: { route: 'Path to Sea Spirit Den', count: 150 }</v>
+        <v>Defeat 150 pokemon from Path to Sea Spirit Den</v>
       </c>
       <c r="C73" t="str">
         <v>Unlock Sea Spirit Den Outer Depths</v>
@@ -9040,7 +9040,7 @@
         <v>Extra Challenge C 2</v>
       </c>
       <c r="B74" t="str">
-        <v>defeatCountRoute: { route: 'Sea Spirit Den Outer Depths', count: 150 }</v>
+        <v>Defeat 150 pokemon from Sea Spirit Den Outer Depths</v>
       </c>
       <c r="C74" t="str">
         <v>Unlock Sea Spirit Den Entrance</v>
@@ -9051,7 +9051,7 @@
         <v>Extra Challenge C 3</v>
       </c>
       <c r="B75" t="str">
-        <v>defeatCountRoute: { route: 'Sea Spirit Den Entrance', count: 150 }</v>
+        <v>Defeat 150 pokemon from Sea Spirit Den Entrance</v>
       </c>
       <c r="C75" t="str">
         <v>Unlock Sea Spirit Den Tunnels</v>
@@ -9062,7 +9062,7 @@
         <v>Extra Challenge C 4</v>
       </c>
       <c r="B76" t="str">
-        <v>defeatCountRoute: { route: 'Sea Spirit Den Tunnels', count: 150 }</v>
+        <v>Defeat 150 pokemon from Sea Spirit Den Tunnels</v>
       </c>
       <c r="C76" t="str">
         <v>Unlock Sea Spirit Den Hall</v>
@@ -9073,7 +9073,7 @@
         <v>Extra Challenge C 5</v>
       </c>
       <c r="B77" t="str">
-        <v>catchSpeciesByQuality: { species: ['Articuno', 'Zapdos', 'Moltres'], quality: 'Legendary', count: 1 }</v>
+        <v>Catch 1 Legendary Articuno, 1 Legendary Zapdos and 1 Legendary Moltres</v>
       </c>
       <c r="C77" t="str">
         <v>Earn 2 Masterball</v>
@@ -9084,7 +9084,7 @@
         <v>Extra Challenge D 1</v>
       </c>
       <c r="B78" t="str">
-        <v>defeatCountRoute: { route: 'Path to Secret Ruins', count: 150 }</v>
+        <v>Defeat 150 pokemon from Path to Secret Ruins</v>
       </c>
       <c r="C78" t="str">
         <v>Unlock Underground Chambers (Crystal Cave Tunnels)</v>
@@ -9095,7 +9095,7 @@
         <v>Extra Challenge D 2</v>
       </c>
       <c r="B79" t="str">
-        <v>defeatCountRoute: { route: 'Underground Chambers', count: 150 }</v>
+        <v>Defeat 150 pokemon from Underground Chambers</v>
       </c>
       <c r="C79" t="str">
         <v>Unlock Garden Chambers (Secret Forest North)</v>
@@ -9106,7 +9106,7 @@
         <v>Extra Challenge D 3</v>
       </c>
       <c r="B80" t="str">
-        <v>defeatCountRoute: { route: 'Garden Chambers', count: 150 }</v>
+        <v>Defeat 150 pokemon from Garden Chambers</v>
       </c>
       <c r="C80" t="str">
         <v>Unlock Chambers of Emptiness</v>
@@ -9117,7 +9117,7 @@
         <v>Extra Challenge D 4</v>
       </c>
       <c r="B81" t="str">
-        <v>defeatCountRoute: { route: 'Chambers of Emptiness', count: 150 }</v>
+        <v>Defeat 150 pokemon from Chambers of Emptiness</v>
       </c>
       <c r="C81" t="str">
         <v>Unlock Ultimate Chamber</v>
@@ -9128,7 +9128,7 @@
         <v>Extra Challenge D 5</v>
       </c>
       <c r="B82" t="str">
-        <v>catchSpeciesByQuality: { species: ['Volcanion', 'Diancie', 'Hoopa', 'Mewtwo'], quality: 'Mythical', count: 1 }</v>
+        <v>Catch 1 Mythical Volcanion, 1 Mythical Diancie, 1 Mythical Hoopa and 1 Mythical Mewtwo</v>
       </c>
       <c r="C82" t="str">
         <v>Earn 2 Masterball</v>
@@ -9139,7 +9139,7 @@
         <v>Extra Challenge E 1</v>
       </c>
       <c r="B83" t="str">
-        <v>defeatCountRoute: { route: 'Path to Team Flare Secret HQ', count: 150 }</v>
+        <v>Defeat 150 pokemon from Path to Team Flare Secret HQ</v>
       </c>
       <c r="C83" t="str">
         <v>Unlock 2nd spot for Extra Challenge E</v>
@@ -9150,7 +9150,7 @@
         <v>Extra Challenge E 2</v>
       </c>
       <c r="B84" t="str">
-        <v>defeatCountRoute: { route: '2nd spot for Extra Challenge E', count: 150 }</v>
+        <v>Defeat 150 pokemon from 2nd spot for Extra Challenge E</v>
       </c>
       <c r="C84" t="str">
         <v>Unlock Team Flare Secret HQ Gate</v>
@@ -9161,7 +9161,7 @@
         <v>Extra Challenge E 3</v>
       </c>
       <c r="B85" t="str">
-        <v>defeatCountRoute: { route: 'Team Flare Secret HQ Gate', count: 150 }</v>
+        <v>Defeat 150 pokemon from Team Flare Secret HQ Gate</v>
       </c>
       <c r="C85" t="str">
         <v>Unlock Team Flare Secret HQ Entrance</v>
@@ -9172,7 +9172,7 @@
         <v>Extra Challenge E 4</v>
       </c>
       <c r="B86" t="str">
-        <v>defeatCountRoute: { route: 'Team Flare Secret HQ Entrance', count: 150 }</v>
+        <v>Defeat 150 pokemon from Team Flare Secret HQ Entrance</v>
       </c>
       <c r="C86" t="str">
         <v>Unlock Team Flare Secret HQ Hall</v>
@@ -9183,7 +9183,7 @@
         <v>Extra Challenge E 5</v>
       </c>
       <c r="B87" t="str">
-        <v>catchSpeciesByQuality: { species: ['Yveltal', 'Zygarde', 'Xerneas'], quality: 'Legendary', count: 1 }</v>
+        <v>Catch 1 Legendary Yveltal, 1 Legendary Zygarde and 1 Legendary Xerneas</v>
       </c>
       <c r="C87" t="str">
         <v>Earn 2 Masterball</v>

</xml_diff>